<commit_message>
UPDATE : detecter les fins de courses, et bloquer le mouvement des moteurs + recul 5 pas
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="364">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -129,9 +129,9 @@
     <t xml:space="preserve">Placements : </t>
   </si>
   <si>
-    <t xml:space="preserve">- En bas, s'aider de la plaque pour bloquer la descente, sur la droite. Limite au niveau des CDs du bas, pour être sur de la hauteur
-- En haut, coller le capteur plus bas, sur le raill. Faire coïencider l'elecaimant et le cd, comme ça on sait qu'on est à la bonne hauteur
--A droite, OK
+    <t xml:space="preserve">- En bas, s'aider de la plaque pour bloquer la descente, sur la droite
+- En haut, coller le capteur plus bas, sur le raill. 
+- A droite, OK
 -A gauche, fixer comme droite</t>
   </si>
   <si>
@@ -153,11 +153,11 @@
     <t xml:space="preserve">0,57cm pour une largeur de 0,6cm</t>
   </si>
   <si>
-    <t xml:space="preserve">Les capteurs haut/bas sont au niveau des CDs, donc pas de calcul à faire
-Les droites gauches ne sont pas aux limites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Utiliser de la colle ? </t>
+    <t xml:space="preserve">On mets au max, la positon des cds se fera via config manuelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utiliser de la colle ? 
+FAIRE des rallonges</t>
   </si>
   <si>
     <t xml:space="preserve">Tester déplacement X et Y</t>
@@ -200,7 +200,10 @@
     <t xml:space="preserve">Plaque avec support Cds et lecteur, prévoir place lecteur !</t>
   </si>
   <si>
-    <t xml:space="preserve">Vérifier le code pour pour tester manuellement</t>
+    <t xml:space="preserve">Vérifier le code pour pour tester manuellement
+- Fonction moveX/Y, ajouter le recul si capteur detecté
+- MAX STEP
+Ajouter retour de pas au compteur, </t>
   </si>
   <si>
     <t xml:space="preserve">Ralonge câbles</t>
@@ -230,6 +233,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Dev menu parametrage des positions manuellement !</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voir dessin</t>
   </si>
   <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
@@ -1706,13 +1715,14 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="15" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1724,11 +1734,10 @@
       <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
@@ -2704,8 +2713,8 @@
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="14">
-        <f>SUM(D14:D20)/7</f>
-        <v>0.14285714285714285</v>
+        <f>SUM(D14:D22)/9</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>22</v>
@@ -2795,7 +2804,7 @@
         <v>36</v>
       </c>
       <c r="D15" s="28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>37</v>
@@ -2834,14 +2843,14 @@
     </row>
     <row r="16" ht="28.5">
       <c r="A16" s="1"/>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="30" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="s">
         <v>45</v>
@@ -2878,7 +2887,7 @@
       <c r="B17" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="31">
+      <c r="D17" s="32">
         <v>0</v>
       </c>
       <c r="F17" s="4"/>
@@ -2904,15 +2913,15 @@
       <c r="B18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="31">
+      <c r="D18" s="32">
         <v>0</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F18" s="33" t="s">
         <v>52</v>
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="33" t="s">
+      <c r="I18" s="34" t="s">
         <v>53</v>
       </c>
       <c r="J18" s="16" t="s">
@@ -2940,10 +2949,10 @@
     </row>
     <row r="19" ht="42.75">
       <c r="A19" s="1"/>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="31">
+      <c r="D19" s="32">
         <v>0</v>
       </c>
       <c r="F19" t="s">
@@ -2965,12 +2974,12 @@
       <c r="Z19" s="1"/>
       <c r="AA19" s="1"/>
     </row>
-    <row r="20" ht="16.5">
+    <row r="20" ht="57">
       <c r="A20" s="1"/>
-      <c r="B20" s="35" t="s">
+      <c r="B20" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="31">
+      <c r="D20" s="32">
         <v>0</v>
       </c>
       <c r="F20" s="15" t="s">
@@ -2990,7 +2999,7 @@
       <c r="L20" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="M20" s="36" t="s">
+      <c r="M20" s="37" t="s">
         <v>62</v>
       </c>
       <c r="N20" s="1"/>
@@ -3006,10 +3015,12 @@
     </row>
     <row r="21" ht="128.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="38"/>
+      <c r="D21" s="32">
+        <v>0</v>
+      </c>
       <c r="F21" t="s">
         <v>64</v>
       </c>
@@ -3021,7 +3032,7 @@
       <c r="L21" t="s">
         <v>65</v>
       </c>
-      <c r="M21" s="36" t="s">
+      <c r="M21" s="37" t="s">
         <v>62</v>
       </c>
       <c r="N21" s="1"/>
@@ -3040,29 +3051,37 @@
     </row>
     <row r="22" ht="16.5">
       <c r="A22" s="1"/>
-      <c r="D22" s="38"/>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="32">
+        <v>0</v>
+      </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="M22" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="M22" s="37" t="s">
         <v>62</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3070,7 +3089,7 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
@@ -3083,23 +3102,23 @@
       <c r="J23" s="39"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>72</v>
-      </c>
-      <c r="M23" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="37" t="s">
         <v>62</v>
       </c>
       <c r="N23" s="1"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
@@ -3107,7 +3126,7 @@
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
       <c r="F24" s="40" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
@@ -3117,10 +3136,10 @@
       <c r="J24" s="43"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3136,7 +3155,7 @@
     <row r="25" ht="16.5">
       <c r="A25" s="1"/>
       <c r="B25" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="14">
@@ -3163,12 +3182,12 @@
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="31">
+        <v>82</v>
+      </c>
+      <c r="D26" s="32">
         <v>0</v>
       </c>
       <c r="F26" s="1"/>
@@ -3181,10 +3200,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3197,9 +3216,9 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="C27" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" s="31">
+        <v>85</v>
+      </c>
+      <c r="D27" s="32">
         <v>0</v>
       </c>
       <c r="N27" s="1"/>
@@ -3211,7 +3230,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3219,9 +3238,9 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="B28" t="s">
-        <v>85</v>
-      </c>
-      <c r="D28" s="31">
+        <v>87</v>
+      </c>
+      <c r="D28" s="32">
         <v>0</v>
       </c>
       <c r="L28" s="19"/>
@@ -3235,7 +3254,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3243,12 +3262,12 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C29" t="s">
-        <v>88</v>
-      </c>
-      <c r="D29" s="31">
+        <v>90</v>
+      </c>
+      <c r="D29" s="32">
         <v>0</v>
       </c>
       <c r="M29" s="1"/>
@@ -3266,12 +3285,12 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="31">
+        <v>92</v>
+      </c>
+      <c r="D30" s="32">
         <v>0</v>
       </c>
       <c r="L30" s="19"/>
@@ -3290,9 +3309,9 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D31" s="31">
+        <v>93</v>
+      </c>
+      <c r="D31" s="32">
         <v>0</v>
       </c>
       <c r="N31" s="1"/>
@@ -3311,7 +3330,7 @@
       <c r="B32" s="44"/>
       <c r="D32" s="38"/>
       <c r="L32" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3321,7 +3340,7 @@
       <c r="B33" s="44"/>
       <c r="D33" s="38"/>
       <c r="L33" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3348,7 +3367,7 @@
     <row r="35" ht="16.5">
       <c r="A35" s="1"/>
       <c r="B35" s="45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="14">
@@ -3369,12 +3388,12 @@
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
       <c r="B36" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D36" s="31">
+        <v>98</v>
+      </c>
+      <c r="D36" s="32">
         <v>0</v>
       </c>
       <c r="L36" s="1"/>
@@ -3391,12 +3410,12 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D37" s="31">
+        <v>100</v>
+      </c>
+      <c r="D37" s="32">
         <v>0</v>
       </c>
       <c r="L37" s="2"/>
@@ -3413,12 +3432,12 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D38" s="31">
+        <v>102</v>
+      </c>
+      <c r="D38" s="32">
         <v>0</v>
       </c>
       <c r="L38" s="2"/>
@@ -3435,12 +3454,12 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C39" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="D39" s="31">
+        <v>104</v>
+      </c>
+      <c r="D39" s="32">
         <v>0</v>
       </c>
     </row>
@@ -3450,7 +3469,7 @@
     <row r="41" ht="16.5">
       <c r="A41" s="1"/>
       <c r="B41" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -3458,7 +3477,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3478,7 +3497,7 @@
     <row r="47" ht="14.25">
       <c r="A47" s="1"/>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" ht="14.25">
@@ -3487,13 +3506,13 @@
     <row r="49" ht="14.25">
       <c r="A49" s="1"/>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" ht="14.25">
@@ -3505,13 +3524,13 @@
     <row r="53" ht="16.5">
       <c r="A53" s="1"/>
       <c r="B53" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3578,52 +3597,52 @@
     </row>
     <row r="68" ht="14.25">
       <c r="B68" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" ht="14.25">
       <c r="B69" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C77" t="s">
         <v>66</v>
@@ -3657,222 +3676,222 @@
     <row r="1" ht="15"/>
     <row r="2" ht="15">
       <c r="F2" s="46" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G2" s="47" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
       <c r="F3" s="48" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
       <c r="F4" s="50" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G4" s="51" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" ht="15">
       <c r="F5" s="52" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G5" s="53" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="F6" s="54"/>
       <c r="G6" s="55" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" ht="15">
       <c r="F7" s="54"/>
       <c r="G7" s="55" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" ht="15">
       <c r="F8" s="54"/>
       <c r="G8" s="55" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F9" s="54"/>
       <c r="G9" s="55" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="55" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" ht="15">
       <c r="C11" s="57" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F11" s="54"/>
       <c r="G11" s="55" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" ht="15">
       <c r="C12" s="56" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F12" s="48"/>
       <c r="G12" s="58" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" ht="15">
       <c r="C13" s="57" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F13" s="50" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G13" s="59" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" ht="15">
       <c r="C14" s="56" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F14" s="60" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G14" s="61" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15">
       <c r="C15" s="57" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F15" s="62" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G15" s="63" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16">
       <c r="C16" s="57" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F16" s="64" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G16" s="65" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17">
       <c r="C17" s="56" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F17" s="64"/>
       <c r="G17" s="65" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18">
       <c r="C18" s="57" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F18" s="64"/>
       <c r="G18" s="65" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19">
       <c r="C19" s="57" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F19" s="64"/>
       <c r="G19" s="65" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20">
       <c r="C20" s="57" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F20" s="64"/>
       <c r="G20" s="65" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21">
       <c r="C21" s="57" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F21" s="64"/>
       <c r="G21" s="65" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22">
       <c r="C22" s="56" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F22" s="64"/>
       <c r="G22" s="65" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="57" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F23" s="64"/>
       <c r="G23" s="65" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24">
       <c r="C24" s="56" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F24" s="64"/>
       <c r="G24" s="65" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="57" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F25" s="64"/>
       <c r="G25" s="65" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26">
       <c r="F26" s="64"/>
       <c r="G26" s="65" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27">
@@ -3882,35 +3901,35 @@
     <row r="28">
       <c r="F28" s="64"/>
       <c r="G28" s="65" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29">
       <c r="F29" s="64"/>
       <c r="G29" s="65" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="66"/>
       <c r="F30" s="64"/>
       <c r="G30" s="65" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31">
       <c r="F31" s="64"/>
       <c r="G31" s="67" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="26"/>
       <c r="F32" s="60" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G32" s="68" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33">
@@ -3957,250 +3976,250 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="K5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H6" s="71" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="K6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B7" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D7" s="72" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H7" s="71" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K7" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8">
       <c r="D8" s="70" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G8" s="73" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H8" s="71" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D9" s="72" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H9" s="71" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D10" s="70"/>
       <c r="G10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H10" s="71" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D11" s="72" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G11" s="73" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H11" s="71" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G12" s="73" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H12" s="71" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D13" s="72" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G13" s="73" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14">
       <c r="D14" s="70" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B15" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D15" s="72"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D16" s="70"/>
       <c r="G16" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="72"/>
       <c r="G17" s="73" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D18" s="70"/>
       <c r="G18" s="74" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="72" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E19" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="G19" s="74" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H19" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="J19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="70"/>
       <c r="G20" s="74" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="70"/>
       <c r="G22" s="74" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23">
@@ -4209,115 +4228,115 @@
     <row r="24">
       <c r="D24" s="70"/>
       <c r="G24" s="73" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="25">
       <c r="G25" s="74" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="70"/>
       <c r="G26" s="74" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27">
       <c r="G27" s="74" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="70"/>
       <c r="G28" s="74" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="75" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E35" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F35" s="76" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="77" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E36" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F36" s="77" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="76" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E37" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F37" s="76" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="77" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E38" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F38" s="77" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="76" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E39" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F39" s="76" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F40" s="77" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F41" s="76" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -4349,15 +4368,15 @@
   <sheetData>
     <row r="4">
       <c r="D4" s="78" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E5" s="78">
         <v>1</v>
@@ -4365,7 +4384,7 @@
     </row>
     <row r="6">
       <c r="D6" s="74" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E6" s="78">
         <v>1</v>
@@ -4373,7 +4392,7 @@
     </row>
     <row r="7">
       <c r="D7" s="79" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E7" s="78">
         <v>1</v>
@@ -4381,7 +4400,7 @@
     </row>
     <row r="8">
       <c r="D8" s="74" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E8" s="78">
         <v>1</v>
@@ -4393,7 +4412,7 @@
     </row>
     <row r="10">
       <c r="D10" s="71" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E10" s="78">
         <v>1</v>
@@ -4401,7 +4420,7 @@
     </row>
     <row r="11">
       <c r="D11" s="74" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E11" s="78">
         <v>1</v>
@@ -4409,7 +4428,7 @@
     </row>
     <row r="12">
       <c r="D12" s="74" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E12" s="78">
         <v>1</v>
@@ -4417,7 +4436,7 @@
     </row>
     <row r="13">
       <c r="D13" s="74" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E13" s="78">
         <v>1</v>
@@ -4429,7 +4448,7 @@
     </row>
     <row r="15">
       <c r="D15" s="71" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E15" s="78">
         <v>2</v>
@@ -4437,7 +4456,7 @@
     </row>
     <row r="16">
       <c r="D16" s="80" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E16" s="78">
         <v>2</v>
@@ -4445,7 +4464,7 @@
     </row>
     <row r="17">
       <c r="D17" s="81" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E17" s="78">
         <v>2</v>
@@ -4453,7 +4472,7 @@
     </row>
     <row r="18">
       <c r="D18" s="81" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E18" s="78">
         <v>2</v>
@@ -4465,7 +4484,7 @@
     </row>
     <row r="20">
       <c r="D20" s="71" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E20" s="78">
         <v>2</v>
@@ -4473,7 +4492,7 @@
     </row>
     <row r="21">
       <c r="D21" s="71" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E21" s="78">
         <v>2</v>
@@ -4518,13 +4537,13 @@
     <row r="39">
       <c r="B39" s="83"/>
       <c r="C39" s="84" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D39" s="84" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E39" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
@@ -4535,60 +4554,60 @@
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E40" s="78"/>
     </row>
     <row r="41">
       <c r="C41" s="78" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D41" s="74" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E41" s="78"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="C42" s="78" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D42" s="74" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43">
       <c r="C43" s="78" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D43" s="74" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="44">
       <c r="C44" s="86" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D44" s="79" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E44" s="87"/>
       <c r="F44" s="87"/>
     </row>
     <row r="45">
       <c r="C45" s="84" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D45" s="74" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E45" s="78"/>
     </row>
     <row r="46">
       <c r="C46" s="84" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D46" s="74" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E46" s="78"/>
     </row>
@@ -4597,16 +4616,16 @@
         <v>2</v>
       </c>
       <c r="D47" s="89" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E47" s="78"/>
     </row>
     <row r="48">
       <c r="C48" s="86" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D48" s="79" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E48" s="78"/>
     </row>
@@ -4615,51 +4634,51 @@
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E49" s="78"/>
     </row>
     <row r="50">
       <c r="C50" s="86" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D50" s="79" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F50" s="90" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="51">
       <c r="C51" s="86" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D51" s="91" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="52">
       <c r="C52" s="86" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D52" s="91" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="53">
       <c r="C53" s="86" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D53" s="91" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="54">
       <c r="C54" s="86" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D54" s="91" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="55">
@@ -4667,39 +4686,39 @@
         <v>4</v>
       </c>
       <c r="D55" s="92" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="56">
       <c r="C56" s="84" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D56" s="74" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="57">
       <c r="C57" s="84" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D57" s="91" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="58">
       <c r="C58" s="84" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D58" s="91" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="59">
       <c r="C59" s="84" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D59" s="91" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
@@ -4709,42 +4728,42 @@
         <v>5</v>
       </c>
       <c r="D60" s="92" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="61">
       <c r="C61" s="84" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D61" s="74" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="62">
       <c r="C62" s="84" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D62" s="91" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F62" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63">
       <c r="C63" s="84" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D63" s="91" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="64">
       <c r="C64" s="84" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D64" s="91" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="65">
@@ -4752,47 +4771,47 @@
         <v>6</v>
       </c>
       <c r="D65" s="92" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="66">
       <c r="C66" s="84" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D66" s="74" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="93" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D67" s="94" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="68">
       <c r="C68" s="84" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D68" s="91" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="69">
       <c r="C69" s="93" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D69" s="91" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="70">
       <c r="C70" s="84" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D70" s="91" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="71">
@@ -4800,15 +4819,15 @@
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="72">
       <c r="C72" s="84" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D72" s="74" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="73">
@@ -4816,15 +4835,15 @@
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="74">
       <c r="C74" s="84" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D74" s="74" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="75">
@@ -4832,31 +4851,31 @@
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="76">
       <c r="C76" s="84" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D76" s="74" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="77">
       <c r="C77" s="84" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D77" s="91" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="78">
       <c r="C78" s="84" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D78" s="91" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="79">
@@ -4864,24 +4883,24 @@
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="80">
       <c r="C80" s="84" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D80" s="74" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E80" s="78"/>
     </row>
     <row r="81">
       <c r="C81" s="84" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D81" s="91" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="82">
@@ -4889,23 +4908,23 @@
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="83">
       <c r="C83" s="84" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D83" s="74" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="84">
       <c r="C84" s="84" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D84" s="74" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE : menu calibrage manuel : affichage coordonnées save + btn save quand chariot bon emplacement
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="363">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -201,9 +201,7 @@
   </si>
   <si>
     <t xml:space="preserve">Vérifier le code pour pour tester manuellement
-- Fonction moveX/Y, ajouter le recul si capteur detecté
-- MAX STEP
-Ajouter retour de pas au compteur, </t>
+- Fonction moveX/Y, ajouter le recul si capteur detecté</t>
   </si>
   <si>
     <t xml:space="preserve">Ralonge câbles</t>
@@ -219,10 +217,15 @@
   </si>
   <si>
     <t xml:space="preserve">Teste manuel déplacement : 
-- Bloquer les fonctions move quand detecté + recule 5 pas par ex
-- Calcul distance max : bas/gauche-haut/droite
-- Calcul positions (prendre en compte limite haute/bassent = position X des cds/lecteur. Trouver donc les positions Y (normalemen ils sont alignés donc 1 meusure suffit ? )
+# Bloquer les fonctions move quand detecté + recule 20 pas par ex
+- Machine a état : simple et efficace (repars à 0 ? + ajouter compteur )
+    # Retourner le nb de pas effectuer dans les move()
+    # Calcul distance max : bas/gauche-haut/droite
+    # Menu parametrage positions manuel
+        # Voir dessin
 -Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
+- Calcul pas de déplacement pour aller àla pos voulu
+- Appeler GoToPos 2 fois : aller de a à b avec action sur CD, PUIS aller de b à c avec action CD
 </t>
   </si>
   <si>
@@ -235,12 +238,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">-Dev menu parametrage des positions manuellement !</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voir dessin</t>
-  </si>
-  <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
   </si>
   <si>
@@ -353,6 +350,9 @@
   </si>
   <si>
     <t xml:space="preserve">1 alim pour moteurs, raspberry, lecteur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fichier update_jukebox : faire tous les scritp en 1 ?</t>
   </si>
   <si>
     <t xml:space="preserve">Dernière vérif avec multimetre pour valider les moteurs PàP</t>
@@ -1268,7 +1268,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -1317,12 +1317,18 @@
     </font>
     <font>
       <b/>
-      <sz val="11.000000"/>
+      <sz val="48.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1672,7 +1678,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="91">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1705,7 +1711,6 @@
     <xf fontId="1" fillId="12" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="1" fillId="13" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="0" fillId="14" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="0" fillId="14" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1715,15 +1720,8 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="15" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1734,11 +1732,11 @@
       <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1748,8 +1746,10 @@
     </xf>
     <xf fontId="8" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="8" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="9" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="9" fillId="7" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="10" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="0" fillId="17" borderId="7" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="17" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -1757,27 +1757,27 @@
     <xf fontId="0" fillId="17" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="13" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="10" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="15" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="10" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
-    <xf fontId="11" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="10" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
-    <xf fontId="10" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="10" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="17" borderId="13" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1789,7 +1789,7 @@
     </xf>
     <xf fontId="0" fillId="17" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="17" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="12" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="13" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="10" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1801,7 +1801,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf fontId="12" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="13" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="10" borderId="3" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
@@ -1810,16 +1810,16 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2" wrapText="1"/>
     </xf>
-    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
@@ -1831,7 +1831,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="16" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2475,7 +2475,7 @@
     <col customWidth="1" min="1" max="1" width="9.140625"/>
     <col customWidth="1" min="2" max="2" width="63.7109375"/>
     <col customWidth="1" min="3" max="3" width="63.421875"/>
-    <col bestFit="1" customWidth="1" min="4" max="4" width="39.11328125"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="42.09375"/>
     <col customWidth="1" min="5" max="5" width="60.00390625"/>
     <col bestFit="1" customWidth="1" min="6" max="6" width="40.171875"/>
     <col customWidth="1" min="7" max="7" width="26.421875"/>
@@ -2706,15 +2706,15 @@
       <c r="Z12" s="1"/>
       <c r="AA12" s="1"/>
     </row>
-    <row r="13" ht="16.5">
+    <row r="13" ht="60">
       <c r="A13" s="1"/>
       <c r="B13" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="14">
-        <f>SUM(D14:D22)/9</f>
-        <v>0.33333333333333331</v>
+        <f>SUM(D14:D21)/8</f>
+        <v>0.80625000000000002</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>22</v>
@@ -2756,8 +2756,8 @@
       <c r="B14" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="25">
+      <c r="C14" s="23"/>
+      <c r="D14" s="24">
         <v>1</v>
       </c>
       <c r="F14" t="s">
@@ -2795,15 +2795,15 @@
       <c r="Z14" s="1"/>
       <c r="AA14" s="1"/>
     </row>
-    <row r="15" ht="85.5">
+    <row r="15" ht="57">
       <c r="A15" s="1"/>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="24">
         <v>1</v>
       </c>
       <c r="F15" s="15" t="s">
@@ -2816,7 +2816,7 @@
       <c r="I15" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="J15" s="29" t="s">
+      <c r="J15" s="27" t="s">
         <v>39</v>
       </c>
       <c r="K15" s="1"/>
@@ -2843,13 +2843,13 @@
     </row>
     <row r="16" ht="28.5">
       <c r="A16" s="1"/>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="31">
+      <c r="D16" s="28">
         <v>1</v>
       </c>
       <c r="F16" t="s">
@@ -2887,8 +2887,8 @@
       <c r="B17" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="32">
-        <v>0</v>
+      <c r="D17" s="28">
+        <v>1</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="16"/>
@@ -2913,15 +2913,15 @@
       <c r="B18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="32">
-        <v>0</v>
-      </c>
-      <c r="F18" s="33" t="s">
+      <c r="D18" s="28">
+        <v>1</v>
+      </c>
+      <c r="F18" s="29" t="s">
         <v>52</v>
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="34" t="s">
+      <c r="I18" s="30" t="s">
         <v>53</v>
       </c>
       <c r="J18" s="16" t="s">
@@ -2949,7 +2949,7 @@
     </row>
     <row r="19" ht="42.75">
       <c r="A19" s="1"/>
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="31" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="32">
@@ -2974,13 +2974,13 @@
       <c r="Z19" s="1"/>
       <c r="AA19" s="1"/>
     </row>
-    <row r="20" ht="57">
+    <row r="20" ht="28.5">
       <c r="A20" s="1"/>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="32">
-        <v>0</v>
+      <c r="D20" s="28">
+        <v>1</v>
       </c>
       <c r="F20" s="15" t="s">
         <v>59</v>
@@ -2999,7 +2999,7 @@
       <c r="L20" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="M20" s="37" t="s">
+      <c r="M20" s="33" t="s">
         <v>62</v>
       </c>
       <c r="N20" s="1"/>
@@ -3013,13 +3013,13 @@
       <c r="Z20" s="1"/>
       <c r="AA20" s="1"/>
     </row>
-    <row r="21" ht="128.25">
+    <row r="21" ht="185.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="34" t="s">
         <v>63</v>
       </c>
       <c r="D21" s="32">
-        <v>0</v>
+        <v>0.45000000000000001</v>
       </c>
       <c r="F21" t="s">
         <v>64</v>
@@ -3032,7 +3032,7 @@
       <c r="L21" t="s">
         <v>65</v>
       </c>
-      <c r="M21" s="37" t="s">
+      <c r="M21" s="33" t="s">
         <v>62</v>
       </c>
       <c r="N21" s="1"/>
@@ -3051,37 +3051,29 @@
     </row>
     <row r="22" ht="16.5">
       <c r="A22" s="1"/>
-      <c r="B22" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="32">
-        <v>0</v>
-      </c>
+      <c r="D22" s="32"/>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="M22" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="M22" s="33" t="s">
         <v>62</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3089,57 +3081,57 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
     </row>
     <row r="23" ht="16.5">
       <c r="A23" s="1"/>
-      <c r="D23" s="38"/>
+      <c r="D23" s="32"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="35"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>74</v>
-      </c>
-      <c r="M23" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="M23" s="33" t="s">
         <v>62</v>
       </c>
       <c r="N23" s="1"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
-      <c r="F24" s="40" t="s">
-        <v>77</v>
+      <c r="F24" s="36" t="s">
+        <v>75</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="41"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="43"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="38"/>
+      <c r="J24" s="39"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3155,10 +3147,10 @@
     <row r="25" ht="16.5">
       <c r="A25" s="1"/>
       <c r="B25" s="12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C25" s="13"/>
-      <c r="D25" s="14">
+      <c r="D25" s="40">
         <f>SUM(D26:D31)/5</f>
         <v>0</v>
       </c>
@@ -3182,10 +3174,10 @@
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D26" s="32">
         <v>0</v>
@@ -3200,10 +3192,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3216,7 +3208,7 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D27" s="32">
         <v>0</v>
@@ -3230,7 +3222,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3238,7 +3230,7 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D28" s="32">
         <v>0</v>
@@ -3254,7 +3246,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3262,10 +3254,10 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C29" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D29" s="32">
         <v>0</v>
@@ -3285,10 +3277,10 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D30" s="32">
         <v>0</v>
@@ -3309,7 +3301,7 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D31" s="32">
         <v>0</v>
@@ -3327,20 +3319,20 @@
     </row>
     <row r="32" ht="28.5">
       <c r="A32" s="1"/>
-      <c r="B32" s="44"/>
-      <c r="D32" s="38"/>
+      <c r="B32" s="4"/>
+      <c r="D32" s="32"/>
       <c r="L32" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
     </row>
     <row r="33" ht="16.5">
       <c r="A33" s="1"/>
-      <c r="B33" s="44"/>
-      <c r="D33" s="38"/>
+      <c r="B33" s="4"/>
+      <c r="D33" s="32"/>
       <c r="L33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3366,11 +3358,11 @@
     </row>
     <row r="35" ht="16.5">
       <c r="A35" s="1"/>
-      <c r="B35" s="45" t="s">
-        <v>96</v>
+      <c r="B35" s="41" t="s">
+        <v>94</v>
       </c>
       <c r="C35" s="13"/>
-      <c r="D35" s="14">
+      <c r="D35" s="40">
         <f>SUM(D36:D39)/4</f>
         <v>0</v>
       </c>
@@ -3388,10 +3380,10 @@
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
       <c r="B36" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D36" s="32">
         <v>0</v>
@@ -3410,10 +3402,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D37" s="32">
         <v>0</v>
@@ -3432,10 +3424,10 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D38" s="32">
         <v>0</v>
@@ -3454,10 +3446,10 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C39" s="30" t="s">
-        <v>104</v>
+        <v>101</v>
+      </c>
+      <c r="C39" s="26" t="s">
+        <v>102</v>
       </c>
       <c r="D39" s="32">
         <v>0</v>
@@ -3469,7 +3461,7 @@
     <row r="41" ht="16.5">
       <c r="A41" s="1"/>
       <c r="B41" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -3477,7 +3469,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3487,6 +3479,9 @@
     </row>
     <row r="44" ht="16.5">
       <c r="A44" s="1"/>
+      <c r="B44" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="45" ht="16.5">
       <c r="A45" s="1"/>
@@ -3497,7 +3492,7 @@
     <row r="47" ht="14.25">
       <c r="A47" s="1"/>
       <c r="B47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" ht="14.25">
@@ -3506,13 +3501,13 @@
     <row r="49" ht="14.25">
       <c r="A49" s="1"/>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="51" ht="14.25">
@@ -3524,13 +3519,13 @@
     <row r="53" ht="16.5">
       <c r="A53" s="1"/>
       <c r="B53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3597,52 +3592,52 @@
     </row>
     <row r="68" ht="14.25">
       <c r="B68" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="69" ht="14.25">
       <c r="B69" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C77" t="s">
         <v>66</v>
@@ -3675,280 +3670,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="46" t="s">
+      <c r="F2" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="47" t="s">
+    </row>
+    <row r="3">
+      <c r="F3" s="44" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="F3" s="48" t="s">
+      <c r="G3" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="G3" s="49" t="s">
+    </row>
+    <row r="4">
+      <c r="F4" s="46" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="F4" s="50" t="s">
+      <c r="G4" s="47" t="s">
         <v>126</v>
       </c>
-      <c r="G4" s="51" t="s">
+    </row>
+    <row r="5" ht="15">
+      <c r="F5" s="48" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="5" ht="15">
-      <c r="F5" s="52" t="s">
+      <c r="G5" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="G5" s="53" t="s">
+    </row>
+    <row r="6" ht="15">
+      <c r="F6" s="50"/>
+      <c r="G6" s="51" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="6" ht="15">
-      <c r="F6" s="54"/>
-      <c r="G6" s="55" t="s">
+    <row r="7" ht="15">
+      <c r="F7" s="50"/>
+      <c r="G7" s="51" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="7" ht="15">
-      <c r="F7" s="54"/>
-      <c r="G7" s="55" t="s">
+    <row r="8" ht="15">
+      <c r="F8" s="50"/>
+      <c r="G8" s="51" t="s">
         <v>131</v>
-      </c>
-    </row>
-    <row r="8" ht="15">
-      <c r="F8" s="54"/>
-      <c r="G8" s="55" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="50"/>
+      <c r="G9" s="51" t="s">
         <v>133</v>
-      </c>
-      <c r="F9" s="54"/>
-      <c r="G9" s="55" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="56" t="s">
+      <c r="F10" s="50"/>
+      <c r="G10" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="F10" s="54"/>
-      <c r="G10" s="55" t="s">
+    </row>
+    <row r="11" ht="15">
+      <c r="C11" s="53" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="11" ht="15">
-      <c r="C11" s="57" t="s">
+      <c r="F11" s="50"/>
+      <c r="G11" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="55" t="s">
+    </row>
+    <row r="12" ht="15">
+      <c r="C12" s="52" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="12" ht="15">
-      <c r="C12" s="56" t="s">
+      <c r="F12" s="44"/>
+      <c r="G12" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="F12" s="48"/>
-      <c r="G12" s="58" t="s">
+    </row>
+    <row r="13" ht="15">
+      <c r="C13" s="53" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="13" ht="15">
-      <c r="C13" s="57" t="s">
+      <c r="F13" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="F13" s="50" t="s">
+      <c r="G13" s="55" t="s">
         <v>143</v>
       </c>
-      <c r="G13" s="59" t="s">
+    </row>
+    <row r="14" ht="15">
+      <c r="C14" s="52" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="14" ht="15">
-      <c r="C14" s="56" t="s">
+      <c r="F14" s="56" t="s">
         <v>145</v>
       </c>
-      <c r="F14" s="60" t="s">
+      <c r="G14" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="G14" s="61" t="s">
+    </row>
+    <row r="15">
+      <c r="C15" s="53" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="C15" s="57" t="s">
+      <c r="F15" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="F15" s="62" t="s">
+      <c r="G15" s="59" t="s">
         <v>149</v>
       </c>
-      <c r="G15" s="63" t="s">
+    </row>
+    <row r="16">
+      <c r="C16" s="53" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="57" t="s">
+      <c r="F16" s="60" t="s">
         <v>151</v>
       </c>
-      <c r="F16" s="64" t="s">
+      <c r="G16" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="G16" s="65" t="s">
+    </row>
+    <row r="17">
+      <c r="C17" s="52" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="C17" s="56" t="s">
+      <c r="F17" s="60"/>
+      <c r="G17" s="61" t="s">
         <v>154</v>
       </c>
-      <c r="F17" s="64"/>
-      <c r="G17" s="65" t="s">
+    </row>
+    <row r="18">
+      <c r="C18" s="53" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="C18" s="57" t="s">
+      <c r="F18" s="60"/>
+      <c r="G18" s="61" t="s">
         <v>156</v>
       </c>
-      <c r="F18" s="64"/>
-      <c r="G18" s="65" t="s">
+    </row>
+    <row r="19">
+      <c r="C19" s="53" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="C19" s="57" t="s">
+      <c r="F19" s="60"/>
+      <c r="G19" s="61" t="s">
         <v>158</v>
       </c>
-      <c r="F19" s="64"/>
-      <c r="G19" s="65" t="s">
+    </row>
+    <row r="20">
+      <c r="C20" s="53" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="57" t="s">
+      <c r="F20" s="60"/>
+      <c r="G20" s="61" t="s">
         <v>160</v>
       </c>
-      <c r="F20" s="64"/>
-      <c r="G20" s="65" t="s">
+    </row>
+    <row r="21">
+      <c r="C21" s="53" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="57" t="s">
+      <c r="F21" s="60"/>
+      <c r="G21" s="61" t="s">
         <v>162</v>
       </c>
-      <c r="F21" s="64"/>
-      <c r="G21" s="65" t="s">
+    </row>
+    <row r="22">
+      <c r="C22" s="52" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="56" t="s">
+      <c r="F22" s="60"/>
+      <c r="G22" s="61" t="s">
         <v>164</v>
       </c>
-      <c r="F22" s="64"/>
-      <c r="G22" s="65" t="s">
+    </row>
+    <row r="23">
+      <c r="C23" s="53" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="C23" s="57" t="s">
+      <c r="F23" s="60"/>
+      <c r="G23" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="F23" s="64"/>
-      <c r="G23" s="65" t="s">
+    </row>
+    <row r="24">
+      <c r="C24" s="52" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="56" t="s">
+      <c r="F24" s="60"/>
+      <c r="G24" s="61" t="s">
         <v>168</v>
       </c>
-      <c r="F24" s="64"/>
-      <c r="G24" s="65" t="s">
+    </row>
+    <row r="25">
+      <c r="C25" s="53" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="57" t="s">
+      <c r="F25" s="60"/>
+      <c r="G25" s="61" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="64"/>
-      <c r="G25" s="65" t="s">
+    </row>
+    <row r="26">
+      <c r="F26" s="60"/>
+      <c r="G26" s="61" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="26">
-      <c r="F26" s="64"/>
-      <c r="G26" s="65" t="s">
+    <row r="27">
+      <c r="F27" s="60"/>
+      <c r="G27" s="61"/>
+    </row>
+    <row r="28">
+      <c r="F28" s="60"/>
+      <c r="G28" s="61" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="27">
-      <c r="F27" s="64"/>
-      <c r="G27" s="65"/>
-    </row>
-    <row r="28">
-      <c r="F28" s="64"/>
-      <c r="G28" s="65" t="s">
+    <row r="29">
+      <c r="F29" s="60"/>
+      <c r="G29" s="61" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="29">
-      <c r="F29" s="64"/>
-      <c r="G29" s="65" t="s">
+    <row r="30">
+      <c r="C30" s="62"/>
+      <c r="F30" s="60"/>
+      <c r="G30" s="61" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="30">
-      <c r="C30" s="66"/>
-      <c r="F30" s="64"/>
-      <c r="G30" s="65" t="s">
+    <row r="31">
+      <c r="F31" s="60"/>
+      <c r="G31" s="63" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="31">
-      <c r="F31" s="64"/>
-      <c r="G31" s="67" t="s">
+    <row r="32">
+      <c r="C32" s="25"/>
+      <c r="F32" s="56" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="26"/>
-      <c r="F32" s="60" t="s">
+      <c r="G32" s="64" t="s">
         <v>177</v>
       </c>
-      <c r="G32" s="68" t="s">
-        <v>178</v>
-      </c>
     </row>
     <row r="33">
-      <c r="C33" s="57"/>
+      <c r="C33" s="53"/>
     </row>
     <row r="34">
-      <c r="C34" s="57"/>
+      <c r="C34" s="53"/>
     </row>
     <row r="36">
-      <c r="C36" s="66"/>
+      <c r="C36" s="62"/>
     </row>
     <row r="38">
-      <c r="C38" s="26"/>
+      <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="57"/>
+      <c r="C39" s="53"/>
     </row>
     <row r="40">
-      <c r="C40" s="57"/>
+      <c r="C40" s="53"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -3976,367 +3971,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" t="s">
         <v>179</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" s="65" t="s">
         <v>180</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="E5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" t="s">
         <v>181</v>
       </c>
-      <c r="E5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>182</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>183</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>184</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>185</v>
-      </c>
-      <c r="K5" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6" t="s">
         <v>187</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" s="66" t="s">
         <v>188</v>
       </c>
-      <c r="D6" s="70" t="s">
+      <c r="E6" t="s">
         <v>189</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>190</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>191</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" s="67" t="s">
         <v>192</v>
       </c>
-      <c r="H6" s="71" t="s">
+      <c r="I6" t="s">
         <v>193</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>194</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>195</v>
-      </c>
-      <c r="K6" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="68" t="s">
         <v>197</v>
       </c>
-      <c r="B7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D7" s="72" t="s">
+      <c r="F7" t="s">
         <v>198</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>199</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="67" t="s">
         <v>200</v>
       </c>
-      <c r="H7" s="71" t="s">
+      <c r="K7" t="s">
         <v>201</v>
       </c>
-      <c r="K7" t="s">
+    </row>
+    <row r="8">
+      <c r="D8" s="66" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="70" t="s">
+      <c r="G8" s="69" t="s">
         <v>203</v>
       </c>
-      <c r="G8" s="73" t="s">
+      <c r="H8" s="67" t="s">
         <v>204</v>
-      </c>
-      <c r="H8" s="71" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" t="s">
         <v>206</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" s="68" t="s">
         <v>207</v>
       </c>
-      <c r="D9" s="72" t="s">
+      <c r="H9" s="67" t="s">
         <v>208</v>
-      </c>
-      <c r="H9" s="71" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B10" t="s">
         <v>210</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" s="66"/>
+      <c r="G10" t="s">
         <v>211</v>
       </c>
-      <c r="D10" s="70"/>
-      <c r="G10" t="s">
+      <c r="H10" s="67" t="s">
         <v>212</v>
-      </c>
-      <c r="H10" s="71" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>213</v>
+      </c>
+      <c r="B11" t="s">
         <v>214</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" s="68" t="s">
         <v>215</v>
       </c>
-      <c r="D11" s="72" t="s">
+      <c r="G11" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="G11" s="73" t="s">
+      <c r="H11" s="67" t="s">
         <v>217</v>
-      </c>
-      <c r="H11" s="71" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B12" t="s">
         <v>219</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" s="66" t="s">
         <v>220</v>
       </c>
-      <c r="D12" s="70" t="s">
+      <c r="G12" s="69" t="s">
         <v>221</v>
       </c>
-      <c r="G12" s="73" t="s">
+      <c r="H12" s="67" t="s">
         <v>222</v>
-      </c>
-      <c r="H12" s="71" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>223</v>
+      </c>
+      <c r="B13" t="s">
         <v>224</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="D13" s="72" t="s">
+      <c r="G13" s="69" t="s">
         <v>226</v>
       </c>
-      <c r="G13" s="73" t="s">
+    </row>
+    <row r="14">
+      <c r="D14" s="66" t="s">
         <v>227</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="70" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>228</v>
+      </c>
+      <c r="B15" t="s">
         <v>229</v>
       </c>
-      <c r="B15" t="s">
-        <v>230</v>
-      </c>
-      <c r="D15" s="72"/>
+      <c r="D15" s="68"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>230</v>
+      </c>
+      <c r="B16" t="s">
         <v>231</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" s="66"/>
+      <c r="G16" t="s">
         <v>232</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="G16" t="s">
+    </row>
+    <row r="17">
+      <c r="D17" s="68"/>
+      <c r="G17" s="69" t="s">
         <v>233</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="72"/>
-      <c r="G17" s="73" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>234</v>
+      </c>
+      <c r="D18" s="66"/>
+      <c r="G18" s="70" t="s">
         <v>235</v>
       </c>
-      <c r="D18" s="70"/>
-      <c r="G18" s="74" t="s">
+    </row>
+    <row r="19">
+      <c r="D19" s="68" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="72" t="s">
+      <c r="E19" t="s">
         <v>237</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" s="70" t="s">
         <v>238</v>
       </c>
-      <c r="G19" s="74" t="s">
+      <c r="H19" t="s">
         <v>239</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>240</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="66"/>
+      <c r="G20" s="70" t="s">
         <v>241</v>
       </c>
-      <c r="J19" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="70"/>
-      <c r="G20" s="74" t="s">
+    </row>
+    <row r="22">
+      <c r="D22" s="66"/>
+      <c r="G22" s="70" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="69"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="66"/>
+      <c r="G24" s="69" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="22">
-      <c r="D22" s="70"/>
-      <c r="G22" s="74" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="G23" s="73"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="70"/>
-      <c r="G24" s="73" t="s">
+    <row r="25">
+      <c r="G25" s="70" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="25">
-      <c r="G25" s="74" t="s">
+    <row r="26">
+      <c r="D26" s="66"/>
+      <c r="G26" s="70" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="26">
-      <c r="D26" s="70"/>
-      <c r="G26" s="74" t="s">
+    <row r="27">
+      <c r="G27" s="70" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="27">
-      <c r="G27" s="74" t="s">
+    <row r="28">
+      <c r="D28" s="66"/>
+      <c r="G28" s="70" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="71" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="70"/>
-      <c r="G28" s="74" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" s="75" t="s">
+      <c r="E35" t="s">
         <v>247</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" s="72" t="s">
         <v>248</v>
       </c>
-      <c r="F35" s="76" t="s">
+    </row>
+    <row r="36">
+      <c r="D36" s="73" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="36">
-      <c r="D36" s="77" t="s">
+      <c r="E36" t="s">
         <v>250</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" s="73" t="s">
         <v>251</v>
       </c>
-      <c r="F36" s="77" t="s">
+    </row>
+    <row r="37">
+      <c r="D37" s="72" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="37">
-      <c r="D37" s="76" t="s">
+      <c r="E37" t="s">
         <v>253</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" s="72" t="s">
         <v>254</v>
       </c>
-      <c r="F37" s="76" t="s">
+    </row>
+    <row r="38">
+      <c r="D38" s="73" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="D38" s="77" t="s">
+      <c r="E38" t="s">
         <v>256</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" s="73" t="s">
         <v>257</v>
       </c>
-      <c r="F38" s="77" t="s">
+    </row>
+    <row r="39">
+      <c r="D39" s="72" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="D39" s="76" t="s">
+      <c r="E39" t="s">
         <v>259</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" s="72" t="s">
         <v>260</v>
-      </c>
-      <c r="F39" s="76" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>251</v>
-      </c>
-      <c r="F40" s="77" t="s">
-        <v>262</v>
+        <v>250</v>
+      </c>
+      <c r="F40" s="73" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>254</v>
-      </c>
-      <c r="F41" s="76" t="s">
-        <v>263</v>
+        <v>253</v>
+      </c>
+      <c r="F41" s="72" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -4367,564 +4362,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="78" t="s">
+      <c r="D4" s="74" t="s">
+        <v>265</v>
+      </c>
+      <c r="E4" t="s">
         <v>266</v>
-      </c>
-      <c r="E4" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" s="74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="70" t="s">
         <v>268</v>
       </c>
-      <c r="E5" s="78">
+      <c r="E6" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="74" t="s">
+    <row r="7">
+      <c r="D7" s="75" t="s">
         <v>269</v>
       </c>
-      <c r="E6" s="78">
+      <c r="E7" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="D7" s="79" t="s">
+    <row r="8">
+      <c r="D8" s="70" t="s">
         <v>270</v>
       </c>
-      <c r="E7" s="78">
+      <c r="E8" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="D8" s="74" t="s">
+    <row r="9">
+      <c r="D9" s="70"/>
+      <c r="E9" s="74"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="67" t="s">
         <v>271</v>
       </c>
-      <c r="E8" s="78">
+      <c r="E10" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="D9" s="74"/>
-      <c r="E9" s="78"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="71" t="s">
+    <row r="11">
+      <c r="D11" s="70" t="s">
         <v>272</v>
       </c>
-      <c r="E10" s="78">
+      <c r="E11" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="D11" s="74" t="s">
+    <row r="12">
+      <c r="D12" s="70" t="s">
         <v>273</v>
       </c>
-      <c r="E11" s="78">
+      <c r="E12" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="12">
-      <c r="D12" s="74" t="s">
+    <row r="13">
+      <c r="D13" s="70" t="s">
         <v>274</v>
       </c>
-      <c r="E12" s="78">
+      <c r="E13" s="74">
         <v>1</v>
       </c>
     </row>
-    <row r="13">
-      <c r="D13" s="74" t="s">
+    <row r="14">
+      <c r="D14" s="70"/>
+      <c r="E14" s="70"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="67" t="s">
         <v>275</v>
       </c>
-      <c r="E13" s="78">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="74"/>
-      <c r="E14" s="74"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="71" t="s">
+      <c r="E15" s="74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="76" t="s">
         <v>276</v>
       </c>
-      <c r="E15" s="78">
+      <c r="E16" s="74">
         <v>2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="D16" s="80" t="s">
+    <row r="17">
+      <c r="D17" s="77" t="s">
         <v>277</v>
       </c>
-      <c r="E16" s="78">
+      <c r="E17" s="74">
         <v>2</v>
       </c>
     </row>
-    <row r="17">
-      <c r="D17" s="81" t="s">
+    <row r="18">
+      <c r="D18" s="77" t="s">
         <v>278</v>
       </c>
-      <c r="E17" s="78">
+      <c r="E18" s="74">
         <v>2</v>
       </c>
     </row>
-    <row r="18">
-      <c r="D18" s="81" t="s">
+    <row r="19">
+      <c r="D19" s="70"/>
+      <c r="E19" s="70"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="67" t="s">
         <v>279</v>
       </c>
-      <c r="E18" s="78">
+      <c r="E20" s="74">
         <v>2</v>
       </c>
     </row>
-    <row r="19">
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="71" t="s">
+    <row r="21">
+      <c r="D21" s="67" t="s">
         <v>280</v>
       </c>
-      <c r="E20" s="78">
+      <c r="E21" s="74">
         <v>2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="D21" s="71" t="s">
+    <row r="22">
+      <c r="D22" s="70"/>
+      <c r="E22" s="70"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="78"/>
+      <c r="E23" s="70"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="70"/>
+      <c r="E24" s="70"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="70"/>
+      <c r="E25" s="70"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="70"/>
+      <c r="E26" s="70"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="70"/>
+      <c r="E27" s="70"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="70"/>
+      <c r="E28" s="70"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="70"/>
+      <c r="E29" s="70"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="70"/>
+      <c r="E30" s="70"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="79"/>
+      <c r="C39" s="80" t="s">
         <v>281</v>
       </c>
-      <c r="E21" s="78">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="82"/>
-      <c r="E23" s="74"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="74"/>
-      <c r="E25" s="74"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="74"/>
-      <c r="E26" s="74"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="74"/>
-      <c r="E27" s="74"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="74"/>
-      <c r="E28" s="74"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="74"/>
-      <c r="E29" s="74"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="74"/>
-      <c r="E30" s="74"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="83"/>
-      <c r="C39" s="84" t="s">
+      <c r="D39" s="80" t="s">
         <v>282</v>
       </c>
-      <c r="D39" s="84" t="s">
-        <v>283</v>
-      </c>
       <c r="E39" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="85">
+      <c r="C40" s="81">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="E40" s="74"/>
+    </row>
+    <row r="41">
+      <c r="C41" s="74" t="s">
         <v>284</v>
       </c>
-      <c r="E40" s="78"/>
-    </row>
-    <row r="41">
-      <c r="C41" s="78" t="s">
+      <c r="D41" s="70" t="s">
         <v>285</v>
       </c>
-      <c r="D41" s="74" t="s">
+      <c r="E41" s="74"/>
+    </row>
+    <row r="42" ht="14.25" customHeight="1">
+      <c r="C42" s="74" t="s">
         <v>286</v>
       </c>
-      <c r="E41" s="78"/>
-    </row>
-    <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="78" t="s">
+      <c r="D42" s="70" t="s">
         <v>287</v>
       </c>
-      <c r="D42" s="74" t="s">
+    </row>
+    <row r="43">
+      <c r="C43" s="74" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="C43" s="78" t="s">
+      <c r="D43" s="70" t="s">
         <v>289</v>
       </c>
-      <c r="D43" s="74" t="s">
+    </row>
+    <row r="44">
+      <c r="C44" s="82" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="44">
-      <c r="C44" s="86" t="s">
+      <c r="D44" s="75" t="s">
         <v>291</v>
       </c>
-      <c r="D44" s="79" t="s">
+      <c r="E44" s="83"/>
+      <c r="F44" s="83"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="80" t="s">
         <v>292</v>
       </c>
-      <c r="E44" s="87"/>
-      <c r="F44" s="87"/>
-    </row>
-    <row r="45">
-      <c r="C45" s="84" t="s">
+      <c r="D45" s="70" t="s">
         <v>293</v>
       </c>
-      <c r="D45" s="74" t="s">
+      <c r="E45" s="74"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="80" t="s">
         <v>294</v>
       </c>
-      <c r="E45" s="78"/>
-    </row>
-    <row r="46">
-      <c r="C46" s="84" t="s">
+      <c r="D46" s="70" t="s">
         <v>295</v>
       </c>
-      <c r="D46" s="74" t="s">
+      <c r="E46" s="74"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="84">
+        <v>2</v>
+      </c>
+      <c r="D47" s="85" t="s">
         <v>296</v>
       </c>
-      <c r="E46" s="78"/>
-    </row>
-    <row r="47">
-      <c r="C47" s="88">
-        <v>2</v>
-      </c>
-      <c r="D47" s="89" t="s">
+      <c r="E47" s="74"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="82" t="s">
         <v>297</v>
       </c>
-      <c r="E47" s="78"/>
-    </row>
-    <row r="48">
-      <c r="C48" s="86" t="s">
+      <c r="D48" s="75" t="s">
         <v>298</v>
       </c>
-      <c r="D48" s="79" t="s">
+      <c r="E48" s="74"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="81">
+        <v>3</v>
+      </c>
+      <c r="D49" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="E48" s="78"/>
-    </row>
-    <row r="49">
-      <c r="C49" s="85">
-        <v>3</v>
-      </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="74"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="82" t="s">
         <v>300</v>
       </c>
-      <c r="E49" s="78"/>
-    </row>
-    <row r="50">
-      <c r="C50" s="86" t="s">
+      <c r="D50" s="75" t="s">
         <v>301</v>
       </c>
-      <c r="D50" s="79" t="s">
+      <c r="F50" s="86" t="s">
         <v>302</v>
       </c>
-      <c r="F50" s="90" t="s">
+    </row>
+    <row r="51">
+      <c r="C51" s="82" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="C51" s="86" t="s">
+      <c r="D51" s="87" t="s">
         <v>304</v>
       </c>
-      <c r="D51" s="91" t="s">
+    </row>
+    <row r="52">
+      <c r="C52" s="82" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="C52" s="86" t="s">
+      <c r="D52" s="87" t="s">
         <v>306</v>
       </c>
-      <c r="D52" s="91" t="s">
+    </row>
+    <row r="53">
+      <c r="C53" s="82" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="86" t="s">
+      <c r="D53" s="87" t="s">
         <v>308</v>
       </c>
-      <c r="D53" s="91" t="s">
+    </row>
+    <row r="54">
+      <c r="C54" s="82" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="86" t="s">
+      <c r="D54" s="87" t="s">
         <v>310</v>
       </c>
-      <c r="D54" s="91" t="s">
+    </row>
+    <row r="55">
+      <c r="C55" s="88">
+        <v>4</v>
+      </c>
+      <c r="D55" s="88" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="55">
-      <c r="C55" s="92">
-        <v>4</v>
-      </c>
-      <c r="D55" s="92" t="s">
+    <row r="56">
+      <c r="C56" s="80" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="84" t="s">
+      <c r="D56" s="70" t="s">
         <v>313</v>
       </c>
-      <c r="D56" s="74" t="s">
+    </row>
+    <row r="57">
+      <c r="C57" s="80" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="84" t="s">
+      <c r="D57" s="87" t="s">
         <v>315</v>
       </c>
-      <c r="D57" s="91" t="s">
+    </row>
+    <row r="58">
+      <c r="C58" s="80" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="C58" s="84" t="s">
+      <c r="D58" s="87" t="s">
         <v>317</v>
       </c>
-      <c r="D58" s="91" t="s">
+    </row>
+    <row r="59">
+      <c r="C59" s="80" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="84" t="s">
+      <c r="D59" s="87" t="s">
         <v>319</v>
-      </c>
-      <c r="D59" s="91" t="s">
-        <v>320</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="92">
+      <c r="C60" s="88">
         <v>5</v>
       </c>
-      <c r="D60" s="92" t="s">
+      <c r="D60" s="88" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" s="80" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="61">
-      <c r="C61" s="84" t="s">
+      <c r="D61" s="70" t="s">
         <v>322</v>
       </c>
-      <c r="D61" s="74" t="s">
+    </row>
+    <row r="62">
+      <c r="C62" s="80" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="62">
-      <c r="C62" s="84" t="s">
+      <c r="D62" s="87" t="s">
         <v>324</v>
       </c>
-      <c r="D62" s="91" t="s">
+      <c r="F62" t="s">
         <v>325</v>
       </c>
-      <c r="F62" t="s">
+    </row>
+    <row r="63">
+      <c r="C63" s="80" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="63">
-      <c r="C63" s="84" t="s">
+      <c r="D63" s="87" t="s">
         <v>327</v>
       </c>
-      <c r="D63" s="91" t="s">
+    </row>
+    <row r="64">
+      <c r="C64" s="80" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="64">
-      <c r="C64" s="84" t="s">
+      <c r="D64" s="87" t="s">
         <v>329</v>
       </c>
-      <c r="D64" s="91" t="s">
+    </row>
+    <row r="65">
+      <c r="C65" s="88">
+        <v>6</v>
+      </c>
+      <c r="D65" s="88" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="65">
-      <c r="C65" s="92">
-        <v>6</v>
-      </c>
-      <c r="D65" s="92" t="s">
+    <row r="66">
+      <c r="C66" s="80" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="66">
-      <c r="C66" s="84" t="s">
+      <c r="D66" s="70" t="s">
         <v>332</v>
       </c>
-      <c r="D66" s="74" t="s">
+    </row>
+    <row r="67">
+      <c r="C67" s="89" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="67">
-      <c r="C67" s="93" t="s">
+      <c r="D67" s="90" t="s">
         <v>334</v>
       </c>
-      <c r="D67" s="94" t="s">
+    </row>
+    <row r="68">
+      <c r="C68" s="80" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="68">
-      <c r="C68" s="84" t="s">
+      <c r="D68" s="87" t="s">
         <v>336</v>
       </c>
-      <c r="D68" s="91" t="s">
+    </row>
+    <row r="69">
+      <c r="C69" s="89" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="69">
-      <c r="C69" s="93" t="s">
+      <c r="D69" s="87" t="s">
         <v>338</v>
       </c>
-      <c r="D69" s="91" t="s">
+    </row>
+    <row r="70">
+      <c r="C70" s="80" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="70">
-      <c r="C70" s="84" t="s">
+      <c r="D70" s="87" t="s">
         <v>340</v>
       </c>
-      <c r="D70" s="91" t="s">
+    </row>
+    <row r="71">
+      <c r="C71" s="88">
+        <v>7</v>
+      </c>
+      <c r="D71" s="5" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="71">
-      <c r="C71" s="92">
-        <v>7</v>
-      </c>
-      <c r="D71" s="5" t="s">
+    <row r="72">
+      <c r="C72" s="80" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="72">
-      <c r="C72" s="84" t="s">
+      <c r="D72" s="70" t="s">
         <v>343</v>
       </c>
-      <c r="D72" s="74" t="s">
+    </row>
+    <row r="73">
+      <c r="C73" s="88">
+        <v>8</v>
+      </c>
+      <c r="D73" s="5" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="73">
-      <c r="C73" s="92">
-        <v>8</v>
-      </c>
-      <c r="D73" s="5" t="s">
+    <row r="74">
+      <c r="C74" s="80" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="74">
-      <c r="C74" s="84" t="s">
+      <c r="D74" s="70" t="s">
         <v>346</v>
       </c>
-      <c r="D74" s="74" t="s">
+    </row>
+    <row r="75">
+      <c r="C75" s="88">
+        <v>9</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" s="80" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="75">
-      <c r="C75" s="92">
-        <v>9</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="C76" s="84" t="s">
+      <c r="D76" s="70" t="s">
         <v>348</v>
       </c>
-      <c r="D76" s="74" t="s">
+    </row>
+    <row r="77">
+      <c r="C77" s="80" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="77">
-      <c r="C77" s="84" t="s">
+      <c r="D77" s="87" t="s">
         <v>350</v>
       </c>
-      <c r="D77" s="91" t="s">
+    </row>
+    <row r="78">
+      <c r="C78" s="80" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="78">
-      <c r="C78" s="84" t="s">
+      <c r="D78" s="87" t="s">
         <v>352</v>
       </c>
-      <c r="D78" s="91" t="s">
+    </row>
+    <row r="79">
+      <c r="C79" s="88">
+        <v>10</v>
+      </c>
+      <c r="D79" s="5" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="79">
-      <c r="C79" s="92">
-        <v>10</v>
-      </c>
-      <c r="D79" s="5" t="s">
+    <row r="80">
+      <c r="C80" s="80" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="80">
-      <c r="C80" s="84" t="s">
+      <c r="D80" s="70" t="s">
         <v>355</v>
       </c>
-      <c r="D80" s="74" t="s">
+      <c r="E80" s="74"/>
+    </row>
+    <row r="81">
+      <c r="C81" s="80" t="s">
         <v>356</v>
       </c>
-      <c r="E80" s="78"/>
-    </row>
-    <row r="81">
-      <c r="C81" s="84" t="s">
+      <c r="D81" s="87" t="s">
         <v>357</v>
       </c>
-      <c r="D81" s="91" t="s">
+    </row>
+    <row r="82">
+      <c r="C82" s="88">
+        <v>11</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="82">
-      <c r="C82" s="92">
-        <v>11</v>
-      </c>
-      <c r="D82" s="5" t="s">
+    <row r="83">
+      <c r="C83" s="80" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="83">
-      <c r="C83" s="84" t="s">
+      <c r="D83" s="70" t="s">
         <v>360</v>
       </c>
-      <c r="D83" s="74" t="s">
+    </row>
+    <row r="84">
+      <c r="C84" s="80" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="84">
-      <c r="C84" s="84" t="s">
+      <c r="D84" s="70" t="s">
         <v>362</v>
-      </c>
-      <c r="D84" s="74" t="s">
-        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove data in response
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="365">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -223,13 +223,19 @@
     # Calcul distance max : bas/gauche-haut/droite
     # Menu parametrage positions manuel
         # Voir dessin
+# Compter nb step marche plus Raspberry voir commit
+- Machine a etat OK local pas sur Raspberry : init ok mais goToPos KO
 - Calcul pas de déplacement pour aller àla pos voulu
+    - OK ça marche? Mais pas de retour API dcp attent dans le vide
 - Appeler GoToPos 2 fois : aller de a à b avec action sur CD, PUIS aller de b à c avec action CD
 -Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
    - Menu parametre être plus précis + save pos haut et pos bas
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Commit 9e907e5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prévoir tiges? pour fixer armature à planche, avec une certaine distance</t>
   </si>
   <si>
@@ -369,6 +375,9 @@
   </si>
   <si>
     <t xml:space="preserve">Animation photo d'un album lancé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image du projet sur la Raspberry</t>
   </si>
   <si>
     <t xml:space="preserve">Vidéo présentation</t>
@@ -1679,7 +1688,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1737,6 +1746,9 @@
     <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
@@ -3014,16 +3026,19 @@
       <c r="Z20" s="1"/>
       <c r="AA20" s="1"/>
     </row>
-    <row r="21" ht="199.5">
+    <row r="21" ht="270.75">
       <c r="A21" s="1"/>
       <c r="B21" s="34" t="s">
         <v>63</v>
       </c>
+      <c r="C21" s="35" t="s">
+        <v>64</v>
+      </c>
       <c r="D21" s="32">
         <v>0.45000000000000001</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>23</v>
@@ -3031,7 +3046,7 @@
       <c r="H21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M21" s="33" t="s">
         <v>62</v>
@@ -3045,7 +3060,7 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="X21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
@@ -3057,24 +3072,24 @@
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M22" s="33" t="s">
         <v>62</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3082,7 +3097,7 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
@@ -3091,11 +3106,11 @@
       <c r="A23" s="1"/>
       <c r="D23" s="32"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M23" s="33" t="s">
         <v>62</v>
@@ -3104,35 +3119,35 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
-      <c r="F24" s="36" t="s">
-        <v>75</v>
+      <c r="F24" s="37" t="s">
+        <v>76</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="37"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="39"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="40"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3148,10 +3163,10 @@
     <row r="25" ht="16.5">
       <c r="A25" s="1"/>
       <c r="B25" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C25" s="13"/>
-      <c r="D25" s="40">
+      <c r="D25" s="41">
         <f>SUM(D26:D31)/5</f>
         <v>0</v>
       </c>
@@ -3175,10 +3190,10 @@
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D26" s="32">
         <v>0</v>
@@ -3193,10 +3208,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3209,7 +3224,7 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="C27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D27" s="32">
         <v>0</v>
@@ -3223,7 +3238,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3231,7 +3246,7 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" s="32">
         <v>0</v>
@@ -3247,7 +3262,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3255,10 +3270,10 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D29" s="32">
         <v>0</v>
@@ -3278,10 +3293,10 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D30" s="32">
         <v>0</v>
@@ -3302,7 +3317,7 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D31" s="32">
         <v>0</v>
@@ -3323,7 +3338,7 @@
       <c r="B32" s="4"/>
       <c r="D32" s="32"/>
       <c r="L32" s="19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3333,7 +3348,7 @@
       <c r="B33" s="4"/>
       <c r="D33" s="32"/>
       <c r="L33" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3359,11 +3374,11 @@
     </row>
     <row r="35" ht="16.5">
       <c r="A35" s="1"/>
-      <c r="B35" s="41" t="s">
-        <v>94</v>
+      <c r="B35" s="42" t="s">
+        <v>95</v>
       </c>
       <c r="C35" s="13"/>
-      <c r="D35" s="40">
+      <c r="D35" s="41">
         <f>SUM(D36:D39)/4</f>
         <v>0</v>
       </c>
@@ -3381,10 +3396,10 @@
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
       <c r="B36" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D36" s="32">
         <v>0</v>
@@ -3403,10 +3418,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D37" s="32">
         <v>0</v>
@@ -3425,10 +3440,10 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D38" s="32">
         <v>0</v>
@@ -3447,10 +3462,10 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D39" s="32">
         <v>0</v>
@@ -3462,7 +3477,7 @@
     <row r="41" ht="16.5">
       <c r="A41" s="1"/>
       <c r="B41" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -3470,7 +3485,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3481,7 +3496,7 @@
     <row r="44" ht="16.5">
       <c r="A44" s="1"/>
       <c r="B44" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" ht="16.5">
@@ -3493,7 +3508,7 @@
     <row r="47" ht="14.25">
       <c r="A47" s="1"/>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" ht="14.25">
@@ -3502,13 +3517,13 @@
     <row r="49" ht="14.25">
       <c r="A49" s="1"/>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" ht="14.25">
@@ -3520,13 +3535,13 @@
     <row r="53" ht="16.5">
       <c r="A53" s="1"/>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3554,6 +3569,9 @@
     </row>
     <row r="56" ht="16.5">
       <c r="A56" s="1"/>
+      <c r="B56" t="s">
+        <v>112</v>
+      </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -3593,55 +3611,55 @@
     </row>
     <row r="68" ht="14.25">
       <c r="B68" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" ht="14.25">
       <c r="B69" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C77" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3671,280 +3689,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="42" t="s">
-        <v>121</v>
-      </c>
-      <c r="G2" s="43" t="s">
-        <v>122</v>
+      <c r="F2" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="44" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="3">
-      <c r="F3" s="44" t="s">
-        <v>123</v>
-      </c>
-      <c r="G3" s="45" t="s">
-        <v>124</v>
+      <c r="F3" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="G3" s="46" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="4">
-      <c r="F4" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="G4" s="47" t="s">
-        <v>126</v>
+      <c r="F4" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="G4" s="48" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="F5" s="48" t="s">
-        <v>127</v>
-      </c>
-      <c r="G5" s="49" t="s">
-        <v>128</v>
+      <c r="F5" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="G5" s="50" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="F6" s="50"/>
-      <c r="G6" s="51" t="s">
-        <v>129</v>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="F7" s="50"/>
-      <c r="G7" s="51" t="s">
-        <v>130</v>
+      <c r="F7" s="51"/>
+      <c r="G7" s="52" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="F8" s="50"/>
-      <c r="G8" s="51" t="s">
-        <v>131</v>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>132</v>
-      </c>
-      <c r="F9" s="50"/>
-      <c r="G9" s="51" t="s">
-        <v>133</v>
+        <v>134</v>
+      </c>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C10" s="52" t="s">
-        <v>135</v>
-      </c>
-      <c r="F10" s="50"/>
-      <c r="G10" s="51" t="s">
         <v>136</v>
       </c>
+      <c r="C10" s="53" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="11" ht="15">
-      <c r="C11" s="53" t="s">
-        <v>137</v>
-      </c>
-      <c r="F11" s="50"/>
-      <c r="G11" s="51" t="s">
-        <v>138</v>
+      <c r="C11" s="54" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="C12" s="52" t="s">
-        <v>139</v>
-      </c>
-      <c r="F12" s="44"/>
-      <c r="G12" s="54" t="s">
-        <v>140</v>
+      <c r="C12" s="53" t="s">
+        <v>141</v>
+      </c>
+      <c r="F12" s="45"/>
+      <c r="G12" s="55" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="13" ht="15">
-      <c r="C13" s="53" t="s">
-        <v>141</v>
-      </c>
-      <c r="F13" s="46" t="s">
-        <v>142</v>
-      </c>
-      <c r="G13" s="55" t="s">
+      <c r="C13" s="54" t="s">
         <v>143</v>
       </c>
+      <c r="F13" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="G13" s="56" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="14" ht="15">
-      <c r="C14" s="52" t="s">
-        <v>144</v>
-      </c>
-      <c r="F14" s="56" t="s">
-        <v>145</v>
-      </c>
-      <c r="G14" s="57" t="s">
+      <c r="C14" s="53" t="s">
         <v>146</v>
       </c>
+      <c r="F14" s="57" t="s">
+        <v>147</v>
+      </c>
+      <c r="G14" s="58" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="15">
-      <c r="C15" s="53" t="s">
-        <v>147</v>
-      </c>
-      <c r="F15" s="58" t="s">
-        <v>148</v>
-      </c>
-      <c r="G15" s="59" t="s">
+      <c r="C15" s="54" t="s">
         <v>149</v>
       </c>
+      <c r="F15" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" s="60" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="16">
-      <c r="C16" s="53" t="s">
-        <v>150</v>
-      </c>
-      <c r="F16" s="60" t="s">
-        <v>151</v>
-      </c>
-      <c r="G16" s="61" t="s">
+      <c r="C16" s="54" t="s">
         <v>152</v>
       </c>
+      <c r="F16" s="61" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" s="62" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="17">
-      <c r="C17" s="52" t="s">
-        <v>153</v>
-      </c>
-      <c r="F17" s="60"/>
-      <c r="G17" s="61" t="s">
-        <v>154</v>
+      <c r="C17" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" s="61"/>
+      <c r="G17" s="62" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="53" t="s">
-        <v>155</v>
-      </c>
-      <c r="F18" s="60"/>
-      <c r="G18" s="61" t="s">
-        <v>156</v>
+      <c r="C18" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="F18" s="61"/>
+      <c r="G18" s="62" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="53" t="s">
-        <v>157</v>
-      </c>
-      <c r="F19" s="60"/>
-      <c r="G19" s="61" t="s">
-        <v>158</v>
+      <c r="C19" s="54" t="s">
+        <v>159</v>
+      </c>
+      <c r="F19" s="61"/>
+      <c r="G19" s="62" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="53" t="s">
-        <v>159</v>
-      </c>
-      <c r="F20" s="60"/>
-      <c r="G20" s="61" t="s">
-        <v>160</v>
+      <c r="C20" s="54" t="s">
+        <v>161</v>
+      </c>
+      <c r="F20" s="61"/>
+      <c r="G20" s="62" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61" t="s">
-        <v>162</v>
+      <c r="C21" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="F21" s="61"/>
+      <c r="G21" s="62" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="52" t="s">
-        <v>163</v>
-      </c>
-      <c r="F22" s="60"/>
-      <c r="G22" s="61" t="s">
-        <v>164</v>
+      <c r="C22" s="53" t="s">
+        <v>165</v>
+      </c>
+      <c r="F22" s="61"/>
+      <c r="G22" s="62" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="53" t="s">
-        <v>165</v>
-      </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="61" t="s">
-        <v>166</v>
+      <c r="C23" s="54" t="s">
+        <v>167</v>
+      </c>
+      <c r="F23" s="61"/>
+      <c r="G23" s="62" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="52" t="s">
-        <v>167</v>
-      </c>
-      <c r="F24" s="60"/>
-      <c r="G24" s="61" t="s">
-        <v>168</v>
+      <c r="C24" s="53" t="s">
+        <v>169</v>
+      </c>
+      <c r="F24" s="61"/>
+      <c r="G24" s="62" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="F25" s="60"/>
-      <c r="G25" s="61" t="s">
-        <v>170</v>
+      <c r="C25" s="54" t="s">
+        <v>171</v>
+      </c>
+      <c r="F25" s="61"/>
+      <c r="G25" s="62" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="26">
-      <c r="F26" s="60"/>
-      <c r="G26" s="61" t="s">
-        <v>171</v>
+      <c r="F26" s="61"/>
+      <c r="G26" s="62" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="60"/>
-      <c r="G27" s="61"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="62"/>
     </row>
     <row r="28">
-      <c r="F28" s="60"/>
-      <c r="G28" s="61" t="s">
-        <v>172</v>
+      <c r="F28" s="61"/>
+      <c r="G28" s="62" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="60"/>
-      <c r="G29" s="61" t="s">
-        <v>173</v>
+      <c r="F29" s="61"/>
+      <c r="G29" s="62" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="62"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="61" t="s">
-        <v>174</v>
+      <c r="C30" s="63"/>
+      <c r="F30" s="61"/>
+      <c r="G30" s="62" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="60"/>
-      <c r="G31" s="63" t="s">
-        <v>175</v>
+      <c r="F31" s="61"/>
+      <c r="G31" s="64" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="56" t="s">
-        <v>176</v>
-      </c>
-      <c r="G32" s="64" t="s">
-        <v>177</v>
+      <c r="F32" s="57" t="s">
+        <v>178</v>
+      </c>
+      <c r="G32" s="65" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="53"/>
+      <c r="C33" s="54"/>
     </row>
     <row r="34">
-      <c r="C34" s="53"/>
+      <c r="C34" s="54"/>
     </row>
     <row r="36">
-      <c r="C36" s="62"/>
+      <c r="C36" s="63"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="53"/>
+      <c r="C39" s="54"/>
     </row>
     <row r="40">
-      <c r="C40" s="53"/>
+      <c r="C40" s="54"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -3972,367 +3990,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D5" s="65" t="s">
-        <v>180</v>
+        <v>181</v>
+      </c>
+      <c r="D5" s="66" t="s">
+        <v>182</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D6" s="66" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+      <c r="D6" s="67" t="s">
+        <v>190</v>
       </c>
       <c r="E6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G6" t="s">
-        <v>191</v>
-      </c>
-      <c r="H6" s="67" t="s">
-        <v>192</v>
+        <v>193</v>
+      </c>
+      <c r="H6" s="68" t="s">
+        <v>194</v>
       </c>
       <c r="I6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="K6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
-        <v>187</v>
-      </c>
-      <c r="D7" s="68" t="s">
-        <v>197</v>
+        <v>189</v>
+      </c>
+      <c r="D7" s="69" t="s">
+        <v>199</v>
       </c>
       <c r="F7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G7" t="s">
-        <v>199</v>
-      </c>
-      <c r="H7" s="67" t="s">
-        <v>200</v>
+        <v>201</v>
+      </c>
+      <c r="H7" s="68" t="s">
+        <v>202</v>
       </c>
       <c r="K7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="66" t="s">
-        <v>202</v>
-      </c>
-      <c r="G8" s="69" t="s">
-        <v>203</v>
-      </c>
-      <c r="H8" s="67" t="s">
+      <c r="D8" s="67" t="s">
         <v>204</v>
+      </c>
+      <c r="G8" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="H8" s="68" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B9" t="s">
-        <v>206</v>
-      </c>
-      <c r="D9" s="68" t="s">
-        <v>207</v>
-      </c>
-      <c r="H9" s="67" t="s">
         <v>208</v>
+      </c>
+      <c r="D9" s="69" t="s">
+        <v>209</v>
+      </c>
+      <c r="H9" s="68" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B10" t="s">
-        <v>210</v>
-      </c>
-      <c r="D10" s="66"/>
+        <v>212</v>
+      </c>
+      <c r="D10" s="67"/>
       <c r="G10" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="67" t="s">
-        <v>212</v>
+        <v>213</v>
+      </c>
+      <c r="H10" s="68" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B11" t="s">
-        <v>214</v>
-      </c>
-      <c r="D11" s="68" t="s">
-        <v>215</v>
-      </c>
-      <c r="G11" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="H11" s="67" t="s">
+      <c r="D11" s="69" t="s">
         <v>217</v>
+      </c>
+      <c r="G11" s="70" t="s">
+        <v>218</v>
+      </c>
+      <c r="H11" s="68" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B12" t="s">
-        <v>219</v>
-      </c>
-      <c r="D12" s="66" t="s">
-        <v>220</v>
-      </c>
-      <c r="G12" s="69" t="s">
         <v>221</v>
       </c>
-      <c r="H12" s="67" t="s">
+      <c r="D12" s="67" t="s">
         <v>222</v>
+      </c>
+      <c r="G12" s="70" t="s">
+        <v>223</v>
+      </c>
+      <c r="H12" s="68" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>224</v>
-      </c>
-      <c r="D13" s="68" t="s">
-        <v>225</v>
-      </c>
-      <c r="G13" s="69" t="s">
         <v>226</v>
       </c>
+      <c r="D13" s="69" t="s">
+        <v>227</v>
+      </c>
+      <c r="G13" s="70" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="14">
-      <c r="D14" s="66" t="s">
-        <v>227</v>
+      <c r="D14" s="67" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B15" t="s">
-        <v>229</v>
-      </c>
-      <c r="D15" s="68"/>
+        <v>231</v>
+      </c>
+      <c r="D15" s="69"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B16" t="s">
-        <v>231</v>
-      </c>
-      <c r="D16" s="66"/>
+        <v>233</v>
+      </c>
+      <c r="D16" s="67"/>
       <c r="G16" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="68"/>
-      <c r="G17" s="69" t="s">
-        <v>233</v>
+      <c r="D17" s="69"/>
+      <c r="G17" s="70" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>234</v>
-      </c>
-      <c r="D18" s="66"/>
-      <c r="G18" s="70" t="s">
-        <v>235</v>
+        <v>236</v>
+      </c>
+      <c r="D18" s="67"/>
+      <c r="G18" s="71" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="68" t="s">
-        <v>236</v>
+      <c r="D19" s="69" t="s">
+        <v>238</v>
       </c>
       <c r="E19" t="s">
-        <v>237</v>
-      </c>
-      <c r="G19" s="70" t="s">
-        <v>238</v>
+        <v>239</v>
+      </c>
+      <c r="G19" s="71" t="s">
+        <v>240</v>
       </c>
       <c r="H19" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I19" t="s">
+        <v>242</v>
+      </c>
+      <c r="J19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="67"/>
+      <c r="G20" s="71" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="67"/>
+      <c r="G22" s="71" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="70"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="67"/>
+      <c r="G24" s="70" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="71" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="67"/>
+      <c r="G26" s="71" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="71" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="67"/>
+      <c r="G28" s="71" t="s">
         <v>240</v>
       </c>
-      <c r="J19" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="66"/>
-      <c r="G20" s="70" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="66"/>
-      <c r="G22" s="70" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="G23" s="69"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="66"/>
-      <c r="G24" s="69" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" s="70" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" s="66"/>
-      <c r="G26" s="70" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="70" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="66"/>
-      <c r="G28" s="70" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="35">
-      <c r="D35" s="71" t="s">
-        <v>246</v>
+      <c r="D35" s="72" t="s">
+        <v>248</v>
       </c>
       <c r="E35" t="s">
-        <v>247</v>
-      </c>
-      <c r="F35" s="72" t="s">
-        <v>248</v>
+        <v>249</v>
+      </c>
+      <c r="F35" s="73" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="36">
-      <c r="D36" s="73" t="s">
-        <v>249</v>
+      <c r="D36" s="74" t="s">
+        <v>251</v>
       </c>
       <c r="E36" t="s">
-        <v>250</v>
-      </c>
-      <c r="F36" s="73" t="s">
-        <v>251</v>
+        <v>252</v>
+      </c>
+      <c r="F36" s="74" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="37">
-      <c r="D37" s="72" t="s">
-        <v>252</v>
+      <c r="D37" s="73" t="s">
+        <v>254</v>
       </c>
       <c r="E37" t="s">
-        <v>253</v>
-      </c>
-      <c r="F37" s="72" t="s">
-        <v>254</v>
+        <v>255</v>
+      </c>
+      <c r="F37" s="73" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="73" t="s">
-        <v>255</v>
+      <c r="D38" s="74" t="s">
+        <v>257</v>
       </c>
       <c r="E38" t="s">
-        <v>256</v>
-      </c>
-      <c r="F38" s="73" t="s">
-        <v>257</v>
+        <v>258</v>
+      </c>
+      <c r="F38" s="74" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="39">
-      <c r="D39" s="72" t="s">
-        <v>258</v>
+      <c r="D39" s="73" t="s">
+        <v>260</v>
       </c>
       <c r="E39" t="s">
-        <v>259</v>
-      </c>
-      <c r="F39" s="72" t="s">
-        <v>260</v>
+        <v>261</v>
+      </c>
+      <c r="F39" s="73" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>250</v>
-      </c>
-      <c r="F40" s="73" t="s">
-        <v>261</v>
+        <v>252</v>
+      </c>
+      <c r="F40" s="74" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>253</v>
-      </c>
-      <c r="F41" s="72" t="s">
-        <v>262</v>
+        <v>255</v>
+      </c>
+      <c r="F41" s="73" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -4363,564 +4381,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="74" t="s">
-        <v>265</v>
+      <c r="D4" s="75" t="s">
+        <v>267</v>
       </c>
       <c r="E4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
-        <v>267</v>
-      </c>
-      <c r="E5" s="74">
+        <v>269</v>
+      </c>
+      <c r="E5" s="75">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="70" t="s">
+      <c r="D6" s="71" t="s">
+        <v>270</v>
+      </c>
+      <c r="E6" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="76" t="s">
+        <v>271</v>
+      </c>
+      <c r="E7" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="71" t="s">
+        <v>272</v>
+      </c>
+      <c r="E8" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="71"/>
+      <c r="E9" s="75"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="68" t="s">
+        <v>273</v>
+      </c>
+      <c r="E10" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="71" t="s">
+        <v>274</v>
+      </c>
+      <c r="E11" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="71" t="s">
+        <v>275</v>
+      </c>
+      <c r="E12" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="71" t="s">
+        <v>276</v>
+      </c>
+      <c r="E13" s="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="68" t="s">
+        <v>277</v>
+      </c>
+      <c r="E15" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="77" t="s">
+        <v>278</v>
+      </c>
+      <c r="E16" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="78" t="s">
+        <v>279</v>
+      </c>
+      <c r="E17" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="78" t="s">
+        <v>280</v>
+      </c>
+      <c r="E18" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="71"/>
+      <c r="E19" s="71"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="68" t="s">
+        <v>281</v>
+      </c>
+      <c r="E20" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" s="68" t="s">
+        <v>282</v>
+      </c>
+      <c r="E21" s="75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="71"/>
+      <c r="E22" s="71"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="79"/>
+      <c r="E23" s="71"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="71"/>
+      <c r="E24" s="71"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="71"/>
+      <c r="E25" s="71"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="71"/>
+      <c r="E28" s="71"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="71"/>
+      <c r="E29" s="71"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="71"/>
+      <c r="E30" s="71"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="80"/>
+      <c r="C39" s="81" t="s">
+        <v>283</v>
+      </c>
+      <c r="D39" s="81" t="s">
+        <v>284</v>
+      </c>
+      <c r="E39" t="s">
         <v>268</v>
-      </c>
-      <c r="E6" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" s="75" t="s">
-        <v>269</v>
-      </c>
-      <c r="E7" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="70" t="s">
-        <v>270</v>
-      </c>
-      <c r="E8" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="70"/>
-      <c r="E9" s="74"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="67" t="s">
-        <v>271</v>
-      </c>
-      <c r="E10" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" s="70" t="s">
-        <v>272</v>
-      </c>
-      <c r="E11" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="70" t="s">
-        <v>273</v>
-      </c>
-      <c r="E12" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="70" t="s">
-        <v>274</v>
-      </c>
-      <c r="E13" s="74">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="70"/>
-      <c r="E14" s="70"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="67" t="s">
-        <v>275</v>
-      </c>
-      <c r="E15" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="76" t="s">
-        <v>276</v>
-      </c>
-      <c r="E16" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="77" t="s">
-        <v>277</v>
-      </c>
-      <c r="E17" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" s="77" t="s">
-        <v>278</v>
-      </c>
-      <c r="E18" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="70"/>
-      <c r="E19" s="70"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="67" t="s">
-        <v>279</v>
-      </c>
-      <c r="E20" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" s="67" t="s">
-        <v>280</v>
-      </c>
-      <c r="E21" s="74">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="70"/>
-      <c r="E22" s="70"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="78"/>
-      <c r="E23" s="70"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="70"/>
-      <c r="E25" s="70"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="70"/>
-      <c r="E26" s="70"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="70"/>
-      <c r="E27" s="70"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="70"/>
-      <c r="E28" s="70"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="70"/>
-      <c r="E29" s="70"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="79"/>
-      <c r="C39" s="80" t="s">
-        <v>281</v>
-      </c>
-      <c r="D39" s="80" t="s">
-        <v>282</v>
-      </c>
-      <c r="E39" t="s">
-        <v>266</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="81">
+      <c r="C40" s="82">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="E40" s="74"/>
+        <v>285</v>
+      </c>
+      <c r="E40" s="75"/>
     </row>
     <row r="41">
-      <c r="C41" s="74" t="s">
-        <v>284</v>
-      </c>
-      <c r="D41" s="70" t="s">
-        <v>285</v>
-      </c>
-      <c r="E41" s="74"/>
+      <c r="C41" s="75" t="s">
+        <v>286</v>
+      </c>
+      <c r="D41" s="71" t="s">
+        <v>287</v>
+      </c>
+      <c r="E41" s="75"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="74" t="s">
-        <v>286</v>
-      </c>
-      <c r="D42" s="70" t="s">
-        <v>287</v>
+      <c r="C42" s="75" t="s">
+        <v>288</v>
+      </c>
+      <c r="D42" s="71" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="74" t="s">
-        <v>288</v>
-      </c>
-      <c r="D43" s="70" t="s">
-        <v>289</v>
+      <c r="C43" s="75" t="s">
+        <v>290</v>
+      </c>
+      <c r="D43" s="71" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="82" t="s">
-        <v>290</v>
-      </c>
-      <c r="D44" s="75" t="s">
-        <v>291</v>
-      </c>
-      <c r="E44" s="83"/>
-      <c r="F44" s="83"/>
+      <c r="C44" s="83" t="s">
+        <v>292</v>
+      </c>
+      <c r="D44" s="76" t="s">
+        <v>293</v>
+      </c>
+      <c r="E44" s="84"/>
+      <c r="F44" s="84"/>
     </row>
     <row r="45">
-      <c r="C45" s="80" t="s">
-        <v>292</v>
-      </c>
-      <c r="D45" s="70" t="s">
-        <v>293</v>
-      </c>
-      <c r="E45" s="74"/>
+      <c r="C45" s="81" t="s">
+        <v>294</v>
+      </c>
+      <c r="D45" s="71" t="s">
+        <v>295</v>
+      </c>
+      <c r="E45" s="75"/>
     </row>
     <row r="46">
-      <c r="C46" s="80" t="s">
-        <v>294</v>
-      </c>
-      <c r="D46" s="70" t="s">
-        <v>295</v>
-      </c>
-      <c r="E46" s="74"/>
+      <c r="C46" s="81" t="s">
+        <v>296</v>
+      </c>
+      <c r="D46" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="E46" s="75"/>
     </row>
     <row r="47">
-      <c r="C47" s="84">
+      <c r="C47" s="85">
         <v>2</v>
       </c>
-      <c r="D47" s="85" t="s">
-        <v>296</v>
-      </c>
-      <c r="E47" s="74"/>
+      <c r="D47" s="86" t="s">
+        <v>298</v>
+      </c>
+      <c r="E47" s="75"/>
     </row>
     <row r="48">
-      <c r="C48" s="82" t="s">
-        <v>297</v>
-      </c>
-      <c r="D48" s="75" t="s">
-        <v>298</v>
-      </c>
-      <c r="E48" s="74"/>
+      <c r="C48" s="83" t="s">
+        <v>299</v>
+      </c>
+      <c r="D48" s="76" t="s">
+        <v>300</v>
+      </c>
+      <c r="E48" s="75"/>
     </row>
     <row r="49">
-      <c r="C49" s="81">
+      <c r="C49" s="82">
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="E49" s="74"/>
+        <v>301</v>
+      </c>
+      <c r="E49" s="75"/>
     </row>
     <row r="50">
-      <c r="C50" s="82" t="s">
-        <v>300</v>
-      </c>
-      <c r="D50" s="75" t="s">
-        <v>301</v>
-      </c>
-      <c r="F50" s="86" t="s">
+      <c r="C50" s="83" t="s">
         <v>302</v>
       </c>
+      <c r="D50" s="76" t="s">
+        <v>303</v>
+      </c>
+      <c r="F50" s="87" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="51">
-      <c r="C51" s="82" t="s">
-        <v>303</v>
-      </c>
-      <c r="D51" s="87" t="s">
-        <v>304</v>
+      <c r="C51" s="83" t="s">
+        <v>305</v>
+      </c>
+      <c r="D51" s="88" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="82" t="s">
-        <v>305</v>
-      </c>
-      <c r="D52" s="87" t="s">
-        <v>306</v>
+      <c r="C52" s="83" t="s">
+        <v>307</v>
+      </c>
+      <c r="D52" s="88" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="82" t="s">
-        <v>307</v>
-      </c>
-      <c r="D53" s="87" t="s">
-        <v>308</v>
+      <c r="C53" s="83" t="s">
+        <v>309</v>
+      </c>
+      <c r="D53" s="88" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="82" t="s">
-        <v>309</v>
-      </c>
-      <c r="D54" s="87" t="s">
-        <v>310</v>
+      <c r="C54" s="83" t="s">
+        <v>311</v>
+      </c>
+      <c r="D54" s="88" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="88">
+      <c r="C55" s="89">
         <v>4</v>
       </c>
-      <c r="D55" s="88" t="s">
-        <v>311</v>
+      <c r="D55" s="89" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="80" t="s">
-        <v>312</v>
-      </c>
-      <c r="D56" s="70" t="s">
-        <v>313</v>
+      <c r="C56" s="81" t="s">
+        <v>314</v>
+      </c>
+      <c r="D56" s="71" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="80" t="s">
-        <v>314</v>
-      </c>
-      <c r="D57" s="87" t="s">
-        <v>315</v>
+      <c r="C57" s="81" t="s">
+        <v>316</v>
+      </c>
+      <c r="D57" s="88" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="80" t="s">
-        <v>316</v>
-      </c>
-      <c r="D58" s="87" t="s">
-        <v>317</v>
+      <c r="C58" s="81" t="s">
+        <v>318</v>
+      </c>
+      <c r="D58" s="88" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="80" t="s">
-        <v>318</v>
-      </c>
-      <c r="D59" s="87" t="s">
-        <v>319</v>
+      <c r="C59" s="81" t="s">
+        <v>320</v>
+      </c>
+      <c r="D59" s="88" t="s">
+        <v>321</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="88">
+      <c r="C60" s="89">
         <v>5</v>
       </c>
-      <c r="D60" s="88" t="s">
-        <v>320</v>
+      <c r="D60" s="89" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="80" t="s">
-        <v>321</v>
-      </c>
-      <c r="D61" s="70" t="s">
-        <v>322</v>
+      <c r="C61" s="81" t="s">
+        <v>323</v>
+      </c>
+      <c r="D61" s="71" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="80" t="s">
-        <v>323</v>
-      </c>
-      <c r="D62" s="87" t="s">
-        <v>324</v>
+      <c r="C62" s="81" t="s">
+        <v>325</v>
+      </c>
+      <c r="D62" s="88" t="s">
+        <v>326</v>
       </c>
       <c r="F62" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="80" t="s">
-        <v>326</v>
-      </c>
-      <c r="D63" s="87" t="s">
-        <v>327</v>
+      <c r="C63" s="81" t="s">
+        <v>328</v>
+      </c>
+      <c r="D63" s="88" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="80" t="s">
-        <v>328</v>
-      </c>
-      <c r="D64" s="87" t="s">
-        <v>329</v>
+      <c r="C64" s="81" t="s">
+        <v>330</v>
+      </c>
+      <c r="D64" s="88" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="88">
+      <c r="C65" s="89">
         <v>6</v>
       </c>
-      <c r="D65" s="88" t="s">
-        <v>330</v>
+      <c r="D65" s="89" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="80" t="s">
-        <v>331</v>
-      </c>
-      <c r="D66" s="70" t="s">
-        <v>332</v>
+      <c r="C66" s="81" t="s">
+        <v>333</v>
+      </c>
+      <c r="D66" s="71" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="89" t="s">
-        <v>333</v>
-      </c>
-      <c r="D67" s="90" t="s">
-        <v>334</v>
+      <c r="C67" s="90" t="s">
+        <v>335</v>
+      </c>
+      <c r="D67" s="91" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="80" t="s">
-        <v>335</v>
-      </c>
-      <c r="D68" s="87" t="s">
-        <v>336</v>
+      <c r="C68" s="81" t="s">
+        <v>337</v>
+      </c>
+      <c r="D68" s="88" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="89" t="s">
-        <v>337</v>
-      </c>
-      <c r="D69" s="87" t="s">
-        <v>338</v>
+      <c r="C69" s="90" t="s">
+        <v>339</v>
+      </c>
+      <c r="D69" s="88" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="80" t="s">
-        <v>339</v>
-      </c>
-      <c r="D70" s="87" t="s">
-        <v>340</v>
+      <c r="C70" s="81" t="s">
+        <v>341</v>
+      </c>
+      <c r="D70" s="88" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="88">
+      <c r="C71" s="89">
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="80" t="s">
-        <v>342</v>
-      </c>
-      <c r="D72" s="70" t="s">
-        <v>343</v>
+      <c r="C72" s="81" t="s">
+        <v>344</v>
+      </c>
+      <c r="D72" s="71" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="88">
+      <c r="C73" s="89">
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="80" t="s">
-        <v>345</v>
-      </c>
-      <c r="D74" s="70" t="s">
-        <v>346</v>
+      <c r="C74" s="81" t="s">
+        <v>347</v>
+      </c>
+      <c r="D74" s="71" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="88">
+      <c r="C75" s="89">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="80" t="s">
-        <v>347</v>
-      </c>
-      <c r="D76" s="70" t="s">
-        <v>348</v>
+      <c r="C76" s="81" t="s">
+        <v>349</v>
+      </c>
+      <c r="D76" s="71" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="80" t="s">
-        <v>349</v>
-      </c>
-      <c r="D77" s="87" t="s">
-        <v>350</v>
+      <c r="C77" s="81" t="s">
+        <v>351</v>
+      </c>
+      <c r="D77" s="88" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="80" t="s">
-        <v>351</v>
-      </c>
-      <c r="D78" s="87" t="s">
-        <v>352</v>
+      <c r="C78" s="81" t="s">
+        <v>353</v>
+      </c>
+      <c r="D78" s="88" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="79">
-      <c r="C79" s="88">
+      <c r="C79" s="89">
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="80" t="s">
-        <v>354</v>
-      </c>
-      <c r="D80" s="70" t="s">
-        <v>355</v>
-      </c>
-      <c r="E80" s="74"/>
+      <c r="C80" s="81" t="s">
+        <v>356</v>
+      </c>
+      <c r="D80" s="71" t="s">
+        <v>357</v>
+      </c>
+      <c r="E80" s="75"/>
     </row>
     <row r="81">
-      <c r="C81" s="80" t="s">
-        <v>356</v>
-      </c>
-      <c r="D81" s="87" t="s">
-        <v>357</v>
+      <c r="C81" s="81" t="s">
+        <v>358</v>
+      </c>
+      <c r="D81" s="88" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="88">
+      <c r="C82" s="89">
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="80" t="s">
-        <v>359</v>
-      </c>
-      <c r="D83" s="70" t="s">
-        <v>360</v>
+      <c r="C83" s="81" t="s">
+        <v>361</v>
+      </c>
+      <c r="D83" s="71" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="84">
-      <c r="C84" s="80" t="s">
-        <v>361</v>
-      </c>
-      <c r="D84" s="70" t="s">
-        <v>362</v>
+      <c r="C84" s="81" t="s">
+        <v>363</v>
+      </c>
+      <c r="D84" s="71" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAJ : enleve animation flou de changement dans finally
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="366">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -217,23 +217,14 @@
   </si>
   <si>
     <t xml:space="preserve">Teste manuel déplacement : 
-# Bloquer les fonctions move quand detecté + recule 20 pas par ex
-- Machine a état : simple et efficace (repars à 0 ? + ajouter compteur )
-    # Retourner le nb de pas effectuer dans les move()
-    # Calcul distance max : bas/gauche-haut/droite
-    # Menu parametrage positions manuel
-        # Voir dessin
-# Compter nb step marche plus Raspberry voir commit
-- Machine a etat OK local pas sur Raspberry : init ok mais goToPos KO
-- Calcul pas de déplacement pour aller àla pos voulu
-    - OK ça marche? Mais pas de retour API dcp attent dans le vide
-- Appeler GoToPos 2 fois : aller de a à b avec action sur CD, PUIS aller de b à c avec action CD
--Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
-   - Menu parametre être plus précis + save pos haut et pos bas
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit 9e907e5</t>
+# Detection des capteurs avec retour marge OK
+# Fonction moveTo/origin/end OK
+# Init machine a etats puis attente actions OK
+# Calibrer les positions OK
+# playCd -&gt; Bouge au CD puis reviens origin OK
+- Pb : timeout de 10s, si mouvement plus long la connexion coupe
+    https://claude.ai/chat/1f9255f3-cb82-455e-8c4a-e6fc560f6c47
+- Tester toute la machine a etat, sur la durée</t>
   </si>
   <si>
     <t xml:space="preserve">Prévoir tiges? pour fixer armature à planche, avec une certaine distance</t>
@@ -245,6 +236,10 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t xml:space="preserve">-Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
+   - Menu calibrage !</t>
+  </si>
+  <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
   </si>
   <si>
@@ -260,6 +255,9 @@
     <t>Font</t>
   </si>
   <si>
+    <t xml:space="preserve">- Logique de placement des CDs sur le lecteur,     Appeler GoToPos 2 fois : aller de a à b avec action sur CD, PUIS aller de b à c avec action CD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Calculer nb step pour chaque positions</t>
   </si>
   <si>
@@ -281,28 +279,28 @@
     <t xml:space="preserve">Lecteur CD</t>
   </si>
   <si>
+    <t>AliExpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Déplacement elec aimant</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nouveau lecteur à trouver</t>
   </si>
   <si>
     <t xml:space="preserve">Trouver ouverture par le dessus, avec une tige de lecteur assez grande</t>
   </si>
   <si>
-    <t>AliExpress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Déplacement elec aimant</t>
+    <t xml:space="preserve">Créer image déjà prête, sans imager toute la carte SD. MàJ doc raspberry/0_software/0_initialisation_raspberry.md</t>
   </si>
   <si>
     <t xml:space="preserve">Avec 4 fixation comme celui actuel</t>
   </si>
   <si>
-    <t xml:space="preserve">Créer image déjà prête, sans imager toute la carte SD. MàJ doc raspberry/0_software/0_initialisation_raspberry.md</t>
+    <t xml:space="preserve">"... the image in XXX filder ..."</t>
   </si>
   <si>
     <t xml:space="preserve">Tester lecture CD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"... the image in XXX filder ..."</t>
   </si>
   <si>
     <t xml:space="preserve">Changer le support</t>
@@ -1688,7 +1686,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="99">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1705,10 +1703,14 @@
     <xf fontId="0" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="6" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="6" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf fontId="7" fillId="7" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
@@ -1750,6 +1752,17 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1759,6 +1772,8 @@
     </xf>
     <xf fontId="8" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="8" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="6" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="9" fillId="7" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1941,8 +1956,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" displayName="Tableau6" ref="B9:D61">
-  <autoFilter ref="B9:D61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" displayName="Tableau6" ref="B9:D62">
+  <autoFilter ref="B9:D62"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Tâches"/>
     <tableColumn id="2" name="Détail"/>
@@ -2726,8 +2741,8 @@
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="14">
-        <f>SUM(D14:D21)/8</f>
-        <v>0.80625000000000002</v>
+        <f>SUM(D14:D22)/9</f>
+        <v>0.75</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>22</v>
@@ -3026,19 +3041,17 @@
       <c r="Z20" s="1"/>
       <c r="AA20" s="1"/>
     </row>
-    <row r="21" ht="270.75">
+    <row r="21" ht="242.25">
       <c r="A21" s="1"/>
       <c r="B21" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="35"/>
+      <c r="D21" s="36">
+        <v>0.75</v>
+      </c>
+      <c r="F21" t="s">
         <v>64</v>
-      </c>
-      <c r="D21" s="32">
-        <v>0.45000000000000001</v>
-      </c>
-      <c r="F21" t="s">
-        <v>65</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>23</v>
@@ -3046,7 +3059,7 @@
       <c r="H21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M21" s="33" t="s">
         <v>62</v>
@@ -3060,14 +3073,20 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="X21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
     <row r="22" ht="16.5">
       <c r="A22" s="1"/>
-      <c r="D22" s="32"/>
+      <c r="B22" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" s="38"/>
+      <c r="D22" s="39">
+        <v>0</v>
+      </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
@@ -3104,13 +3123,16 @@
     </row>
     <row r="23" ht="16.5">
       <c r="A23" s="1"/>
+      <c r="B23" s="40" t="s">
+        <v>73</v>
+      </c>
       <c r="D23" s="32"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M23" s="33" t="s">
         <v>62</v>
@@ -3119,35 +3141,37 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
-      <c r="F24" s="37" t="s">
-        <v>76</v>
+      <c r="B24"/>
+      <c r="D24" s="32"/>
+      <c r="F24" s="42" t="s">
+        <v>77</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="38"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="40"/>
+      <c r="H24" s="43"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="45"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3162,14 +3186,6 @@
     </row>
     <row r="25" ht="16.5">
       <c r="A25" s="1"/>
-      <c r="B25" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="41">
-        <f>SUM(D26:D31)/5</f>
-        <v>0</v>
-      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -3189,13 +3205,12 @@
     </row>
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
-      <c r="B26" t="s">
+      <c r="B26" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="C26" t="s">
-        <v>81</v>
-      </c>
-      <c r="D26" s="32">
+      <c r="C26" s="47"/>
+      <c r="D26" s="48">
+        <f>SUM(D27:D32)/5</f>
         <v>0</v>
       </c>
       <c r="F26" s="1"/>
@@ -3208,10 +3223,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="P26" s="22" t="s">
         <v>82</v>
-      </c>
-      <c r="P26" s="22" t="s">
-        <v>83</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3223,6 +3238,9 @@
     </row>
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
+      <c r="B27" t="s">
+        <v>83</v>
+      </c>
       <c r="C27" t="s">
         <v>84</v>
       </c>
@@ -3245,7 +3263,7 @@
     </row>
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>86</v>
       </c>
       <c r="D28" s="32">
@@ -3272,9 +3290,6 @@
       <c r="B29" t="s">
         <v>88</v>
       </c>
-      <c r="C29" t="s">
-        <v>89</v>
-      </c>
       <c r="D29" s="32">
         <v>0</v>
       </c>
@@ -3292,11 +3307,11 @@
     </row>
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
-      <c r="B30" s="4" t="s">
+      <c r="B30" t="s">
+        <v>89</v>
+      </c>
+      <c r="C30" t="s">
         <v>90</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="D30" s="32">
         <v>0</v>
@@ -3317,6 +3332,9 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>92</v>
       </c>
       <c r="D31" s="32">
@@ -3335,10 +3353,14 @@
     </row>
     <row r="32" ht="28.5">
       <c r="A32" s="1"/>
-      <c r="B32" s="4"/>
-      <c r="D32" s="32"/>
+      <c r="B32" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32" s="32">
+        <v>0</v>
+      </c>
       <c r="L32" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3348,7 +3370,7 @@
       <c r="B33" s="4"/>
       <c r="D33" s="32"/>
       <c r="L33" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3361,6 +3383,8 @@
     </row>
     <row r="34" ht="16.5">
       <c r="A34" s="1"/>
+      <c r="B34" s="4"/>
+      <c r="D34" s="32"/>
       <c r="L34" s="19"/>
       <c r="M34" s="19"/>
       <c r="N34" s="1"/>
@@ -3374,14 +3398,6 @@
     </row>
     <row r="35" ht="16.5">
       <c r="A35" s="1"/>
-      <c r="B35" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="C35" s="13"/>
-      <c r="D35" s="41">
-        <f>SUM(D36:D39)/4</f>
-        <v>0</v>
-      </c>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
@@ -3395,13 +3411,12 @@
     </row>
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="49" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D36" s="32">
+      <c r="C36" s="47"/>
+      <c r="D36" s="48">
+        <f>SUM(D37:D40)/4</f>
         <v>0</v>
       </c>
       <c r="L36" s="1"/>
@@ -3418,10 +3433,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>98</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>99</v>
       </c>
       <c r="D37" s="32">
         <v>0</v>
@@ -3440,10 +3455,10 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>101</v>
       </c>
       <c r="D38" s="32">
         <v>0</v>
@@ -3462,29 +3477,33 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="C39" s="26" t="s">
-        <v>103</v>
       </c>
       <c r="D39" s="32">
         <v>0</v>
       </c>
     </row>
-    <row r="40" ht="16.5">
+    <row r="40" ht="28.5">
       <c r="A40" s="1"/>
+      <c r="B40" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="D40" s="32">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" ht="16.5">
       <c r="A41" s="1"/>
-      <c r="B41" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
     </row>
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="5" t="s">
         <v>105</v>
       </c>
       <c r="C42" s="4"/>
@@ -3492,33 +3511,35 @@
     </row>
     <row r="43" ht="16.5">
       <c r="A43" s="1"/>
+      <c r="B43" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
     </row>
     <row r="44" ht="16.5">
       <c r="A44" s="1"/>
-      <c r="B44" t="s">
-        <v>106</v>
-      </c>
     </row>
     <row r="45" ht="16.5">
       <c r="A45" s="1"/>
+      <c r="B45" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="46" ht="14.25">
       <c r="A46" s="1"/>
     </row>
     <row r="47" ht="14.25">
       <c r="A47" s="1"/>
-      <c r="B47" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="48" ht="14.25">
       <c r="A48" s="1"/>
+      <c r="B48" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="49" ht="14.25">
       <c r="A49" s="1"/>
-      <c r="B49" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
@@ -3528,15 +3549,15 @@
     </row>
     <row r="51" ht="14.25">
       <c r="A51" s="1"/>
+      <c r="B51" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="52" ht="16.5">
       <c r="A52" s="1"/>
     </row>
     <row r="53" ht="16.5">
       <c r="A53" s="1"/>
-      <c r="B53" t="s">
-        <v>110</v>
-      </c>
     </row>
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
@@ -3556,6 +3577,9 @@
     </row>
     <row r="55" ht="16.5">
       <c r="A55" s="1"/>
+      <c r="B55" t="s">
+        <v>112</v>
+      </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
@@ -3569,9 +3593,6 @@
     </row>
     <row r="56" ht="16.5">
       <c r="A56" s="1"/>
-      <c r="B56" t="s">
-        <v>112</v>
-      </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -3585,6 +3606,9 @@
     </row>
     <row r="57" ht="16.5">
       <c r="A57" s="1"/>
+      <c r="B57" t="s">
+        <v>113</v>
+      </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="2"/>
@@ -3609,13 +3633,8 @@
       <c r="N58" s="2"/>
       <c r="O58" s="1"/>
     </row>
-    <row r="68" ht="14.25">
-      <c r="B68" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
     <row r="69" ht="14.25">
-      <c r="B69" t="s">
+      <c r="B69" s="5" t="s">
         <v>114</v>
       </c>
     </row>
@@ -3658,8 +3677,13 @@
       <c r="B77" t="s">
         <v>122</v>
       </c>
-      <c r="C77" t="s">
-        <v>67</v>
+    </row>
+    <row r="78" ht="14.25">
+      <c r="B78" t="s">
+        <v>123</v>
+      </c>
+      <c r="C78" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3689,280 +3713,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="43" t="s">
-        <v>123</v>
-      </c>
-      <c r="G2" s="44" t="s">
+      <c r="F2" s="50" t="s">
         <v>124</v>
       </c>
+      <c r="G2" s="51" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="3">
-      <c r="F3" s="45" t="s">
-        <v>125</v>
-      </c>
-      <c r="G3" s="46" t="s">
+      <c r="F3" s="52" t="s">
         <v>126</v>
       </c>
+      <c r="G3" s="53" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="4">
-      <c r="F4" s="47" t="s">
-        <v>127</v>
-      </c>
-      <c r="G4" s="48" t="s">
+      <c r="F4" s="54" t="s">
         <v>128</v>
       </c>
+      <c r="G4" s="55" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="5" ht="15">
-      <c r="F5" s="49" t="s">
-        <v>129</v>
-      </c>
-      <c r="G5" s="50" t="s">
+      <c r="F5" s="56" t="s">
         <v>130</v>
       </c>
+      <c r="G5" s="57" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="6" ht="15">
-      <c r="F6" s="51"/>
-      <c r="G6" s="52" t="s">
-        <v>131</v>
+      <c r="F6" s="58"/>
+      <c r="G6" s="59" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="F7" s="51"/>
-      <c r="G7" s="52" t="s">
-        <v>132</v>
+      <c r="F7" s="58"/>
+      <c r="G7" s="59" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="F8" s="51"/>
-      <c r="G8" s="52" t="s">
-        <v>133</v>
+      <c r="F8" s="58"/>
+      <c r="G8" s="59" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F9" s="51"/>
-      <c r="G9" s="52" t="s">
         <v>135</v>
+      </c>
+      <c r="F9" s="58"/>
+      <c r="G9" s="59" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
-        <v>136</v>
-      </c>
-      <c r="C10" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="51"/>
-      <c r="G10" s="52" t="s">
+      <c r="C10" s="60" t="s">
         <v>138</v>
       </c>
+      <c r="F10" s="58"/>
+      <c r="G10" s="59" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="11" ht="15">
-      <c r="C11" s="54" t="s">
-        <v>139</v>
-      </c>
-      <c r="F11" s="51"/>
-      <c r="G11" s="52" t="s">
+      <c r="C11" s="61" t="s">
         <v>140</v>
       </c>
+      <c r="F11" s="58"/>
+      <c r="G11" s="59" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="12" ht="15">
-      <c r="C12" s="53" t="s">
-        <v>141</v>
-      </c>
-      <c r="F12" s="45"/>
-      <c r="G12" s="55" t="s">
+      <c r="C12" s="60" t="s">
         <v>142</v>
       </c>
+      <c r="F12" s="52"/>
+      <c r="G12" s="62" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="13" ht="15">
-      <c r="C13" s="54" t="s">
-        <v>143</v>
-      </c>
-      <c r="F13" s="47" t="s">
+      <c r="C13" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="G13" s="56" t="s">
+      <c r="F13" s="54" t="s">
         <v>145</v>
       </c>
+      <c r="G13" s="63" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="14" ht="15">
-      <c r="C14" s="53" t="s">
-        <v>146</v>
-      </c>
-      <c r="F14" s="57" t="s">
+      <c r="C14" s="60" t="s">
         <v>147</v>
       </c>
-      <c r="G14" s="58" t="s">
+      <c r="F14" s="64" t="s">
         <v>148</v>
       </c>
+      <c r="G14" s="65" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="15">
-      <c r="C15" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="F15" s="59" t="s">
+      <c r="C15" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="G15" s="60" t="s">
+      <c r="F15" s="66" t="s">
         <v>151</v>
       </c>
+      <c r="G15" s="67" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="16">
-      <c r="C16" s="54" t="s">
-        <v>152</v>
-      </c>
-      <c r="F16" s="61" t="s">
+      <c r="C16" s="61" t="s">
         <v>153</v>
       </c>
-      <c r="G16" s="62" t="s">
+      <c r="F16" s="68" t="s">
         <v>154</v>
       </c>
+      <c r="G16" s="69" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="17">
-      <c r="C17" s="53" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" s="61"/>
-      <c r="G17" s="62" t="s">
+      <c r="C17" s="60" t="s">
         <v>156</v>
       </c>
+      <c r="F17" s="68"/>
+      <c r="G17" s="69" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="18">
-      <c r="C18" s="54" t="s">
-        <v>157</v>
-      </c>
-      <c r="F18" s="61"/>
-      <c r="G18" s="62" t="s">
+      <c r="C18" s="61" t="s">
         <v>158</v>
       </c>
+      <c r="F18" s="68"/>
+      <c r="G18" s="69" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="19">
-      <c r="C19" s="54" t="s">
-        <v>159</v>
-      </c>
-      <c r="F19" s="61"/>
-      <c r="G19" s="62" t="s">
+      <c r="C19" s="61" t="s">
         <v>160</v>
       </c>
+      <c r="F19" s="68"/>
+      <c r="G19" s="69" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="20">
-      <c r="C20" s="54" t="s">
-        <v>161</v>
-      </c>
-      <c r="F20" s="61"/>
-      <c r="G20" s="62" t="s">
+      <c r="C20" s="61" t="s">
         <v>162</v>
       </c>
+      <c r="F20" s="68"/>
+      <c r="G20" s="69" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="21">
-      <c r="C21" s="54" t="s">
-        <v>163</v>
-      </c>
-      <c r="F21" s="61"/>
-      <c r="G21" s="62" t="s">
+      <c r="C21" s="61" t="s">
         <v>164</v>
       </c>
+      <c r="F21" s="68"/>
+      <c r="G21" s="69" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="22">
-      <c r="C22" s="53" t="s">
-        <v>165</v>
-      </c>
-      <c r="F22" s="61"/>
-      <c r="G22" s="62" t="s">
+      <c r="C22" s="60" t="s">
         <v>166</v>
       </c>
+      <c r="F22" s="68"/>
+      <c r="G22" s="69" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="23">
-      <c r="C23" s="54" t="s">
-        <v>167</v>
-      </c>
-      <c r="F23" s="61"/>
-      <c r="G23" s="62" t="s">
+      <c r="C23" s="61" t="s">
         <v>168</v>
       </c>
+      <c r="F23" s="68"/>
+      <c r="G23" s="69" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="24">
-      <c r="C24" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="F24" s="61"/>
-      <c r="G24" s="62" t="s">
+      <c r="C24" s="60" t="s">
         <v>170</v>
       </c>
+      <c r="F24" s="68"/>
+      <c r="G24" s="69" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="25">
-      <c r="C25" s="54" t="s">
-        <v>171</v>
-      </c>
-      <c r="F25" s="61"/>
-      <c r="G25" s="62" t="s">
+      <c r="C25" s="61" t="s">
         <v>172</v>
       </c>
+      <c r="F25" s="68"/>
+      <c r="G25" s="69" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="26">
-      <c r="F26" s="61"/>
-      <c r="G26" s="62" t="s">
-        <v>173</v>
+      <c r="F26" s="68"/>
+      <c r="G26" s="69" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="61"/>
-      <c r="G27" s="62"/>
+      <c r="F27" s="68"/>
+      <c r="G27" s="69"/>
     </row>
     <row r="28">
-      <c r="F28" s="61"/>
-      <c r="G28" s="62" t="s">
-        <v>174</v>
+      <c r="F28" s="68"/>
+      <c r="G28" s="69" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="61"/>
-      <c r="G29" s="62" t="s">
-        <v>175</v>
+      <c r="F29" s="68"/>
+      <c r="G29" s="69" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="63"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="62" t="s">
-        <v>176</v>
+      <c r="C30" s="70"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="69" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="61"/>
-      <c r="G31" s="64" t="s">
-        <v>177</v>
+      <c r="F31" s="68"/>
+      <c r="G31" s="71" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="57" t="s">
-        <v>178</v>
-      </c>
-      <c r="G32" s="65" t="s">
+      <c r="F32" s="64" t="s">
         <v>179</v>
       </c>
+      <c r="G32" s="72" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="33">
-      <c r="C33" s="54"/>
+      <c r="C33" s="61"/>
     </row>
     <row r="34">
-      <c r="C34" s="54"/>
+      <c r="C34" s="61"/>
     </row>
     <row r="36">
-      <c r="C36" s="63"/>
+      <c r="C36" s="70"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="54"/>
+      <c r="C39" s="61"/>
     </row>
     <row r="40">
-      <c r="C40" s="54"/>
+      <c r="C40" s="61"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -3990,367 +4014,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B5" t="s">
-        <v>181</v>
-      </c>
-      <c r="D5" s="66" t="s">
         <v>182</v>
       </c>
+      <c r="D5" s="73" t="s">
+        <v>183</v>
+      </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="67" t="s">
         <v>190</v>
       </c>
+      <c r="D6" s="74" t="s">
+        <v>191</v>
+      </c>
       <c r="E6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H6" s="68" t="s">
         <v>194</v>
       </c>
+      <c r="H6" s="75" t="s">
+        <v>195</v>
+      </c>
       <c r="I6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B7" t="s">
-        <v>189</v>
-      </c>
-      <c r="D7" s="69" t="s">
-        <v>199</v>
+        <v>190</v>
+      </c>
+      <c r="D7" s="76" t="s">
+        <v>200</v>
       </c>
       <c r="F7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G7" t="s">
-        <v>201</v>
-      </c>
-      <c r="H7" s="68" t="s">
         <v>202</v>
       </c>
+      <c r="H7" s="75" t="s">
+        <v>203</v>
+      </c>
       <c r="K7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="67" t="s">
-        <v>204</v>
-      </c>
-      <c r="G8" s="70" t="s">
+      <c r="D8" s="74" t="s">
         <v>205</v>
       </c>
-      <c r="H8" s="68" t="s">
+      <c r="G8" s="77" t="s">
         <v>206</v>
+      </c>
+      <c r="H8" s="75" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B9" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="69" t="s">
         <v>209</v>
       </c>
-      <c r="H9" s="68" t="s">
+      <c r="D9" s="76" t="s">
         <v>210</v>
+      </c>
+      <c r="H9" s="75" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B10" t="s">
-        <v>212</v>
-      </c>
-      <c r="D10" s="67"/>
+        <v>213</v>
+      </c>
+      <c r="D10" s="74"/>
       <c r="G10" t="s">
-        <v>213</v>
-      </c>
-      <c r="H10" s="68" t="s">
         <v>214</v>
+      </c>
+      <c r="H10" s="75" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B11" t="s">
-        <v>216</v>
-      </c>
-      <c r="D11" s="69" t="s">
         <v>217</v>
       </c>
-      <c r="G11" s="70" t="s">
+      <c r="D11" s="76" t="s">
         <v>218</v>
       </c>
-      <c r="H11" s="68" t="s">
+      <c r="G11" s="77" t="s">
         <v>219</v>
+      </c>
+      <c r="H11" s="75" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B12" t="s">
-        <v>221</v>
-      </c>
-      <c r="D12" s="67" t="s">
         <v>222</v>
       </c>
-      <c r="G12" s="70" t="s">
+      <c r="D12" s="74" t="s">
         <v>223</v>
       </c>
-      <c r="H12" s="68" t="s">
+      <c r="G12" s="77" t="s">
         <v>224</v>
+      </c>
+      <c r="H12" s="75" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B13" t="s">
-        <v>226</v>
-      </c>
-      <c r="D13" s="69" t="s">
         <v>227</v>
       </c>
-      <c r="G13" s="70" t="s">
+      <c r="D13" s="76" t="s">
         <v>228</v>
       </c>
+      <c r="G13" s="77" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="14">
-      <c r="D14" s="67" t="s">
-        <v>229</v>
+      <c r="D14" s="74" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B15" t="s">
-        <v>231</v>
-      </c>
-      <c r="D15" s="69"/>
+        <v>232</v>
+      </c>
+      <c r="D15" s="76"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B16" t="s">
-        <v>233</v>
-      </c>
-      <c r="D16" s="67"/>
+        <v>234</v>
+      </c>
+      <c r="D16" s="74"/>
       <c r="G16" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="69"/>
-      <c r="G17" s="70" t="s">
-        <v>235</v>
+      <c r="D17" s="76"/>
+      <c r="G17" s="77" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>236</v>
-      </c>
-      <c r="D18" s="67"/>
-      <c r="G18" s="71" t="s">
         <v>237</v>
       </c>
+      <c r="D18" s="74"/>
+      <c r="G18" s="78" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="19">
-      <c r="D19" s="69" t="s">
-        <v>238</v>
+      <c r="D19" s="76" t="s">
+        <v>239</v>
       </c>
       <c r="E19" t="s">
-        <v>239</v>
-      </c>
-      <c r="G19" s="71" t="s">
         <v>240</v>
       </c>
+      <c r="G19" s="78" t="s">
+        <v>241</v>
+      </c>
       <c r="H19" t="s">
+        <v>242</v>
+      </c>
+      <c r="I19" t="s">
+        <v>243</v>
+      </c>
+      <c r="J19" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="74"/>
+      <c r="G20" s="78" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="74"/>
+      <c r="G22" s="78" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="77"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="74"/>
+      <c r="G24" s="77" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="78" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="74"/>
+      <c r="G26" s="78" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="78" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="74"/>
+      <c r="G28" s="78" t="s">
         <v>241</v>
       </c>
-      <c r="I19" t="s">
-        <v>242</v>
-      </c>
-      <c r="J19" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="67"/>
-      <c r="G20" s="71" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="67"/>
-      <c r="G22" s="71" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="G23" s="70"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="67"/>
-      <c r="G24" s="70" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" s="71" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" s="67"/>
-      <c r="G26" s="71" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="71" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="67"/>
-      <c r="G28" s="71" t="s">
-        <v>240</v>
-      </c>
     </row>
     <row r="35">
-      <c r="D35" s="72" t="s">
-        <v>248</v>
+      <c r="D35" s="79" t="s">
+        <v>249</v>
       </c>
       <c r="E35" t="s">
-        <v>249</v>
-      </c>
-      <c r="F35" s="73" t="s">
         <v>250</v>
       </c>
+      <c r="F35" s="80" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="36">
-      <c r="D36" s="74" t="s">
-        <v>251</v>
+      <c r="D36" s="81" t="s">
+        <v>252</v>
       </c>
       <c r="E36" t="s">
-        <v>252</v>
-      </c>
-      <c r="F36" s="74" t="s">
         <v>253</v>
       </c>
+      <c r="F36" s="81" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="37">
-      <c r="D37" s="73" t="s">
-        <v>254</v>
+      <c r="D37" s="80" t="s">
+        <v>255</v>
       </c>
       <c r="E37" t="s">
-        <v>255</v>
-      </c>
-      <c r="F37" s="73" t="s">
         <v>256</v>
       </c>
+      <c r="F37" s="80" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="38">
-      <c r="D38" s="74" t="s">
-        <v>257</v>
+      <c r="D38" s="81" t="s">
+        <v>258</v>
       </c>
       <c r="E38" t="s">
-        <v>258</v>
-      </c>
-      <c r="F38" s="74" t="s">
         <v>259</v>
       </c>
+      <c r="F38" s="81" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="39">
-      <c r="D39" s="73" t="s">
-        <v>260</v>
+      <c r="D39" s="80" t="s">
+        <v>261</v>
       </c>
       <c r="E39" t="s">
-        <v>261</v>
-      </c>
-      <c r="F39" s="73" t="s">
         <v>262</v>
+      </c>
+      <c r="F39" s="80" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>252</v>
-      </c>
-      <c r="F40" s="74" t="s">
-        <v>263</v>
+        <v>253</v>
+      </c>
+      <c r="F40" s="81" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>255</v>
-      </c>
-      <c r="F41" s="73" t="s">
-        <v>264</v>
+        <v>256</v>
+      </c>
+      <c r="F41" s="80" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -4381,564 +4405,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="75" t="s">
-        <v>267</v>
+      <c r="D4" s="82" t="s">
+        <v>268</v>
       </c>
       <c r="E4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
+        <v>270</v>
+      </c>
+      <c r="E5" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="78" t="s">
+        <v>271</v>
+      </c>
+      <c r="E6" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="83" t="s">
+        <v>272</v>
+      </c>
+      <c r="E7" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="78" t="s">
+        <v>273</v>
+      </c>
+      <c r="E8" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="78"/>
+      <c r="E9" s="82"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="75" t="s">
+        <v>274</v>
+      </c>
+      <c r="E10" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="78" t="s">
+        <v>275</v>
+      </c>
+      <c r="E11" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="78" t="s">
+        <v>276</v>
+      </c>
+      <c r="E12" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="78" t="s">
+        <v>277</v>
+      </c>
+      <c r="E13" s="82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="75" t="s">
+        <v>278</v>
+      </c>
+      <c r="E15" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="84" t="s">
+        <v>279</v>
+      </c>
+      <c r="E16" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="85" t="s">
+        <v>280</v>
+      </c>
+      <c r="E17" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="85" t="s">
+        <v>281</v>
+      </c>
+      <c r="E18" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="78"/>
+      <c r="E19" s="78"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="75" t="s">
+        <v>282</v>
+      </c>
+      <c r="E20" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" s="75" t="s">
+        <v>283</v>
+      </c>
+      <c r="E21" s="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="78"/>
+      <c r="E22" s="78"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="86"/>
+      <c r="E23" s="78"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="78"/>
+      <c r="E24" s="78"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="78"/>
+      <c r="E25" s="78"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="78"/>
+      <c r="E27" s="78"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="78"/>
+      <c r="E29" s="78"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="78"/>
+      <c r="E30" s="78"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="87"/>
+      <c r="C39" s="88" t="s">
+        <v>284</v>
+      </c>
+      <c r="D39" s="88" t="s">
+        <v>285</v>
+      </c>
+      <c r="E39" t="s">
         <v>269</v>
-      </c>
-      <c r="E5" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="D6" s="71" t="s">
-        <v>270</v>
-      </c>
-      <c r="E6" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" s="76" t="s">
-        <v>271</v>
-      </c>
-      <c r="E7" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="71" t="s">
-        <v>272</v>
-      </c>
-      <c r="E8" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="71"/>
-      <c r="E9" s="75"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="68" t="s">
-        <v>273</v>
-      </c>
-      <c r="E10" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" s="71" t="s">
-        <v>274</v>
-      </c>
-      <c r="E11" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="71" t="s">
-        <v>275</v>
-      </c>
-      <c r="E12" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="71" t="s">
-        <v>276</v>
-      </c>
-      <c r="E13" s="75">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="71"/>
-      <c r="E14" s="71"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="68" t="s">
-        <v>277</v>
-      </c>
-      <c r="E15" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="77" t="s">
-        <v>278</v>
-      </c>
-      <c r="E16" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="78" t="s">
-        <v>279</v>
-      </c>
-      <c r="E17" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" s="78" t="s">
-        <v>280</v>
-      </c>
-      <c r="E18" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="71"/>
-      <c r="E19" s="71"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="68" t="s">
-        <v>281</v>
-      </c>
-      <c r="E20" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" s="68" t="s">
-        <v>282</v>
-      </c>
-      <c r="E21" s="75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="79"/>
-      <c r="E23" s="71"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="71"/>
-      <c r="E24" s="71"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="71"/>
-      <c r="E25" s="71"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="71"/>
-      <c r="E26" s="71"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="71"/>
-      <c r="E27" s="71"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="71"/>
-      <c r="E28" s="71"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="71"/>
-      <c r="E29" s="71"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="80"/>
-      <c r="C39" s="81" t="s">
-        <v>283</v>
-      </c>
-      <c r="D39" s="81" t="s">
-        <v>284</v>
-      </c>
-      <c r="E39" t="s">
-        <v>268</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="82">
+      <c r="C40" s="89">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="E40" s="75"/>
+        <v>286</v>
+      </c>
+      <c r="E40" s="82"/>
     </row>
     <row r="41">
-      <c r="C41" s="75" t="s">
-        <v>286</v>
-      </c>
-      <c r="D41" s="71" t="s">
+      <c r="C41" s="82" t="s">
         <v>287</v>
       </c>
-      <c r="E41" s="75"/>
+      <c r="D41" s="78" t="s">
+        <v>288</v>
+      </c>
+      <c r="E41" s="82"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="75" t="s">
-        <v>288</v>
-      </c>
-      <c r="D42" s="71" t="s">
+      <c r="C42" s="82" t="s">
         <v>289</v>
       </c>
+      <c r="D42" s="78" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="43">
-      <c r="C43" s="75" t="s">
-        <v>290</v>
-      </c>
-      <c r="D43" s="71" t="s">
+      <c r="C43" s="82" t="s">
         <v>291</v>
       </c>
+      <c r="D43" s="78" t="s">
+        <v>292</v>
+      </c>
     </row>
     <row r="44">
-      <c r="C44" s="83" t="s">
-        <v>292</v>
-      </c>
-      <c r="D44" s="76" t="s">
+      <c r="C44" s="90" t="s">
         <v>293</v>
       </c>
-      <c r="E44" s="84"/>
-      <c r="F44" s="84"/>
+      <c r="D44" s="83" t="s">
+        <v>294</v>
+      </c>
+      <c r="E44" s="91"/>
+      <c r="F44" s="91"/>
     </row>
     <row r="45">
-      <c r="C45" s="81" t="s">
-        <v>294</v>
-      </c>
-      <c r="D45" s="71" t="s">
+      <c r="C45" s="88" t="s">
         <v>295</v>
       </c>
-      <c r="E45" s="75"/>
+      <c r="D45" s="78" t="s">
+        <v>296</v>
+      </c>
+      <c r="E45" s="82"/>
     </row>
     <row r="46">
-      <c r="C46" s="81" t="s">
-        <v>296</v>
-      </c>
-      <c r="D46" s="71" t="s">
+      <c r="C46" s="88" t="s">
         <v>297</v>
       </c>
-      <c r="E46" s="75"/>
+      <c r="D46" s="78" t="s">
+        <v>298</v>
+      </c>
+      <c r="E46" s="82"/>
     </row>
     <row r="47">
-      <c r="C47" s="85">
+      <c r="C47" s="92">
         <v>2</v>
       </c>
-      <c r="D47" s="86" t="s">
-        <v>298</v>
-      </c>
-      <c r="E47" s="75"/>
+      <c r="D47" s="93" t="s">
+        <v>299</v>
+      </c>
+      <c r="E47" s="82"/>
     </row>
     <row r="48">
-      <c r="C48" s="83" t="s">
-        <v>299</v>
-      </c>
-      <c r="D48" s="76" t="s">
+      <c r="C48" s="90" t="s">
         <v>300</v>
       </c>
-      <c r="E48" s="75"/>
+      <c r="D48" s="83" t="s">
+        <v>301</v>
+      </c>
+      <c r="E48" s="82"/>
     </row>
     <row r="49">
-      <c r="C49" s="82">
+      <c r="C49" s="89">
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="E49" s="75"/>
+        <v>302</v>
+      </c>
+      <c r="E49" s="82"/>
     </row>
     <row r="50">
-      <c r="C50" s="83" t="s">
-        <v>302</v>
-      </c>
-      <c r="D50" s="76" t="s">
+      <c r="C50" s="90" t="s">
         <v>303</v>
       </c>
-      <c r="F50" s="87" t="s">
+      <c r="D50" s="83" t="s">
         <v>304</v>
       </c>
+      <c r="F50" s="94" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="51">
-      <c r="C51" s="83" t="s">
-        <v>305</v>
-      </c>
-      <c r="D51" s="88" t="s">
+      <c r="C51" s="90" t="s">
         <v>306</v>
       </c>
+      <c r="D51" s="95" t="s">
+        <v>307</v>
+      </c>
     </row>
     <row r="52">
-      <c r="C52" s="83" t="s">
-        <v>307</v>
-      </c>
-      <c r="D52" s="88" t="s">
+      <c r="C52" s="90" t="s">
         <v>308</v>
       </c>
+      <c r="D52" s="95" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="53">
-      <c r="C53" s="83" t="s">
-        <v>309</v>
-      </c>
-      <c r="D53" s="88" t="s">
+      <c r="C53" s="90" t="s">
         <v>310</v>
       </c>
+      <c r="D53" s="95" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="54">
-      <c r="C54" s="83" t="s">
-        <v>311</v>
-      </c>
-      <c r="D54" s="88" t="s">
+      <c r="C54" s="90" t="s">
         <v>312</v>
       </c>
+      <c r="D54" s="95" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="55">
-      <c r="C55" s="89">
+      <c r="C55" s="96">
         <v>4</v>
       </c>
-      <c r="D55" s="89" t="s">
-        <v>313</v>
+      <c r="D55" s="96" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="81" t="s">
-        <v>314</v>
-      </c>
-      <c r="D56" s="71" t="s">
+      <c r="C56" s="88" t="s">
         <v>315</v>
       </c>
+      <c r="D56" s="78" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="57">
-      <c r="C57" s="81" t="s">
-        <v>316</v>
-      </c>
-      <c r="D57" s="88" t="s">
+      <c r="C57" s="88" t="s">
         <v>317</v>
       </c>
+      <c r="D57" s="95" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="58">
-      <c r="C58" s="81" t="s">
-        <v>318</v>
-      </c>
-      <c r="D58" s="88" t="s">
+      <c r="C58" s="88" t="s">
         <v>319</v>
       </c>
+      <c r="D58" s="95" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="59">
-      <c r="C59" s="81" t="s">
-        <v>320</v>
-      </c>
-      <c r="D59" s="88" t="s">
+      <c r="C59" s="88" t="s">
         <v>321</v>
+      </c>
+      <c r="D59" s="95" t="s">
+        <v>322</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="89">
+      <c r="C60" s="96">
         <v>5</v>
       </c>
-      <c r="D60" s="89" t="s">
-        <v>322</v>
+      <c r="D60" s="96" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="81" t="s">
-        <v>323</v>
-      </c>
-      <c r="D61" s="71" t="s">
+      <c r="C61" s="88" t="s">
         <v>324</v>
       </c>
+      <c r="D61" s="78" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="62">
-      <c r="C62" s="81" t="s">
-        <v>325</v>
-      </c>
-      <c r="D62" s="88" t="s">
+      <c r="C62" s="88" t="s">
         <v>326</v>
       </c>
+      <c r="D62" s="95" t="s">
+        <v>327</v>
+      </c>
       <c r="F62" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="81" t="s">
-        <v>328</v>
-      </c>
-      <c r="D63" s="88" t="s">
+      <c r="C63" s="88" t="s">
         <v>329</v>
       </c>
+      <c r="D63" s="95" t="s">
+        <v>330</v>
+      </c>
     </row>
     <row r="64">
-      <c r="C64" s="81" t="s">
-        <v>330</v>
-      </c>
-      <c r="D64" s="88" t="s">
+      <c r="C64" s="88" t="s">
         <v>331</v>
       </c>
+      <c r="D64" s="95" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="65">
-      <c r="C65" s="89">
+      <c r="C65" s="96">
         <v>6</v>
       </c>
-      <c r="D65" s="89" t="s">
-        <v>332</v>
+      <c r="D65" s="96" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="81" t="s">
-        <v>333</v>
-      </c>
-      <c r="D66" s="71" t="s">
+      <c r="C66" s="88" t="s">
         <v>334</v>
       </c>
+      <c r="D66" s="78" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="67">
-      <c r="C67" s="90" t="s">
-        <v>335</v>
-      </c>
-      <c r="D67" s="91" t="s">
+      <c r="C67" s="97" t="s">
         <v>336</v>
       </c>
+      <c r="D67" s="98" t="s">
+        <v>337</v>
+      </c>
     </row>
     <row r="68">
-      <c r="C68" s="81" t="s">
-        <v>337</v>
-      </c>
-      <c r="D68" s="88" t="s">
+      <c r="C68" s="88" t="s">
         <v>338</v>
       </c>
+      <c r="D68" s="95" t="s">
+        <v>339</v>
+      </c>
     </row>
     <row r="69">
-      <c r="C69" s="90" t="s">
-        <v>339</v>
-      </c>
-      <c r="D69" s="88" t="s">
+      <c r="C69" s="97" t="s">
         <v>340</v>
       </c>
+      <c r="D69" s="95" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="70">
-      <c r="C70" s="81" t="s">
-        <v>341</v>
-      </c>
-      <c r="D70" s="88" t="s">
+      <c r="C70" s="88" t="s">
         <v>342</v>
       </c>
+      <c r="D70" s="95" t="s">
+        <v>343</v>
+      </c>
     </row>
     <row r="71">
-      <c r="C71" s="89">
+      <c r="C71" s="96">
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="81" t="s">
-        <v>344</v>
-      </c>
-      <c r="D72" s="71" t="s">
+      <c r="C72" s="88" t="s">
         <v>345</v>
       </c>
+      <c r="D72" s="78" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="73">
-      <c r="C73" s="89">
+      <c r="C73" s="96">
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="81" t="s">
-        <v>347</v>
-      </c>
-      <c r="D74" s="71" t="s">
+      <c r="C74" s="88" t="s">
         <v>348</v>
       </c>
+      <c r="D74" s="78" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="75">
-      <c r="C75" s="89">
+      <c r="C75" s="96">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="81" t="s">
-        <v>349</v>
-      </c>
-      <c r="D76" s="71" t="s">
+      <c r="C76" s="88" t="s">
         <v>350</v>
       </c>
+      <c r="D76" s="78" t="s">
+        <v>351</v>
+      </c>
     </row>
     <row r="77">
-      <c r="C77" s="81" t="s">
-        <v>351</v>
-      </c>
-      <c r="D77" s="88" t="s">
+      <c r="C77" s="88" t="s">
         <v>352</v>
       </c>
+      <c r="D77" s="95" t="s">
+        <v>353</v>
+      </c>
     </row>
     <row r="78">
-      <c r="C78" s="81" t="s">
-        <v>353</v>
-      </c>
-      <c r="D78" s="88" t="s">
+      <c r="C78" s="88" t="s">
         <v>354</v>
       </c>
+      <c r="D78" s="95" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="79">
-      <c r="C79" s="89">
+      <c r="C79" s="96">
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="81" t="s">
-        <v>356</v>
-      </c>
-      <c r="D80" s="71" t="s">
+      <c r="C80" s="88" t="s">
         <v>357</v>
       </c>
-      <c r="E80" s="75"/>
+      <c r="D80" s="78" t="s">
+        <v>358</v>
+      </c>
+      <c r="E80" s="82"/>
     </row>
     <row r="81">
-      <c r="C81" s="81" t="s">
-        <v>358</v>
-      </c>
-      <c r="D81" s="88" t="s">
+      <c r="C81" s="88" t="s">
         <v>359</v>
       </c>
+      <c r="D81" s="95" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="82">
-      <c r="C82" s="89">
+      <c r="C82" s="96">
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="81" t="s">
-        <v>361</v>
-      </c>
-      <c r="D83" s="71" t="s">
+      <c r="C83" s="88" t="s">
         <v>362</v>
       </c>
+      <c r="D83" s="78" t="s">
+        <v>363</v>
+      </c>
     </row>
     <row r="84">
-      <c r="C84" s="81" t="s">
-        <v>363</v>
-      </c>
-      <c r="D84" s="71" t="s">
+      <c r="C84" s="88" t="s">
         <v>364</v>
+      </c>
+      <c r="D84" s="78" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bordezu + bonne gestion lecteur, dispay... OK
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -7,9 +7,10 @@
   </bookViews>
   <sheets>
     <sheet name="Reprise" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Archive - Setup Raspberry" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Archive - Mache à état" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Archive - Cahier des charges" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Matos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Archive - Setup Raspberry" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Archive - Mache à état" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Archive - Cahier des charges" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -194,7 +195,11 @@
   </si>
   <si>
     <t xml:space="preserve">Vérifier potentiomètres moteurs, calcul à la main !! Sans IA au début, puis on vérifie
-Pb : Moteur X fait du bruit quand branché</t>
+Pb : Moteur X fait du bruit quand branché, chauffe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A4988 -&gt; Je ne trouve pas RSens, donc galère de calculer Vref
+Si pas trop de bruits ~ Okk</t>
   </si>
   <si>
     <t xml:space="preserve">Plaque avec support Cds et lecteur, prévoir place lecteur !</t>
@@ -222,9 +227,9 @@
 # Init machine a etats puis attente actions OK
 # Calibrer les positions OK
 # playCd -&gt; Bouge au CD puis reviens origin OK
-- Pb : timeout de 10s, si mouvement plus long la connexion coupe
+// Pb : timeout de 10s, si mouvement plus long la connexion coupe
     https://claude.ai/chat/1f9255f3-cb82-455e-8c4a-e6fc560f6c47
-- Tester toute la machine a etat, sur la durée</t>
+    MIS EN PLACE 30s : TESTER</t>
   </si>
   <si>
     <t xml:space="preserve">Prévoir tiges? pour fixer armature à planche, avec une certaine distance</t>
@@ -255,7 +260,8 @@
     <t>Font</t>
   </si>
   <si>
-    <t xml:space="preserve">- Logique de placement des CDs sur le lecteur,     Appeler GoToPos 2 fois : aller de a à b avec action sur CD, PUIS aller de b à c avec action CD</t>
+    <t xml:space="preserve">Ajouter le lecteur sur le front avec cd qui tourne + borderau en quand on ferme le lecteur
+    - Voir dessin</t>
   </si>
   <si>
     <t xml:space="preserve">Calculer nb step pour chaque positions</t>
@@ -406,6 +412,15 @@
   </si>
   <si>
     <t xml:space="preserve">Lancement nouveau CD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moteur 17HS15-0404S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilote A4988</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raspberry PI 3B</t>
   </si>
   <si>
     <t>Steps</t>
@@ -1276,7 +1291,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -1343,6 +1358,11 @@
       <sz val="12.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF212529"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10.000000"/>
@@ -1686,7 +1706,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="96">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1744,25 +1764,17 @@
       <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="16" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1778,6 +1790,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf fontId="10" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="11" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf fontId="0" fillId="17" borderId="7" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="17" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -1785,27 +1800,27 @@
     <xf fontId="0" fillId="17" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="13" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="11" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="15" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="11" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
-    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="11" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
-    <xf fontId="11" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="17" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="11" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="17" borderId="13" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1817,7 +1832,7 @@
     </xf>
     <xf fontId="0" fillId="17" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="17" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="13" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="14" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="10" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1829,7 +1844,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf fontId="13" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="14" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="10" borderId="3" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
@@ -1838,16 +1853,16 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2" wrapText="1"/>
     </xf>
-    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="16" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
@@ -1859,7 +1874,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="16" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="17" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2742,7 +2757,7 @@
       <c r="C13" s="13"/>
       <c r="D13" s="14">
         <f>SUM(D14:D22)/9</f>
-        <v>0.75</v>
+        <v>0.76666666666666672</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>22</v>
@@ -2980,11 +2995,14 @@
       <c r="B19" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="32">
+      <c r="C19" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="33">
         <v>0</v>
       </c>
       <c r="F19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G19" s="16" t="s">
         <v>23</v>
@@ -3005,30 +3023,30 @@
     <row r="20" ht="28.5">
       <c r="A20" s="1"/>
       <c r="B20" s="26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D20" s="28">
         <v>1</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>23</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="M20" s="33" t="s">
         <v>62</v>
+      </c>
+      <c r="M20" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="N20" s="1"/>
       <c r="O20" s="22"/>
@@ -3041,17 +3059,17 @@
       <c r="Z20" s="1"/>
       <c r="AA20" s="1"/>
     </row>
-    <row r="21" ht="242.25">
+    <row r="21" ht="128.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="34" t="s">
-        <v>63</v>
+      <c r="B21" s="26" t="s">
+        <v>64</v>
       </c>
       <c r="C21" s="35"/>
       <c r="D21" s="36">
-        <v>0.75</v>
+        <v>0.90000000000000002</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>23</v>
@@ -3059,10 +3077,10 @@
       <c r="H21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" t="s">
-        <v>65</v>
-      </c>
-      <c r="M21" s="33" t="s">
-        <v>62</v>
+        <v>66</v>
+      </c>
+      <c r="M21" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="N21" s="1"/>
       <c r="O21" s="2"/>
@@ -3073,42 +3091,42 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="X21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" ht="16.5">
+    <row r="22" ht="42.75">
       <c r="A22" s="1"/>
-      <c r="B22" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="38"/>
-      <c r="D22" s="39">
+      <c r="B22" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="35"/>
+      <c r="D22" s="33">
         <v>0</v>
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="M22" s="33" t="s">
-        <v>62</v>
+        <v>70</v>
+      </c>
+      <c r="M22" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3116,62 +3134,61 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
     </row>
-    <row r="23" ht="16.5">
+    <row r="23" ht="42.75">
       <c r="A23" s="1"/>
-      <c r="B23" s="40" t="s">
-        <v>73</v>
-      </c>
-      <c r="D23" s="32"/>
+      <c r="B23" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="33"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="41"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>74</v>
-      </c>
-      <c r="M23" s="33" t="s">
-        <v>62</v>
+        <v>75</v>
+      </c>
+      <c r="M23" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="N23" s="1"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
-      <c r="B24"/>
-      <c r="D24" s="32"/>
-      <c r="F24" s="42" t="s">
-        <v>77</v>
+      <c r="D24" s="33"/>
+      <c r="F24" s="38" t="s">
+        <v>78</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="43"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="45"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="41"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3205,11 +3222,11 @@
     </row>
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="46" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48">
+      <c r="B26" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="43"/>
+      <c r="D26" s="44">
         <f>SUM(D27:D32)/5</f>
         <v>0</v>
       </c>
@@ -3223,10 +3240,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3239,12 +3256,12 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="32">
+        <v>85</v>
+      </c>
+      <c r="D27" s="33">
         <v>0</v>
       </c>
       <c r="N27" s="1"/>
@@ -3256,7 +3273,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3264,9 +3281,9 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="C28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="32">
+        <v>87</v>
+      </c>
+      <c r="D28" s="33">
         <v>0</v>
       </c>
       <c r="L28" s="19"/>
@@ -3280,7 +3297,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3288,9 +3305,9 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>88</v>
-      </c>
-      <c r="D29" s="32">
+        <v>89</v>
+      </c>
+      <c r="D29" s="33">
         <v>0</v>
       </c>
       <c r="M29" s="1"/>
@@ -3308,12 +3325,12 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="32">
+        <v>91</v>
+      </c>
+      <c r="D30" s="33">
         <v>0</v>
       </c>
       <c r="L30" s="19"/>
@@ -3332,12 +3349,12 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D31" s="32">
+        <v>93</v>
+      </c>
+      <c r="D31" s="33">
         <v>0</v>
       </c>
       <c r="N31" s="1"/>
@@ -3354,13 +3371,13 @@
     <row r="32" ht="28.5">
       <c r="A32" s="1"/>
       <c r="B32" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D32" s="32">
+        <v>94</v>
+      </c>
+      <c r="D32" s="33">
         <v>0</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3368,9 +3385,9 @@
     <row r="33" ht="16.5">
       <c r="A33" s="1"/>
       <c r="B33" s="4"/>
-      <c r="D33" s="32"/>
+      <c r="D33" s="33"/>
       <c r="L33" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3384,7 +3401,7 @@
     <row r="34" ht="16.5">
       <c r="A34" s="1"/>
       <c r="B34" s="4"/>
-      <c r="D34" s="32"/>
+      <c r="D34" s="33"/>
       <c r="L34" s="19"/>
       <c r="M34" s="19"/>
       <c r="N34" s="1"/>
@@ -3411,11 +3428,11 @@
     </row>
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
-      <c r="B36" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="C36" s="47"/>
-      <c r="D36" s="48">
+      <c r="B36" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="43"/>
+      <c r="D36" s="44">
         <f>SUM(D37:D40)/4</f>
         <v>0</v>
       </c>
@@ -3433,12 +3450,12 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D37" s="32">
+        <v>99</v>
+      </c>
+      <c r="D37" s="33">
         <v>0</v>
       </c>
       <c r="L37" s="2"/>
@@ -3455,12 +3472,12 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D38" s="32">
+        <v>101</v>
+      </c>
+      <c r="D38" s="33">
         <v>0</v>
       </c>
       <c r="L38" s="2"/>
@@ -3477,24 +3494,24 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="D39" s="32">
+        <v>103</v>
+      </c>
+      <c r="D39" s="33">
         <v>0</v>
       </c>
     </row>
     <row r="40" ht="28.5">
       <c r="A40" s="1"/>
       <c r="B40" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="D40" s="32">
+        <v>105</v>
+      </c>
+      <c r="D40" s="33">
         <v>0</v>
       </c>
     </row>
@@ -3504,7 +3521,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3512,7 +3529,7 @@
     <row r="43" ht="16.5">
       <c r="A43" s="1"/>
       <c r="B43" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -3523,7 +3540,7 @@
     <row r="45" ht="16.5">
       <c r="A45" s="1"/>
       <c r="B45" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="46" ht="14.25">
@@ -3535,7 +3552,7 @@
     <row r="48" ht="14.25">
       <c r="A48" s="1"/>
       <c r="B48" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" ht="14.25">
@@ -3544,13 +3561,13 @@
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" ht="14.25">
       <c r="A51" s="1"/>
       <c r="B51" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="52" ht="16.5">
@@ -3562,7 +3579,7 @@
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3578,7 +3595,7 @@
     <row r="55" ht="16.5">
       <c r="A55" s="1"/>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -3607,7 +3624,7 @@
     <row r="57" ht="16.5">
       <c r="A57" s="1"/>
       <c r="B57" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -3635,55 +3652,55 @@
     </row>
     <row r="69" ht="14.25">
       <c r="B69" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="78" ht="14.25">
       <c r="B78" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C78" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3703,6 +3720,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="21.00390625"/>
+    <col customWidth="1" min="3" max="3" width="9.28125"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="14.25">
+      <c r="B2" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="43.5546875"/>
@@ -3713,280 +3759,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="50" t="s">
-        <v>124</v>
-      </c>
-      <c r="G2" s="51" t="s">
-        <v>125</v>
+      <c r="F2" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="G2" s="48" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="3">
-      <c r="F3" s="52" t="s">
-        <v>126</v>
-      </c>
-      <c r="G3" s="53" t="s">
-        <v>127</v>
+      <c r="F3" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="G3" s="50" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="4">
-      <c r="F4" s="54" t="s">
-        <v>128</v>
-      </c>
-      <c r="G4" s="55" t="s">
-        <v>129</v>
+      <c r="F4" s="51" t="s">
+        <v>132</v>
+      </c>
+      <c r="G4" s="52" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="F5" s="56" t="s">
-        <v>130</v>
-      </c>
-      <c r="G5" s="57" t="s">
-        <v>131</v>
+      <c r="F5" s="53" t="s">
+        <v>134</v>
+      </c>
+      <c r="G5" s="54" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="F6" s="58"/>
-      <c r="G6" s="59" t="s">
-        <v>132</v>
+      <c r="F6" s="55"/>
+      <c r="G6" s="56" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="F7" s="58"/>
-      <c r="G7" s="59" t="s">
-        <v>133</v>
+      <c r="F7" s="55"/>
+      <c r="G7" s="56" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="F8" s="58"/>
-      <c r="G8" s="59" t="s">
-        <v>134</v>
+      <c r="F8" s="55"/>
+      <c r="G8" s="56" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>135</v>
-      </c>
-      <c r="F9" s="58"/>
-      <c r="G9" s="59" t="s">
-        <v>136</v>
+        <v>139</v>
+      </c>
+      <c r="F9" s="55"/>
+      <c r="G9" s="56" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C10" s="60" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="58"/>
-      <c r="G10" s="59" t="s">
-        <v>139</v>
+        <v>141</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>142</v>
+      </c>
+      <c r="F10" s="55"/>
+      <c r="G10" s="56" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="11" ht="15">
-      <c r="C11" s="61" t="s">
-        <v>140</v>
-      </c>
-      <c r="F11" s="58"/>
-      <c r="G11" s="59" t="s">
-        <v>141</v>
+      <c r="C11" s="58" t="s">
+        <v>144</v>
+      </c>
+      <c r="F11" s="55"/>
+      <c r="G11" s="56" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="C12" s="60" t="s">
-        <v>142</v>
-      </c>
-      <c r="F12" s="52"/>
-      <c r="G12" s="62" t="s">
-        <v>143</v>
+      <c r="C12" s="57" t="s">
+        <v>146</v>
+      </c>
+      <c r="F12" s="49"/>
+      <c r="G12" s="59" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="13" ht="15">
-      <c r="C13" s="61" t="s">
-        <v>144</v>
-      </c>
-      <c r="F13" s="54" t="s">
-        <v>145</v>
-      </c>
-      <c r="G13" s="63" t="s">
-        <v>146</v>
+      <c r="C13" s="58" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="60" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="14" ht="15">
-      <c r="C14" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="F14" s="64" t="s">
-        <v>148</v>
-      </c>
-      <c r="G14" s="65" t="s">
-        <v>149</v>
+      <c r="C14" s="57" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="61" t="s">
+        <v>152</v>
+      </c>
+      <c r="G14" s="62" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="61" t="s">
-        <v>150</v>
-      </c>
-      <c r="F15" s="66" t="s">
-        <v>151</v>
-      </c>
-      <c r="G15" s="67" t="s">
-        <v>152</v>
+      <c r="C15" s="58" t="s">
+        <v>154</v>
+      </c>
+      <c r="F15" s="63" t="s">
+        <v>155</v>
+      </c>
+      <c r="G15" s="64" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="61" t="s">
-        <v>153</v>
-      </c>
-      <c r="F16" s="68" t="s">
-        <v>154</v>
-      </c>
-      <c r="G16" s="69" t="s">
-        <v>155</v>
+      <c r="C16" s="58" t="s">
+        <v>157</v>
+      </c>
+      <c r="F16" s="65" t="s">
+        <v>158</v>
+      </c>
+      <c r="G16" s="66" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="60" t="s">
-        <v>156</v>
-      </c>
-      <c r="F17" s="68"/>
-      <c r="G17" s="69" t="s">
-        <v>157</v>
+      <c r="C17" s="57" t="s">
+        <v>160</v>
+      </c>
+      <c r="F17" s="65"/>
+      <c r="G17" s="66" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="61" t="s">
-        <v>158</v>
-      </c>
-      <c r="F18" s="68"/>
-      <c r="G18" s="69" t="s">
-        <v>159</v>
+      <c r="C18" s="58" t="s">
+        <v>162</v>
+      </c>
+      <c r="F18" s="65"/>
+      <c r="G18" s="66" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="61" t="s">
-        <v>160</v>
-      </c>
-      <c r="F19" s="68"/>
-      <c r="G19" s="69" t="s">
-        <v>161</v>
+      <c r="C19" s="58" t="s">
+        <v>164</v>
+      </c>
+      <c r="F19" s="65"/>
+      <c r="G19" s="66" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="61" t="s">
-        <v>162</v>
-      </c>
-      <c r="F20" s="68"/>
-      <c r="G20" s="69" t="s">
-        <v>163</v>
+      <c r="C20" s="58" t="s">
+        <v>166</v>
+      </c>
+      <c r="F20" s="65"/>
+      <c r="G20" s="66" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="61" t="s">
-        <v>164</v>
-      </c>
-      <c r="F21" s="68"/>
-      <c r="G21" s="69" t="s">
-        <v>165</v>
+      <c r="C21" s="58" t="s">
+        <v>168</v>
+      </c>
+      <c r="F21" s="65"/>
+      <c r="G21" s="66" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="60" t="s">
-        <v>166</v>
-      </c>
-      <c r="F22" s="68"/>
-      <c r="G22" s="69" t="s">
-        <v>167</v>
+      <c r="C22" s="57" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" s="65"/>
+      <c r="G22" s="66" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="61" t="s">
-        <v>168</v>
-      </c>
-      <c r="F23" s="68"/>
-      <c r="G23" s="69" t="s">
-        <v>169</v>
+      <c r="C23" s="58" t="s">
+        <v>172</v>
+      </c>
+      <c r="F23" s="65"/>
+      <c r="G23" s="66" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="60" t="s">
-        <v>170</v>
-      </c>
-      <c r="F24" s="68"/>
-      <c r="G24" s="69" t="s">
-        <v>171</v>
+      <c r="C24" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="F24" s="65"/>
+      <c r="G24" s="66" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="61" t="s">
-        <v>172</v>
-      </c>
-      <c r="F25" s="68"/>
-      <c r="G25" s="69" t="s">
-        <v>173</v>
+      <c r="C25" s="58" t="s">
+        <v>176</v>
+      </c>
+      <c r="F25" s="65"/>
+      <c r="G25" s="66" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="26">
-      <c r="F26" s="68"/>
-      <c r="G26" s="69" t="s">
-        <v>174</v>
+      <c r="F26" s="65"/>
+      <c r="G26" s="66" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="68"/>
-      <c r="G27" s="69"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="66"/>
     </row>
     <row r="28">
-      <c r="F28" s="68"/>
-      <c r="G28" s="69" t="s">
-        <v>175</v>
+      <c r="F28" s="65"/>
+      <c r="G28" s="66" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="68"/>
-      <c r="G29" s="69" t="s">
-        <v>176</v>
+      <c r="F29" s="65"/>
+      <c r="G29" s="66" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="70"/>
-      <c r="F30" s="68"/>
-      <c r="G30" s="69" t="s">
-        <v>177</v>
+      <c r="C30" s="67"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="66" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="68"/>
-      <c r="G31" s="71" t="s">
-        <v>178</v>
+      <c r="F31" s="65"/>
+      <c r="G31" s="68" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="64" t="s">
-        <v>179</v>
-      </c>
-      <c r="G32" s="72" t="s">
-        <v>180</v>
+      <c r="F32" s="61" t="s">
+        <v>183</v>
+      </c>
+      <c r="G32" s="69" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="61"/>
+      <c r="C33" s="58"/>
     </row>
     <row r="34">
-      <c r="C34" s="61"/>
+      <c r="C34" s="58"/>
     </row>
     <row r="36">
-      <c r="C36" s="70"/>
+      <c r="C36" s="67"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="61"/>
+      <c r="C39" s="58"/>
     </row>
     <row r="40">
-      <c r="C40" s="61"/>
+      <c r="C40" s="58"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -3996,7 +4042,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
@@ -4014,367 +4060,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D5" s="73" t="s">
-        <v>183</v>
+        <v>186</v>
+      </c>
+      <c r="D5" s="70" t="s">
+        <v>187</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G5" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="H5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="I5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="J5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="K5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D6" s="74" t="s">
-        <v>191</v>
+        <v>194</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>195</v>
       </c>
       <c r="E6" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F6" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="G6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H6" s="75" t="s">
-        <v>195</v>
+        <v>198</v>
+      </c>
+      <c r="H6" s="72" t="s">
+        <v>199</v>
       </c>
       <c r="I6" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="J6" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="K6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
-      </c>
-      <c r="D7" s="76" t="s">
-        <v>200</v>
+        <v>194</v>
+      </c>
+      <c r="D7" s="73" t="s">
+        <v>204</v>
       </c>
       <c r="F7" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="G7" t="s">
-        <v>202</v>
-      </c>
-      <c r="H7" s="75" t="s">
-        <v>203</v>
+        <v>206</v>
+      </c>
+      <c r="H7" s="72" t="s">
+        <v>207</v>
       </c>
       <c r="K7" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="74" t="s">
-        <v>205</v>
-      </c>
-      <c r="G8" s="77" t="s">
-        <v>206</v>
-      </c>
-      <c r="H8" s="75" t="s">
-        <v>207</v>
+      <c r="D8" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="G8" s="74" t="s">
+        <v>210</v>
+      </c>
+      <c r="H8" s="72" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B9" t="s">
-        <v>209</v>
-      </c>
-      <c r="D9" s="76" t="s">
-        <v>210</v>
-      </c>
-      <c r="H9" s="75" t="s">
-        <v>211</v>
+        <v>213</v>
+      </c>
+      <c r="D9" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="H9" s="72" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B10" t="s">
-        <v>213</v>
-      </c>
-      <c r="D10" s="74"/>
+        <v>217</v>
+      </c>
+      <c r="D10" s="71"/>
       <c r="G10" t="s">
-        <v>214</v>
-      </c>
-      <c r="H10" s="75" t="s">
-        <v>215</v>
+        <v>218</v>
+      </c>
+      <c r="H10" s="72" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
-      </c>
-      <c r="D11" s="76" t="s">
-        <v>218</v>
-      </c>
-      <c r="G11" s="77" t="s">
-        <v>219</v>
-      </c>
-      <c r="H11" s="75" t="s">
-        <v>220</v>
+        <v>221</v>
+      </c>
+      <c r="D11" s="73" t="s">
+        <v>222</v>
+      </c>
+      <c r="G11" s="74" t="s">
+        <v>223</v>
+      </c>
+      <c r="H11" s="72" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B12" t="s">
-        <v>222</v>
-      </c>
-      <c r="D12" s="74" t="s">
-        <v>223</v>
-      </c>
-      <c r="G12" s="77" t="s">
-        <v>224</v>
-      </c>
-      <c r="H12" s="75" t="s">
-        <v>225</v>
+        <v>226</v>
+      </c>
+      <c r="D12" s="71" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" s="74" t="s">
+        <v>228</v>
+      </c>
+      <c r="H12" s="72" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D13" s="76" t="s">
-        <v>228</v>
-      </c>
-      <c r="G13" s="77" t="s">
-        <v>229</v>
+        <v>231</v>
+      </c>
+      <c r="D13" s="73" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" s="74" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="74" t="s">
-        <v>230</v>
+      <c r="D14" s="71" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B15" t="s">
-        <v>232</v>
-      </c>
-      <c r="D15" s="76"/>
+        <v>236</v>
+      </c>
+      <c r="D15" s="73"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B16" t="s">
-        <v>234</v>
-      </c>
-      <c r="D16" s="74"/>
+        <v>238</v>
+      </c>
+      <c r="D16" s="71"/>
       <c r="G16" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="76"/>
-      <c r="G17" s="77" t="s">
-        <v>236</v>
+      <c r="D17" s="73"/>
+      <c r="G17" s="74" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>237</v>
-      </c>
-      <c r="D18" s="74"/>
-      <c r="G18" s="78" t="s">
-        <v>238</v>
+        <v>241</v>
+      </c>
+      <c r="D18" s="71"/>
+      <c r="G18" s="75" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="76" t="s">
-        <v>239</v>
+      <c r="D19" s="73" t="s">
+        <v>243</v>
       </c>
       <c r="E19" t="s">
-        <v>240</v>
-      </c>
-      <c r="G19" s="78" t="s">
-        <v>241</v>
+        <v>244</v>
+      </c>
+      <c r="G19" s="75" t="s">
+        <v>245</v>
       </c>
       <c r="H19" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="I19" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="J19" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="74"/>
-      <c r="G20" s="78" t="s">
-        <v>244</v>
+      <c r="D20" s="71"/>
+      <c r="G20" s="75" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="74"/>
-      <c r="G22" s="78" t="s">
-        <v>229</v>
+      <c r="D22" s="71"/>
+      <c r="G22" s="75" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="23">
-      <c r="G23" s="77"/>
+      <c r="G23" s="74"/>
     </row>
     <row r="24">
-      <c r="D24" s="74"/>
-      <c r="G24" s="77" t="s">
+      <c r="D24" s="71"/>
+      <c r="G24" s="74" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="75" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="71"/>
+      <c r="G26" s="75" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="75" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="71"/>
+      <c r="G28" s="75" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="25">
-      <c r="G25" s="78" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" s="74"/>
-      <c r="G26" s="78" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="78" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="74"/>
-      <c r="G28" s="78" t="s">
-        <v>241</v>
-      </c>
-    </row>
     <row r="35">
-      <c r="D35" s="79" t="s">
-        <v>249</v>
+      <c r="D35" s="76" t="s">
+        <v>253</v>
       </c>
       <c r="E35" t="s">
-        <v>250</v>
-      </c>
-      <c r="F35" s="80" t="s">
-        <v>251</v>
+        <v>254</v>
+      </c>
+      <c r="F35" s="77" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="36">
-      <c r="D36" s="81" t="s">
-        <v>252</v>
+      <c r="D36" s="78" t="s">
+        <v>256</v>
       </c>
       <c r="E36" t="s">
-        <v>253</v>
-      </c>
-      <c r="F36" s="81" t="s">
-        <v>254</v>
+        <v>257</v>
+      </c>
+      <c r="F36" s="78" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="37">
-      <c r="D37" s="80" t="s">
-        <v>255</v>
+      <c r="D37" s="77" t="s">
+        <v>259</v>
       </c>
       <c r="E37" t="s">
-        <v>256</v>
-      </c>
-      <c r="F37" s="80" t="s">
-        <v>257</v>
+        <v>260</v>
+      </c>
+      <c r="F37" s="77" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="81" t="s">
-        <v>258</v>
+      <c r="D38" s="78" t="s">
+        <v>262</v>
       </c>
       <c r="E38" t="s">
-        <v>259</v>
-      </c>
-      <c r="F38" s="81" t="s">
-        <v>260</v>
+        <v>263</v>
+      </c>
+      <c r="F38" s="78" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="39">
-      <c r="D39" s="80" t="s">
-        <v>261</v>
+      <c r="D39" s="77" t="s">
+        <v>265</v>
       </c>
       <c r="E39" t="s">
-        <v>262</v>
-      </c>
-      <c r="F39" s="80" t="s">
-        <v>263</v>
+        <v>266</v>
+      </c>
+      <c r="F39" s="77" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>253</v>
-      </c>
-      <c r="F40" s="81" t="s">
-        <v>264</v>
+        <v>257</v>
+      </c>
+      <c r="F40" s="78" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>256</v>
-      </c>
-      <c r="F41" s="80" t="s">
-        <v>265</v>
+        <v>260</v>
+      </c>
+      <c r="F41" s="77" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4389,7 +4435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
@@ -4405,564 +4451,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="82" t="s">
-        <v>268</v>
+      <c r="D4" s="79" t="s">
+        <v>272</v>
       </c>
       <c r="E4" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
-        <v>270</v>
-      </c>
-      <c r="E5" s="82">
+        <v>274</v>
+      </c>
+      <c r="E5" s="79">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="78" t="s">
-        <v>271</v>
-      </c>
-      <c r="E6" s="82">
+      <c r="D6" s="75" t="s">
+        <v>275</v>
+      </c>
+      <c r="E6" s="79">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="83" t="s">
-        <v>272</v>
-      </c>
-      <c r="E7" s="82">
+      <c r="D7" s="80" t="s">
+        <v>276</v>
+      </c>
+      <c r="E7" s="79">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="75" t="s">
+        <v>277</v>
+      </c>
+      <c r="E8" s="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="75"/>
+      <c r="E9" s="79"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="72" t="s">
+        <v>278</v>
+      </c>
+      <c r="E10" s="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="75" t="s">
+        <v>279</v>
+      </c>
+      <c r="E11" s="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="75" t="s">
+        <v>280</v>
+      </c>
+      <c r="E12" s="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="75" t="s">
+        <v>281</v>
+      </c>
+      <c r="E13" s="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="75"/>
+      <c r="E14" s="75"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="72" t="s">
+        <v>282</v>
+      </c>
+      <c r="E15" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="81" t="s">
+        <v>283</v>
+      </c>
+      <c r="E16" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="82" t="s">
+        <v>284</v>
+      </c>
+      <c r="E17" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="82" t="s">
+        <v>285</v>
+      </c>
+      <c r="E18" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="75"/>
+      <c r="E19" s="75"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="72" t="s">
+        <v>286</v>
+      </c>
+      <c r="E20" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" s="72" t="s">
+        <v>287</v>
+      </c>
+      <c r="E21" s="79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="75"/>
+      <c r="E22" s="75"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="83"/>
+      <c r="E23" s="75"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="75"/>
+      <c r="E24" s="75"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="75"/>
+      <c r="E25" s="75"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="75"/>
+      <c r="E26" s="75"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="75"/>
+      <c r="E27" s="75"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="75"/>
+      <c r="E28" s="75"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="75"/>
+      <c r="E29" s="75"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="75"/>
+      <c r="E30" s="75"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="84"/>
+      <c r="C39" s="85" t="s">
+        <v>288</v>
+      </c>
+      <c r="D39" s="85" t="s">
+        <v>289</v>
+      </c>
+      <c r="E39" t="s">
         <v>273</v>
-      </c>
-      <c r="E8" s="82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="78"/>
-      <c r="E9" s="82"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="75" t="s">
-        <v>274</v>
-      </c>
-      <c r="E10" s="82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" s="78" t="s">
-        <v>275</v>
-      </c>
-      <c r="E11" s="82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="78" t="s">
-        <v>276</v>
-      </c>
-      <c r="E12" s="82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="78" t="s">
-        <v>277</v>
-      </c>
-      <c r="E13" s="82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="78"/>
-      <c r="E14" s="78"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="75" t="s">
-        <v>278</v>
-      </c>
-      <c r="E15" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="84" t="s">
-        <v>279</v>
-      </c>
-      <c r="E16" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="85" t="s">
-        <v>280</v>
-      </c>
-      <c r="E17" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" s="85" t="s">
-        <v>281</v>
-      </c>
-      <c r="E18" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="78"/>
-      <c r="E19" s="78"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="75" t="s">
-        <v>282</v>
-      </c>
-      <c r="E20" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" s="75" t="s">
-        <v>283</v>
-      </c>
-      <c r="E21" s="82">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="78"/>
-      <c r="E22" s="78"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="86"/>
-      <c r="E23" s="78"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="78"/>
-      <c r="E24" s="78"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="78"/>
-      <c r="E25" s="78"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="78"/>
-      <c r="E26" s="78"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="78"/>
-      <c r="E27" s="78"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="78"/>
-      <c r="E28" s="78"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="78"/>
-      <c r="E30" s="78"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="87"/>
-      <c r="C39" s="88" t="s">
-        <v>284</v>
-      </c>
-      <c r="D39" s="88" t="s">
-        <v>285</v>
-      </c>
-      <c r="E39" t="s">
-        <v>269</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="89">
+      <c r="C40" s="86">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>286</v>
-      </c>
-      <c r="E40" s="82"/>
+        <v>290</v>
+      </c>
+      <c r="E40" s="79"/>
     </row>
     <row r="41">
-      <c r="C41" s="82" t="s">
-        <v>287</v>
-      </c>
-      <c r="D41" s="78" t="s">
-        <v>288</v>
-      </c>
-      <c r="E41" s="82"/>
+      <c r="C41" s="79" t="s">
+        <v>291</v>
+      </c>
+      <c r="D41" s="75" t="s">
+        <v>292</v>
+      </c>
+      <c r="E41" s="79"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="82" t="s">
-        <v>289</v>
-      </c>
-      <c r="D42" s="78" t="s">
-        <v>290</v>
+      <c r="C42" s="79" t="s">
+        <v>293</v>
+      </c>
+      <c r="D42" s="75" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="82" t="s">
-        <v>291</v>
-      </c>
-      <c r="D43" s="78" t="s">
-        <v>292</v>
+      <c r="C43" s="79" t="s">
+        <v>295</v>
+      </c>
+      <c r="D43" s="75" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="90" t="s">
-        <v>293</v>
-      </c>
-      <c r="D44" s="83" t="s">
-        <v>294</v>
-      </c>
-      <c r="E44" s="91"/>
-      <c r="F44" s="91"/>
+      <c r="C44" s="87" t="s">
+        <v>297</v>
+      </c>
+      <c r="D44" s="80" t="s">
+        <v>298</v>
+      </c>
+      <c r="E44" s="88"/>
+      <c r="F44" s="88"/>
     </row>
     <row r="45">
-      <c r="C45" s="88" t="s">
-        <v>295</v>
-      </c>
-      <c r="D45" s="78" t="s">
-        <v>296</v>
-      </c>
-      <c r="E45" s="82"/>
+      <c r="C45" s="85" t="s">
+        <v>299</v>
+      </c>
+      <c r="D45" s="75" t="s">
+        <v>300</v>
+      </c>
+      <c r="E45" s="79"/>
     </row>
     <row r="46">
-      <c r="C46" s="88" t="s">
-        <v>297</v>
-      </c>
-      <c r="D46" s="78" t="s">
-        <v>298</v>
-      </c>
-      <c r="E46" s="82"/>
+      <c r="C46" s="85" t="s">
+        <v>301</v>
+      </c>
+      <c r="D46" s="75" t="s">
+        <v>302</v>
+      </c>
+      <c r="E46" s="79"/>
     </row>
     <row r="47">
-      <c r="C47" s="92">
+      <c r="C47" s="89">
         <v>2</v>
       </c>
-      <c r="D47" s="93" t="s">
-        <v>299</v>
-      </c>
-      <c r="E47" s="82"/>
+      <c r="D47" s="90" t="s">
+        <v>303</v>
+      </c>
+      <c r="E47" s="79"/>
     </row>
     <row r="48">
-      <c r="C48" s="90" t="s">
-        <v>300</v>
-      </c>
-      <c r="D48" s="83" t="s">
-        <v>301</v>
-      </c>
-      <c r="E48" s="82"/>
+      <c r="C48" s="87" t="s">
+        <v>304</v>
+      </c>
+      <c r="D48" s="80" t="s">
+        <v>305</v>
+      </c>
+      <c r="E48" s="79"/>
     </row>
     <row r="49">
-      <c r="C49" s="89">
+      <c r="C49" s="86">
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="E49" s="82"/>
+        <v>306</v>
+      </c>
+      <c r="E49" s="79"/>
     </row>
     <row r="50">
-      <c r="C50" s="90" t="s">
-        <v>303</v>
-      </c>
-      <c r="D50" s="83" t="s">
-        <v>304</v>
-      </c>
-      <c r="F50" s="94" t="s">
-        <v>305</v>
+      <c r="C50" s="87" t="s">
+        <v>307</v>
+      </c>
+      <c r="D50" s="80" t="s">
+        <v>308</v>
+      </c>
+      <c r="F50" s="91" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="51">
-      <c r="C51" s="90" t="s">
-        <v>306</v>
-      </c>
-      <c r="D51" s="95" t="s">
-        <v>307</v>
+      <c r="C51" s="87" t="s">
+        <v>310</v>
+      </c>
+      <c r="D51" s="92" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="90" t="s">
-        <v>308</v>
-      </c>
-      <c r="D52" s="95" t="s">
-        <v>309</v>
+      <c r="C52" s="87" t="s">
+        <v>312</v>
+      </c>
+      <c r="D52" s="92" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="90" t="s">
-        <v>310</v>
-      </c>
-      <c r="D53" s="95" t="s">
-        <v>311</v>
+      <c r="C53" s="87" t="s">
+        <v>314</v>
+      </c>
+      <c r="D53" s="92" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="90" t="s">
-        <v>312</v>
-      </c>
-      <c r="D54" s="95" t="s">
-        <v>313</v>
+      <c r="C54" s="87" t="s">
+        <v>316</v>
+      </c>
+      <c r="D54" s="92" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="96">
+      <c r="C55" s="93">
         <v>4</v>
       </c>
-      <c r="D55" s="96" t="s">
-        <v>314</v>
+      <c r="D55" s="93" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="88" t="s">
-        <v>315</v>
-      </c>
-      <c r="D56" s="78" t="s">
-        <v>316</v>
+      <c r="C56" s="85" t="s">
+        <v>319</v>
+      </c>
+      <c r="D56" s="75" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="88" t="s">
-        <v>317</v>
-      </c>
-      <c r="D57" s="95" t="s">
-        <v>318</v>
+      <c r="C57" s="85" t="s">
+        <v>321</v>
+      </c>
+      <c r="D57" s="92" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="88" t="s">
-        <v>319</v>
-      </c>
-      <c r="D58" s="95" t="s">
-        <v>320</v>
+      <c r="C58" s="85" t="s">
+        <v>323</v>
+      </c>
+      <c r="D58" s="92" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="88" t="s">
-        <v>321</v>
-      </c>
-      <c r="D59" s="95" t="s">
-        <v>322</v>
+      <c r="C59" s="85" t="s">
+        <v>325</v>
+      </c>
+      <c r="D59" s="92" t="s">
+        <v>326</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="96">
+      <c r="C60" s="93">
         <v>5</v>
       </c>
-      <c r="D60" s="96" t="s">
-        <v>323</v>
+      <c r="D60" s="93" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="88" t="s">
-        <v>324</v>
-      </c>
-      <c r="D61" s="78" t="s">
-        <v>325</v>
+      <c r="C61" s="85" t="s">
+        <v>328</v>
+      </c>
+      <c r="D61" s="75" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="88" t="s">
-        <v>326</v>
-      </c>
-      <c r="D62" s="95" t="s">
-        <v>327</v>
+      <c r="C62" s="85" t="s">
+        <v>330</v>
+      </c>
+      <c r="D62" s="92" t="s">
+        <v>331</v>
       </c>
       <c r="F62" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="88" t="s">
-        <v>329</v>
-      </c>
-      <c r="D63" s="95" t="s">
-        <v>330</v>
+      <c r="C63" s="85" t="s">
+        <v>333</v>
+      </c>
+      <c r="D63" s="92" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="88" t="s">
-        <v>331</v>
-      </c>
-      <c r="D64" s="95" t="s">
-        <v>332</v>
+      <c r="C64" s="85" t="s">
+        <v>335</v>
+      </c>
+      <c r="D64" s="92" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="96">
+      <c r="C65" s="93">
         <v>6</v>
       </c>
-      <c r="D65" s="96" t="s">
-        <v>333</v>
+      <c r="D65" s="93" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="88" t="s">
-        <v>334</v>
-      </c>
-      <c r="D66" s="78" t="s">
-        <v>335</v>
+      <c r="C66" s="85" t="s">
+        <v>338</v>
+      </c>
+      <c r="D66" s="75" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="97" t="s">
-        <v>336</v>
-      </c>
-      <c r="D67" s="98" t="s">
-        <v>337</v>
+      <c r="C67" s="94" t="s">
+        <v>340</v>
+      </c>
+      <c r="D67" s="95" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="88" t="s">
-        <v>338</v>
-      </c>
-      <c r="D68" s="95" t="s">
-        <v>339</v>
+      <c r="C68" s="85" t="s">
+        <v>342</v>
+      </c>
+      <c r="D68" s="92" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="97" t="s">
-        <v>340</v>
-      </c>
-      <c r="D69" s="95" t="s">
-        <v>341</v>
+      <c r="C69" s="94" t="s">
+        <v>344</v>
+      </c>
+      <c r="D69" s="92" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="88" t="s">
-        <v>342</v>
-      </c>
-      <c r="D70" s="95" t="s">
-        <v>343</v>
+      <c r="C70" s="85" t="s">
+        <v>346</v>
+      </c>
+      <c r="D70" s="92" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="96">
+      <c r="C71" s="93">
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="88" t="s">
-        <v>345</v>
-      </c>
-      <c r="D72" s="78" t="s">
-        <v>346</v>
+      <c r="C72" s="85" t="s">
+        <v>349</v>
+      </c>
+      <c r="D72" s="75" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="96">
+      <c r="C73" s="93">
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="88" t="s">
-        <v>348</v>
-      </c>
-      <c r="D74" s="78" t="s">
-        <v>349</v>
+      <c r="C74" s="85" t="s">
+        <v>352</v>
+      </c>
+      <c r="D74" s="75" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="96">
+      <c r="C75" s="93">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="88" t="s">
-        <v>350</v>
-      </c>
-      <c r="D76" s="78" t="s">
-        <v>351</v>
+      <c r="C76" s="85" t="s">
+        <v>354</v>
+      </c>
+      <c r="D76" s="75" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="88" t="s">
-        <v>352</v>
-      </c>
-      <c r="D77" s="95" t="s">
-        <v>353</v>
+      <c r="C77" s="85" t="s">
+        <v>356</v>
+      </c>
+      <c r="D77" s="92" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="88" t="s">
-        <v>354</v>
-      </c>
-      <c r="D78" s="95" t="s">
-        <v>355</v>
+      <c r="C78" s="85" t="s">
+        <v>358</v>
+      </c>
+      <c r="D78" s="92" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="79">
-      <c r="C79" s="96">
+      <c r="C79" s="93">
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="88" t="s">
-        <v>357</v>
-      </c>
-      <c r="D80" s="78" t="s">
-        <v>358</v>
-      </c>
-      <c r="E80" s="82"/>
+      <c r="C80" s="85" t="s">
+        <v>361</v>
+      </c>
+      <c r="D80" s="75" t="s">
+        <v>362</v>
+      </c>
+      <c r="E80" s="79"/>
     </row>
     <row r="81">
-      <c r="C81" s="88" t="s">
-        <v>359</v>
-      </c>
-      <c r="D81" s="95" t="s">
-        <v>360</v>
+      <c r="C81" s="85" t="s">
+        <v>363</v>
+      </c>
+      <c r="D81" s="92" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="96">
+      <c r="C82" s="93">
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="88" t="s">
-        <v>362</v>
-      </c>
-      <c r="D83" s="78" t="s">
-        <v>363</v>
+      <c r="C83" s="85" t="s">
+        <v>366</v>
+      </c>
+      <c r="D83" s="75" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="84">
-      <c r="C84" s="88" t="s">
-        <v>364</v>
-      </c>
-      <c r="D84" s="78" t="s">
-        <v>365</v>
+      <c r="C84" s="85" t="s">
+        <v>368</v>
+      </c>
+      <c r="D84" s="75" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calibrage Z OK ? + Step machine récupère CD, aiamnt, déplace...+ Ajout gestion fhciier data et positions : si pas de fichier on créé un nouveau, sinon on prend elui actuel
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -242,7 +242,14 @@
   </si>
   <si>
     <t xml:space="preserve">-Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
-   - Menu calibrage !</t>
+   - Menu calibrage !
+comment ça marche ? Dans le sens si on lui va a X degrés, ccela correspond tjrs à la meme position
+- Calibrage origine ? Calibrage cd, Calibrage Lecteur
+Sauvegarder kes données avex X e Y
+les récupérers dans le fichiers quand besoin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A TESTER</t>
   </si>
   <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
@@ -271,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tous les cd se refresh quand on dragNdrop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIEN PLACER STEP MOTEUR POUR STEP 0 TOUT EN HAUT (ORIGINE)</t>
   </si>
   <si>
     <t xml:space="preserve">Construire machine</t>
@@ -1706,7 +1716,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="98">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1772,8 +1782,14 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
@@ -2756,8 +2772,8 @@
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="14">
-        <f>SUM(D14:D22)/9</f>
-        <v>0.76666666666666672</v>
+        <f>SUM(D14:D23)/10</f>
+        <v>0.89000000000000001</v>
       </c>
       <c r="F13" s="15" t="s">
         <v>22</v>
@@ -3066,7 +3082,7 @@
       </c>
       <c r="C21" s="35"/>
       <c r="D21" s="36">
-        <v>0.90000000000000002</v>
+        <v>1</v>
       </c>
       <c r="F21" t="s">
         <v>65</v>
@@ -3096,37 +3112,39 @@
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" ht="42.75">
+    <row r="22" ht="114">
       <c r="A22" s="1"/>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="35"/>
+      <c r="C22" s="38" t="s">
+        <v>69</v>
+      </c>
       <c r="D22" s="33">
-        <v>0</v>
+        <v>0.90000000000000002</v>
       </c>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M22" s="34" t="s">
         <v>63</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3134,7 +3152,7 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
@@ -3142,15 +3160,17 @@
     <row r="23" ht="42.75">
       <c r="A23" s="1"/>
       <c r="B23" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D23" s="33"/>
+        <v>75</v>
+      </c>
+      <c r="D23" s="28">
+        <v>1</v>
+      </c>
       <c r="H23" s="1"/>
-      <c r="I23" s="37"/>
-      <c r="J23" s="37"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="M23" s="34" t="s">
         <v>63</v>
@@ -3159,36 +3179,39 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
     </row>
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
+      <c r="B24" s="5" t="s">
+        <v>79</v>
+      </c>
       <c r="D24" s="33"/>
-      <c r="F24" s="38" t="s">
-        <v>78</v>
+      <c r="F24" s="40" t="s">
+        <v>80</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="39"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="43"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3203,6 +3226,7 @@
     </row>
     <row r="25" ht="16.5">
       <c r="A25" s="1"/>
+      <c r="B25" s="5"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -3222,11 +3246,11 @@
     </row>
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="42" t="s">
-        <v>81</v>
-      </c>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44">
+      <c r="B26" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="45"/>
+      <c r="D26" s="46">
         <f>SUM(D27:D32)/5</f>
         <v>0</v>
       </c>
@@ -3240,10 +3264,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3256,10 +3280,10 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D27" s="33">
         <v>0</v>
@@ -3273,7 +3297,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3281,7 +3305,7 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D28" s="33">
         <v>0</v>
@@ -3297,7 +3321,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3305,7 +3329,7 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D29" s="33">
         <v>0</v>
@@ -3325,10 +3349,10 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D30" s="33">
         <v>0</v>
@@ -3349,10 +3373,10 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D31" s="33">
         <v>0</v>
@@ -3371,13 +3395,13 @@
     <row r="32" ht="28.5">
       <c r="A32" s="1"/>
       <c r="B32" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D32" s="33">
         <v>0</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3387,7 +3411,7 @@
       <c r="B33" s="4"/>
       <c r="D33" s="33"/>
       <c r="L33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3428,11 +3452,11 @@
     </row>
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
-      <c r="B36" s="45" t="s">
-        <v>97</v>
-      </c>
-      <c r="C36" s="43"/>
-      <c r="D36" s="44">
+      <c r="B36" s="47" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" s="45"/>
+      <c r="D36" s="46">
         <f>SUM(D37:D40)/4</f>
         <v>0</v>
       </c>
@@ -3450,10 +3474,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D37" s="33">
         <v>0</v>
@@ -3472,10 +3496,10 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D38" s="33">
         <v>0</v>
@@ -3494,10 +3518,10 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D39" s="33">
         <v>0</v>
@@ -3506,10 +3530,10 @@
     <row r="40" ht="28.5">
       <c r="A40" s="1"/>
       <c r="B40" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D40" s="33">
         <v>0</v>
@@ -3521,7 +3545,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3529,7 +3553,7 @@
     <row r="43" ht="16.5">
       <c r="A43" s="1"/>
       <c r="B43" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -3540,7 +3564,7 @@
     <row r="45" ht="16.5">
       <c r="A45" s="1"/>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" ht="14.25">
@@ -3552,7 +3576,7 @@
     <row r="48" ht="14.25">
       <c r="A48" s="1"/>
       <c r="B48" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49" ht="14.25">
@@ -3561,13 +3585,13 @@
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="51" ht="14.25">
       <c r="A51" s="1"/>
       <c r="B51" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" ht="16.5">
@@ -3579,7 +3603,7 @@
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3595,7 +3619,7 @@
     <row r="55" ht="16.5">
       <c r="A55" s="1"/>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -3624,7 +3648,7 @@
     <row r="57" ht="16.5">
       <c r="A57" s="1"/>
       <c r="B57" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -3652,52 +3676,52 @@
     </row>
     <row r="69" ht="14.25">
       <c r="B69" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="78" ht="14.25">
       <c r="B78" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C78" t="s">
         <v>67</v>
@@ -3727,16 +3751,16 @@
   </cols>
   <sheetData>
     <row r="2" ht="14.25">
-      <c r="B2" s="46" t="s">
-        <v>125</v>
+      <c r="B2" s="48" t="s">
+        <v>127</v>
       </c>
       <c r="C2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" ht="14.25">
       <c r="B3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3759,280 +3783,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="47" t="s">
-        <v>128</v>
-      </c>
-      <c r="G2" s="48" t="s">
-        <v>129</v>
+      <c r="F2" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="50" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="3">
-      <c r="F3" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="G3" s="50" t="s">
-        <v>131</v>
+      <c r="F3" s="51" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" s="52" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="4">
-      <c r="F4" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="G4" s="52" t="s">
-        <v>133</v>
+      <c r="F4" s="53" t="s">
+        <v>134</v>
+      </c>
+      <c r="G4" s="54" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="F5" s="53" t="s">
-        <v>134</v>
-      </c>
-      <c r="G5" s="54" t="s">
-        <v>135</v>
+      <c r="F5" s="55" t="s">
+        <v>136</v>
+      </c>
+      <c r="G5" s="56" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="F6" s="55"/>
-      <c r="G6" s="56" t="s">
-        <v>136</v>
+      <c r="F6" s="57"/>
+      <c r="G6" s="58" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="F7" s="55"/>
-      <c r="G7" s="56" t="s">
-        <v>137</v>
+      <c r="F7" s="57"/>
+      <c r="G7" s="58" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="F8" s="55"/>
-      <c r="G8" s="56" t="s">
-        <v>138</v>
+      <c r="F8" s="57"/>
+      <c r="G8" s="58" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" s="55"/>
-      <c r="G9" s="56" t="s">
-        <v>140</v>
+        <v>141</v>
+      </c>
+      <c r="F9" s="57"/>
+      <c r="G9" s="58" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
-        <v>141</v>
-      </c>
-      <c r="C10" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="F10" s="55"/>
-      <c r="G10" s="56" t="s">
         <v>143</v>
       </c>
+      <c r="C10" s="59" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="57"/>
+      <c r="G10" s="58" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="11" ht="15">
-      <c r="C11" s="58" t="s">
-        <v>144</v>
-      </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="56" t="s">
-        <v>145</v>
+      <c r="C11" s="60" t="s">
+        <v>146</v>
+      </c>
+      <c r="F11" s="57"/>
+      <c r="G11" s="58" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="C12" s="57" t="s">
-        <v>146</v>
-      </c>
-      <c r="F12" s="49"/>
-      <c r="G12" s="59" t="s">
-        <v>147</v>
+      <c r="C12" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="F12" s="51"/>
+      <c r="G12" s="61" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="13" ht="15">
-      <c r="C13" s="58" t="s">
-        <v>148</v>
-      </c>
-      <c r="F13" s="51" t="s">
-        <v>149</v>
-      </c>
-      <c r="G13" s="60" t="s">
+      <c r="C13" s="60" t="s">
         <v>150</v>
       </c>
+      <c r="F13" s="53" t="s">
+        <v>151</v>
+      </c>
+      <c r="G13" s="62" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="14" ht="15">
-      <c r="C14" s="57" t="s">
-        <v>151</v>
-      </c>
-      <c r="F14" s="61" t="s">
-        <v>152</v>
-      </c>
-      <c r="G14" s="62" t="s">
+      <c r="C14" s="59" t="s">
         <v>153</v>
       </c>
+      <c r="F14" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="64" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="15">
-      <c r="C15" s="58" t="s">
-        <v>154</v>
-      </c>
-      <c r="F15" s="63" t="s">
-        <v>155</v>
-      </c>
-      <c r="G15" s="64" t="s">
+      <c r="C15" s="60" t="s">
         <v>156</v>
       </c>
+      <c r="F15" s="65" t="s">
+        <v>157</v>
+      </c>
+      <c r="G15" s="66" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="16">
-      <c r="C16" s="58" t="s">
-        <v>157</v>
-      </c>
-      <c r="F16" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="G16" s="66" t="s">
+      <c r="C16" s="60" t="s">
         <v>159</v>
       </c>
+      <c r="F16" s="67" t="s">
+        <v>160</v>
+      </c>
+      <c r="G16" s="68" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="17">
-      <c r="C17" s="57" t="s">
-        <v>160</v>
-      </c>
-      <c r="F17" s="65"/>
-      <c r="G17" s="66" t="s">
-        <v>161</v>
+      <c r="C17" s="59" t="s">
+        <v>162</v>
+      </c>
+      <c r="F17" s="67"/>
+      <c r="G17" s="68" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="58" t="s">
-        <v>162</v>
-      </c>
-      <c r="F18" s="65"/>
-      <c r="G18" s="66" t="s">
-        <v>163</v>
+      <c r="C18" s="60" t="s">
+        <v>164</v>
+      </c>
+      <c r="F18" s="67"/>
+      <c r="G18" s="68" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="58" t="s">
-        <v>164</v>
-      </c>
-      <c r="F19" s="65"/>
-      <c r="G19" s="66" t="s">
-        <v>165</v>
+      <c r="C19" s="60" t="s">
+        <v>166</v>
+      </c>
+      <c r="F19" s="67"/>
+      <c r="G19" s="68" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="58" t="s">
-        <v>166</v>
-      </c>
-      <c r="F20" s="65"/>
-      <c r="G20" s="66" t="s">
-        <v>167</v>
+      <c r="C20" s="60" t="s">
+        <v>168</v>
+      </c>
+      <c r="F20" s="67"/>
+      <c r="G20" s="68" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="58" t="s">
-        <v>168</v>
-      </c>
-      <c r="F21" s="65"/>
-      <c r="G21" s="66" t="s">
-        <v>169</v>
+      <c r="C21" s="60" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" s="67"/>
+      <c r="G21" s="68" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="57" t="s">
-        <v>170</v>
-      </c>
-      <c r="F22" s="65"/>
-      <c r="G22" s="66" t="s">
-        <v>171</v>
+      <c r="C22" s="59" t="s">
+        <v>172</v>
+      </c>
+      <c r="F22" s="67"/>
+      <c r="G22" s="68" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="58" t="s">
-        <v>172</v>
-      </c>
-      <c r="F23" s="65"/>
-      <c r="G23" s="66" t="s">
-        <v>173</v>
+      <c r="C23" s="60" t="s">
+        <v>174</v>
+      </c>
+      <c r="F23" s="67"/>
+      <c r="G23" s="68" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="57" t="s">
-        <v>174</v>
-      </c>
-      <c r="F24" s="65"/>
-      <c r="G24" s="66" t="s">
-        <v>175</v>
+      <c r="C24" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="F24" s="67"/>
+      <c r="G24" s="68" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="58" t="s">
-        <v>176</v>
-      </c>
-      <c r="F25" s="65"/>
-      <c r="G25" s="66" t="s">
-        <v>177</v>
+      <c r="C25" s="60" t="s">
+        <v>178</v>
+      </c>
+      <c r="F25" s="67"/>
+      <c r="G25" s="68" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="26">
-      <c r="F26" s="65"/>
-      <c r="G26" s="66" t="s">
-        <v>178</v>
+      <c r="F26" s="67"/>
+      <c r="G26" s="68" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="65"/>
-      <c r="G27" s="66"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="68"/>
     </row>
     <row r="28">
-      <c r="F28" s="65"/>
-      <c r="G28" s="66" t="s">
-        <v>179</v>
+      <c r="F28" s="67"/>
+      <c r="G28" s="68" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="65"/>
-      <c r="G29" s="66" t="s">
-        <v>180</v>
+      <c r="F29" s="67"/>
+      <c r="G29" s="68" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="67"/>
-      <c r="F30" s="65"/>
-      <c r="G30" s="66" t="s">
-        <v>181</v>
+      <c r="C30" s="69"/>
+      <c r="F30" s="67"/>
+      <c r="G30" s="68" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="65"/>
-      <c r="G31" s="68" t="s">
-        <v>182</v>
+      <c r="F31" s="67"/>
+      <c r="G31" s="70" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="61" t="s">
-        <v>183</v>
-      </c>
-      <c r="G32" s="69" t="s">
-        <v>184</v>
+      <c r="F32" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="G32" s="71" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="58"/>
+      <c r="C33" s="60"/>
     </row>
     <row r="34">
-      <c r="C34" s="58"/>
+      <c r="C34" s="60"/>
     </row>
     <row r="36">
-      <c r="C36" s="67"/>
+      <c r="C36" s="69"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="58"/>
+      <c r="C39" s="60"/>
     </row>
     <row r="40">
-      <c r="C40" s="58"/>
+      <c r="C40" s="60"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -4060,367 +4084,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D5" s="70" t="s">
-        <v>187</v>
+        <v>188</v>
+      </c>
+      <c r="D5" s="72" t="s">
+        <v>189</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="H5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="K5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B6" t="s">
-        <v>194</v>
-      </c>
-      <c r="D6" s="71" t="s">
-        <v>195</v>
+        <v>196</v>
+      </c>
+      <c r="D6" s="73" t="s">
+        <v>197</v>
       </c>
       <c r="E6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G6" t="s">
-        <v>198</v>
-      </c>
-      <c r="H6" s="72" t="s">
-        <v>199</v>
+        <v>200</v>
+      </c>
+      <c r="H6" s="74" t="s">
+        <v>201</v>
       </c>
       <c r="I6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="J6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="K6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>194</v>
-      </c>
-      <c r="D7" s="73" t="s">
-        <v>204</v>
+        <v>196</v>
+      </c>
+      <c r="D7" s="75" t="s">
+        <v>206</v>
       </c>
       <c r="F7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G7" t="s">
-        <v>206</v>
-      </c>
-      <c r="H7" s="72" t="s">
-        <v>207</v>
+        <v>208</v>
+      </c>
+      <c r="H7" s="74" t="s">
+        <v>209</v>
       </c>
       <c r="K7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="71" t="s">
-        <v>209</v>
-      </c>
-      <c r="G8" s="74" t="s">
-        <v>210</v>
-      </c>
-      <c r="H8" s="72" t="s">
+      <c r="D8" s="73" t="s">
         <v>211</v>
+      </c>
+      <c r="G8" s="76" t="s">
+        <v>212</v>
+      </c>
+      <c r="H8" s="74" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B9" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="H9" s="72" t="s">
         <v>215</v>
+      </c>
+      <c r="D9" s="75" t="s">
+        <v>216</v>
+      </c>
+      <c r="H9" s="74" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B10" t="s">
-        <v>217</v>
-      </c>
-      <c r="D10" s="71"/>
+        <v>219</v>
+      </c>
+      <c r="D10" s="73"/>
       <c r="G10" t="s">
-        <v>218</v>
-      </c>
-      <c r="H10" s="72" t="s">
-        <v>219</v>
+        <v>220</v>
+      </c>
+      <c r="H10" s="74" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B11" t="s">
-        <v>221</v>
-      </c>
-      <c r="D11" s="73" t="s">
-        <v>222</v>
-      </c>
-      <c r="G11" s="74" t="s">
         <v>223</v>
       </c>
-      <c r="H11" s="72" t="s">
+      <c r="D11" s="75" t="s">
         <v>224</v>
+      </c>
+      <c r="G11" s="76" t="s">
+        <v>225</v>
+      </c>
+      <c r="H11" s="74" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B12" t="s">
-        <v>226</v>
-      </c>
-      <c r="D12" s="71" t="s">
-        <v>227</v>
-      </c>
-      <c r="G12" s="74" t="s">
         <v>228</v>
       </c>
-      <c r="H12" s="72" t="s">
+      <c r="D12" s="73" t="s">
         <v>229</v>
+      </c>
+      <c r="G12" s="76" t="s">
+        <v>230</v>
+      </c>
+      <c r="H12" s="74" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B13" t="s">
-        <v>231</v>
-      </c>
-      <c r="D13" s="73" t="s">
-        <v>232</v>
-      </c>
-      <c r="G13" s="74" t="s">
         <v>233</v>
       </c>
+      <c r="D13" s="75" t="s">
+        <v>234</v>
+      </c>
+      <c r="G13" s="76" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="14">
-      <c r="D14" s="71" t="s">
-        <v>234</v>
+      <c r="D14" s="73" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B15" t="s">
-        <v>236</v>
-      </c>
-      <c r="D15" s="73"/>
+        <v>238</v>
+      </c>
+      <c r="D15" s="75"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B16" t="s">
-        <v>238</v>
-      </c>
-      <c r="D16" s="71"/>
+        <v>240</v>
+      </c>
+      <c r="D16" s="73"/>
       <c r="G16" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="73"/>
-      <c r="G17" s="74" t="s">
-        <v>240</v>
+      <c r="D17" s="75"/>
+      <c r="G17" s="76" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>241</v>
-      </c>
-      <c r="D18" s="71"/>
-      <c r="G18" s="75" t="s">
-        <v>242</v>
+        <v>243</v>
+      </c>
+      <c r="D18" s="73"/>
+      <c r="G18" s="77" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="73" t="s">
-        <v>243</v>
+      <c r="D19" s="75" t="s">
+        <v>245</v>
       </c>
       <c r="E19" t="s">
-        <v>244</v>
-      </c>
-      <c r="G19" s="75" t="s">
-        <v>245</v>
+        <v>246</v>
+      </c>
+      <c r="G19" s="77" t="s">
+        <v>247</v>
       </c>
       <c r="H19" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="I19" t="s">
+        <v>249</v>
+      </c>
+      <c r="J19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="73"/>
+      <c r="G20" s="77" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="73"/>
+      <c r="G22" s="77" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="76"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="73"/>
+      <c r="G24" s="76" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="77" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="73"/>
+      <c r="G26" s="77" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="77" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="73"/>
+      <c r="G28" s="77" t="s">
         <v>247</v>
       </c>
-      <c r="J19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="71"/>
-      <c r="G20" s="75" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="71"/>
-      <c r="G22" s="75" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="G23" s="74"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="71"/>
-      <c r="G24" s="74" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" s="75" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" s="71"/>
-      <c r="G26" s="75" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="75" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="71"/>
-      <c r="G28" s="75" t="s">
-        <v>245</v>
-      </c>
     </row>
     <row r="35">
-      <c r="D35" s="76" t="s">
-        <v>253</v>
+      <c r="D35" s="78" t="s">
+        <v>255</v>
       </c>
       <c r="E35" t="s">
-        <v>254</v>
-      </c>
-      <c r="F35" s="77" t="s">
-        <v>255</v>
+        <v>256</v>
+      </c>
+      <c r="F35" s="79" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="36">
-      <c r="D36" s="78" t="s">
-        <v>256</v>
+      <c r="D36" s="80" t="s">
+        <v>258</v>
       </c>
       <c r="E36" t="s">
-        <v>257</v>
-      </c>
-      <c r="F36" s="78" t="s">
-        <v>258</v>
+        <v>259</v>
+      </c>
+      <c r="F36" s="80" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="37">
-      <c r="D37" s="77" t="s">
-        <v>259</v>
+      <c r="D37" s="79" t="s">
+        <v>261</v>
       </c>
       <c r="E37" t="s">
-        <v>260</v>
-      </c>
-      <c r="F37" s="77" t="s">
-        <v>261</v>
+        <v>262</v>
+      </c>
+      <c r="F37" s="79" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="78" t="s">
-        <v>262</v>
+      <c r="D38" s="80" t="s">
+        <v>264</v>
       </c>
       <c r="E38" t="s">
-        <v>263</v>
-      </c>
-      <c r="F38" s="78" t="s">
-        <v>264</v>
+        <v>265</v>
+      </c>
+      <c r="F38" s="80" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="39">
-      <c r="D39" s="77" t="s">
-        <v>265</v>
+      <c r="D39" s="79" t="s">
+        <v>267</v>
       </c>
       <c r="E39" t="s">
-        <v>266</v>
-      </c>
-      <c r="F39" s="77" t="s">
-        <v>267</v>
+        <v>268</v>
+      </c>
+      <c r="F39" s="79" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>257</v>
-      </c>
-      <c r="F40" s="78" t="s">
-        <v>268</v>
+        <v>259</v>
+      </c>
+      <c r="F40" s="80" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>260</v>
-      </c>
-      <c r="F41" s="77" t="s">
-        <v>269</v>
+        <v>262</v>
+      </c>
+      <c r="F41" s="79" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -4451,564 +4475,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="79" t="s">
-        <v>272</v>
+      <c r="D4" s="81" t="s">
+        <v>274</v>
       </c>
       <c r="E4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
-        <v>274</v>
-      </c>
-      <c r="E5" s="79">
+        <v>276</v>
+      </c>
+      <c r="E5" s="81">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="75" t="s">
+      <c r="D6" s="77" t="s">
+        <v>277</v>
+      </c>
+      <c r="E6" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="82" t="s">
+        <v>278</v>
+      </c>
+      <c r="E7" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="77" t="s">
+        <v>279</v>
+      </c>
+      <c r="E8" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="77"/>
+      <c r="E9" s="81"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="74" t="s">
+        <v>280</v>
+      </c>
+      <c r="E10" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="77" t="s">
+        <v>281</v>
+      </c>
+      <c r="E11" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="77" t="s">
+        <v>282</v>
+      </c>
+      <c r="E12" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="77" t="s">
+        <v>283</v>
+      </c>
+      <c r="E13" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="74" t="s">
+        <v>284</v>
+      </c>
+      <c r="E15" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="83" t="s">
+        <v>285</v>
+      </c>
+      <c r="E16" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="84" t="s">
+        <v>286</v>
+      </c>
+      <c r="E17" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="84" t="s">
+        <v>287</v>
+      </c>
+      <c r="E18" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="77"/>
+      <c r="E19" s="77"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="74" t="s">
+        <v>288</v>
+      </c>
+      <c r="E20" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" s="74" t="s">
+        <v>289</v>
+      </c>
+      <c r="E21" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="85"/>
+      <c r="E23" s="77"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="77"/>
+      <c r="E24" s="77"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="77"/>
+      <c r="E25" s="77"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="77"/>
+      <c r="E26" s="77"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="77"/>
+      <c r="E27" s="77"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="77"/>
+      <c r="E28" s="77"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="77"/>
+      <c r="E29" s="77"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="86"/>
+      <c r="C39" s="87" t="s">
+        <v>290</v>
+      </c>
+      <c r="D39" s="87" t="s">
+        <v>291</v>
+      </c>
+      <c r="E39" t="s">
         <v>275</v>
-      </c>
-      <c r="E6" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" s="80" t="s">
-        <v>276</v>
-      </c>
-      <c r="E7" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="75" t="s">
-        <v>277</v>
-      </c>
-      <c r="E8" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="75"/>
-      <c r="E9" s="79"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="72" t="s">
-        <v>278</v>
-      </c>
-      <c r="E10" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" s="75" t="s">
-        <v>279</v>
-      </c>
-      <c r="E11" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="75" t="s">
-        <v>280</v>
-      </c>
-      <c r="E12" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="75" t="s">
-        <v>281</v>
-      </c>
-      <c r="E13" s="79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="75"/>
-      <c r="E14" s="75"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="72" t="s">
-        <v>282</v>
-      </c>
-      <c r="E15" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="81" t="s">
-        <v>283</v>
-      </c>
-      <c r="E16" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="82" t="s">
-        <v>284</v>
-      </c>
-      <c r="E17" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" s="82" t="s">
-        <v>285</v>
-      </c>
-      <c r="E18" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="75"/>
-      <c r="E19" s="75"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="72" t="s">
-        <v>286</v>
-      </c>
-      <c r="E20" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" s="72" t="s">
-        <v>287</v>
-      </c>
-      <c r="E21" s="79">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="75"/>
-      <c r="E22" s="75"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="83"/>
-      <c r="E23" s="75"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="75"/>
-      <c r="E24" s="75"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="75"/>
-      <c r="E25" s="75"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="75"/>
-      <c r="E26" s="75"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="75"/>
-      <c r="E27" s="75"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="75"/>
-      <c r="E28" s="75"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="75"/>
-      <c r="E29" s="75"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="75"/>
-      <c r="E30" s="75"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="84"/>
-      <c r="C39" s="85" t="s">
-        <v>288</v>
-      </c>
-      <c r="D39" s="85" t="s">
-        <v>289</v>
-      </c>
-      <c r="E39" t="s">
-        <v>273</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="86">
+      <c r="C40" s="88">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="E40" s="79"/>
+        <v>292</v>
+      </c>
+      <c r="E40" s="81"/>
     </row>
     <row r="41">
-      <c r="C41" s="79" t="s">
-        <v>291</v>
-      </c>
-      <c r="D41" s="75" t="s">
-        <v>292</v>
-      </c>
-      <c r="E41" s="79"/>
+      <c r="C41" s="81" t="s">
+        <v>293</v>
+      </c>
+      <c r="D41" s="77" t="s">
+        <v>294</v>
+      </c>
+      <c r="E41" s="81"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="79" t="s">
-        <v>293</v>
-      </c>
-      <c r="D42" s="75" t="s">
-        <v>294</v>
+      <c r="C42" s="81" t="s">
+        <v>295</v>
+      </c>
+      <c r="D42" s="77" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="79" t="s">
-        <v>295</v>
-      </c>
-      <c r="D43" s="75" t="s">
-        <v>296</v>
+      <c r="C43" s="81" t="s">
+        <v>297</v>
+      </c>
+      <c r="D43" s="77" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="87" t="s">
-        <v>297</v>
-      </c>
-      <c r="D44" s="80" t="s">
-        <v>298</v>
-      </c>
-      <c r="E44" s="88"/>
-      <c r="F44" s="88"/>
+      <c r="C44" s="89" t="s">
+        <v>299</v>
+      </c>
+      <c r="D44" s="82" t="s">
+        <v>300</v>
+      </c>
+      <c r="E44" s="90"/>
+      <c r="F44" s="90"/>
     </row>
     <row r="45">
-      <c r="C45" s="85" t="s">
-        <v>299</v>
-      </c>
-      <c r="D45" s="75" t="s">
-        <v>300</v>
-      </c>
-      <c r="E45" s="79"/>
+      <c r="C45" s="87" t="s">
+        <v>301</v>
+      </c>
+      <c r="D45" s="77" t="s">
+        <v>302</v>
+      </c>
+      <c r="E45" s="81"/>
     </row>
     <row r="46">
-      <c r="C46" s="85" t="s">
-        <v>301</v>
-      </c>
-      <c r="D46" s="75" t="s">
-        <v>302</v>
-      </c>
-      <c r="E46" s="79"/>
+      <c r="C46" s="87" t="s">
+        <v>303</v>
+      </c>
+      <c r="D46" s="77" t="s">
+        <v>304</v>
+      </c>
+      <c r="E46" s="81"/>
     </row>
     <row r="47">
-      <c r="C47" s="89">
+      <c r="C47" s="91">
         <v>2</v>
       </c>
-      <c r="D47" s="90" t="s">
-        <v>303</v>
-      </c>
-      <c r="E47" s="79"/>
+      <c r="D47" s="92" t="s">
+        <v>305</v>
+      </c>
+      <c r="E47" s="81"/>
     </row>
     <row r="48">
-      <c r="C48" s="87" t="s">
-        <v>304</v>
-      </c>
-      <c r="D48" s="80" t="s">
-        <v>305</v>
-      </c>
-      <c r="E48" s="79"/>
+      <c r="C48" s="89" t="s">
+        <v>306</v>
+      </c>
+      <c r="D48" s="82" t="s">
+        <v>307</v>
+      </c>
+      <c r="E48" s="81"/>
     </row>
     <row r="49">
-      <c r="C49" s="86">
+      <c r="C49" s="88">
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="E49" s="79"/>
+        <v>308</v>
+      </c>
+      <c r="E49" s="81"/>
     </row>
     <row r="50">
-      <c r="C50" s="87" t="s">
-        <v>307</v>
-      </c>
-      <c r="D50" s="80" t="s">
-        <v>308</v>
-      </c>
-      <c r="F50" s="91" t="s">
+      <c r="C50" s="89" t="s">
         <v>309</v>
       </c>
+      <c r="D50" s="82" t="s">
+        <v>310</v>
+      </c>
+      <c r="F50" s="93" t="s">
+        <v>311</v>
+      </c>
     </row>
     <row r="51">
-      <c r="C51" s="87" t="s">
-        <v>310</v>
-      </c>
-      <c r="D51" s="92" t="s">
-        <v>311</v>
+      <c r="C51" s="89" t="s">
+        <v>312</v>
+      </c>
+      <c r="D51" s="94" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="87" t="s">
-        <v>312</v>
-      </c>
-      <c r="D52" s="92" t="s">
-        <v>313</v>
+      <c r="C52" s="89" t="s">
+        <v>314</v>
+      </c>
+      <c r="D52" s="94" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="87" t="s">
-        <v>314</v>
-      </c>
-      <c r="D53" s="92" t="s">
-        <v>315</v>
+      <c r="C53" s="89" t="s">
+        <v>316</v>
+      </c>
+      <c r="D53" s="94" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="87" t="s">
-        <v>316</v>
-      </c>
-      <c r="D54" s="92" t="s">
-        <v>317</v>
+      <c r="C54" s="89" t="s">
+        <v>318</v>
+      </c>
+      <c r="D54" s="94" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="93">
+      <c r="C55" s="95">
         <v>4</v>
       </c>
-      <c r="D55" s="93" t="s">
-        <v>318</v>
+      <c r="D55" s="95" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="85" t="s">
-        <v>319</v>
-      </c>
-      <c r="D56" s="75" t="s">
-        <v>320</v>
+      <c r="C56" s="87" t="s">
+        <v>321</v>
+      </c>
+      <c r="D56" s="77" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="85" t="s">
-        <v>321</v>
-      </c>
-      <c r="D57" s="92" t="s">
-        <v>322</v>
+      <c r="C57" s="87" t="s">
+        <v>323</v>
+      </c>
+      <c r="D57" s="94" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="85" t="s">
-        <v>323</v>
-      </c>
-      <c r="D58" s="92" t="s">
-        <v>324</v>
+      <c r="C58" s="87" t="s">
+        <v>325</v>
+      </c>
+      <c r="D58" s="94" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="85" t="s">
-        <v>325</v>
-      </c>
-      <c r="D59" s="92" t="s">
-        <v>326</v>
+      <c r="C59" s="87" t="s">
+        <v>327</v>
+      </c>
+      <c r="D59" s="94" t="s">
+        <v>328</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="93">
+      <c r="C60" s="95">
         <v>5</v>
       </c>
-      <c r="D60" s="93" t="s">
-        <v>327</v>
+      <c r="D60" s="95" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="85" t="s">
-        <v>328</v>
-      </c>
-      <c r="D61" s="75" t="s">
-        <v>329</v>
+      <c r="C61" s="87" t="s">
+        <v>330</v>
+      </c>
+      <c r="D61" s="77" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="85" t="s">
-        <v>330</v>
-      </c>
-      <c r="D62" s="92" t="s">
-        <v>331</v>
+      <c r="C62" s="87" t="s">
+        <v>332</v>
+      </c>
+      <c r="D62" s="94" t="s">
+        <v>333</v>
       </c>
       <c r="F62" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="85" t="s">
-        <v>333</v>
-      </c>
-      <c r="D63" s="92" t="s">
-        <v>334</v>
+      <c r="C63" s="87" t="s">
+        <v>335</v>
+      </c>
+      <c r="D63" s="94" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="85" t="s">
-        <v>335</v>
-      </c>
-      <c r="D64" s="92" t="s">
-        <v>336</v>
+      <c r="C64" s="87" t="s">
+        <v>337</v>
+      </c>
+      <c r="D64" s="94" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="93">
+      <c r="C65" s="95">
         <v>6</v>
       </c>
-      <c r="D65" s="93" t="s">
-        <v>337</v>
+      <c r="D65" s="95" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="85" t="s">
-        <v>338</v>
-      </c>
-      <c r="D66" s="75" t="s">
-        <v>339</v>
+      <c r="C66" s="87" t="s">
+        <v>340</v>
+      </c>
+      <c r="D66" s="77" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="94" t="s">
-        <v>340</v>
-      </c>
-      <c r="D67" s="95" t="s">
-        <v>341</v>
+      <c r="C67" s="96" t="s">
+        <v>342</v>
+      </c>
+      <c r="D67" s="97" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="85" t="s">
-        <v>342</v>
-      </c>
-      <c r="D68" s="92" t="s">
-        <v>343</v>
+      <c r="C68" s="87" t="s">
+        <v>344</v>
+      </c>
+      <c r="D68" s="94" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="94" t="s">
-        <v>344</v>
-      </c>
-      <c r="D69" s="92" t="s">
-        <v>345</v>
+      <c r="C69" s="96" t="s">
+        <v>346</v>
+      </c>
+      <c r="D69" s="94" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="85" t="s">
-        <v>346</v>
-      </c>
-      <c r="D70" s="92" t="s">
-        <v>347</v>
+      <c r="C70" s="87" t="s">
+        <v>348</v>
+      </c>
+      <c r="D70" s="94" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="93">
+      <c r="C71" s="95">
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="85" t="s">
-        <v>349</v>
-      </c>
-      <c r="D72" s="75" t="s">
-        <v>350</v>
+      <c r="C72" s="87" t="s">
+        <v>351</v>
+      </c>
+      <c r="D72" s="77" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="93">
+      <c r="C73" s="95">
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="85" t="s">
-        <v>352</v>
-      </c>
-      <c r="D74" s="75" t="s">
-        <v>353</v>
+      <c r="C74" s="87" t="s">
+        <v>354</v>
+      </c>
+      <c r="D74" s="77" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="93">
+      <c r="C75" s="95">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="85" t="s">
-        <v>354</v>
-      </c>
-      <c r="D76" s="75" t="s">
-        <v>355</v>
+      <c r="C76" s="87" t="s">
+        <v>356</v>
+      </c>
+      <c r="D76" s="77" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="85" t="s">
-        <v>356</v>
-      </c>
-      <c r="D77" s="92" t="s">
-        <v>357</v>
+      <c r="C77" s="87" t="s">
+        <v>358</v>
+      </c>
+      <c r="D77" s="94" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="85" t="s">
-        <v>358</v>
-      </c>
-      <c r="D78" s="92" t="s">
-        <v>359</v>
+      <c r="C78" s="87" t="s">
+        <v>360</v>
+      </c>
+      <c r="D78" s="94" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="79">
-      <c r="C79" s="93">
+      <c r="C79" s="95">
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="85" t="s">
-        <v>361</v>
-      </c>
-      <c r="D80" s="75" t="s">
-        <v>362</v>
-      </c>
-      <c r="E80" s="79"/>
+      <c r="C80" s="87" t="s">
+        <v>363</v>
+      </c>
+      <c r="D80" s="77" t="s">
+        <v>364</v>
+      </c>
+      <c r="E80" s="81"/>
     </row>
     <row r="81">
-      <c r="C81" s="85" t="s">
-        <v>363</v>
-      </c>
-      <c r="D81" s="92" t="s">
-        <v>364</v>
+      <c r="C81" s="87" t="s">
+        <v>365</v>
+      </c>
+      <c r="D81" s="94" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="93">
+      <c r="C82" s="95">
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="85" t="s">
-        <v>366</v>
-      </c>
-      <c r="D83" s="75" t="s">
-        <v>367</v>
+      <c r="C83" s="87" t="s">
+        <v>368</v>
+      </c>
+      <c r="D83" s="77" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="84">
-      <c r="C84" s="85" t="s">
-        <v>368</v>
-      </c>
-      <c r="D84" s="75" t="s">
-        <v>369</v>
+      <c r="C84" s="87" t="s">
+        <v>370</v>
+      </c>
+      <c r="D84" s="77" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: les pas retour sur un bord sont décrémenters
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -249,7 +249,7 @@
 les récupérers dans le fichiers quand besoin</t>
   </si>
   <si>
-    <t xml:space="preserve">A TESTER</t>
+    <t xml:space="preserve">A TESTER + Vérifier le nb de pas : quand on arrive au bout et recule on fait fait pas -5, a voir si ça gène</t>
   </si>
   <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
@@ -1716,7 +1716,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="97">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1786,10 +1786,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
@@ -3114,10 +3111,10 @@
     </row>
     <row r="22" ht="114">
       <c r="A22" s="1"/>
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="37" t="s">
         <v>69</v>
       </c>
       <c r="D22" s="33">
@@ -3166,8 +3163,8 @@
         <v>1</v>
       </c>
       <c r="H23" s="1"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
+      <c r="I23" s="38"/>
+      <c r="J23" s="38"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
         <v>76</v>
@@ -3197,15 +3194,15 @@
         <v>79</v>
       </c>
       <c r="D24" s="33"/>
-      <c r="F24" s="40" t="s">
+      <c r="F24" s="39" t="s">
         <v>80</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="41"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="43"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="42"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
         <v>81</v>
@@ -3246,11 +3243,11 @@
     </row>
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="44" t="s">
+      <c r="B26" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="45"/>
-      <c r="D26" s="46">
+      <c r="C26" s="44"/>
+      <c r="D26" s="45">
         <f>SUM(D27:D32)/5</f>
         <v>0</v>
       </c>
@@ -3452,11 +3449,11 @@
     </row>
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
-      <c r="B36" s="47" t="s">
+      <c r="B36" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="45"/>
-      <c r="D36" s="46">
+      <c r="C36" s="44"/>
+      <c r="D36" s="45">
         <f>SUM(D37:D40)/4</f>
         <v>0</v>
       </c>
@@ -3751,7 +3748,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="14.25">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="47" t="s">
         <v>127</v>
       </c>
       <c r="C2" t="s">
@@ -3783,52 +3780,52 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="49" t="s">
+      <c r="F2" s="48" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="50" t="s">
+      <c r="G2" s="49" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="3">
-      <c r="F3" s="51" t="s">
+      <c r="F3" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="52" t="s">
+      <c r="G3" s="51" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="4">
-      <c r="F4" s="53" t="s">
+      <c r="F4" s="52" t="s">
         <v>134</v>
       </c>
-      <c r="G4" s="54" t="s">
+      <c r="G4" s="53" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="G5" s="56" t="s">
+      <c r="G5" s="55" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="F6" s="57"/>
-      <c r="G6" s="58" t="s">
+      <c r="F6" s="56"/>
+      <c r="G6" s="57" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="F7" s="57"/>
-      <c r="G7" s="58" t="s">
+      <c r="F7" s="56"/>
+      <c r="G7" s="57" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="F8" s="57"/>
-      <c r="G8" s="58" t="s">
+      <c r="F8" s="56"/>
+      <c r="G8" s="57" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3836,8 +3833,8 @@
       <c r="B9" t="s">
         <v>141</v>
       </c>
-      <c r="F9" s="57"/>
-      <c r="G9" s="58" t="s">
+      <c r="F9" s="56"/>
+      <c r="G9" s="57" t="s">
         <v>142</v>
       </c>
     </row>
@@ -3845,218 +3842,218 @@
       <c r="B10" t="s">
         <v>143</v>
       </c>
-      <c r="C10" s="59" t="s">
+      <c r="C10" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="F10" s="57"/>
-      <c r="G10" s="58" t="s">
+      <c r="F10" s="56"/>
+      <c r="G10" s="57" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="11" ht="15">
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="59" t="s">
         <v>146</v>
       </c>
-      <c r="F11" s="57"/>
-      <c r="G11" s="58" t="s">
+      <c r="F11" s="56"/>
+      <c r="G11" s="57" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="C12" s="59" t="s">
+      <c r="C12" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="F12" s="51"/>
-      <c r="G12" s="61" t="s">
+      <c r="F12" s="50"/>
+      <c r="G12" s="60" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="13" ht="15">
-      <c r="C13" s="60" t="s">
+      <c r="C13" s="59" t="s">
         <v>150</v>
       </c>
-      <c r="F13" s="53" t="s">
+      <c r="F13" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="G13" s="62" t="s">
+      <c r="G13" s="61" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="14" ht="15">
-      <c r="C14" s="59" t="s">
+      <c r="C14" s="58" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="63" t="s">
+      <c r="F14" s="62" t="s">
         <v>154</v>
       </c>
-      <c r="G14" s="64" t="s">
+      <c r="G14" s="63" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="60" t="s">
+      <c r="C15" s="59" t="s">
         <v>156</v>
       </c>
-      <c r="F15" s="65" t="s">
+      <c r="F15" s="64" t="s">
         <v>157</v>
       </c>
-      <c r="G15" s="66" t="s">
+      <c r="G15" s="65" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="60" t="s">
+      <c r="C16" s="59" t="s">
         <v>159</v>
       </c>
-      <c r="F16" s="67" t="s">
+      <c r="F16" s="66" t="s">
         <v>160</v>
       </c>
-      <c r="G16" s="68" t="s">
+      <c r="G16" s="67" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="59" t="s">
+      <c r="C17" s="58" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="67"/>
-      <c r="G17" s="68" t="s">
+      <c r="F17" s="66"/>
+      <c r="G17" s="67" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="59" t="s">
         <v>164</v>
       </c>
-      <c r="F18" s="67"/>
-      <c r="G18" s="68" t="s">
+      <c r="F18" s="66"/>
+      <c r="G18" s="67" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="60" t="s">
+      <c r="C19" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="67"/>
-      <c r="G19" s="68" t="s">
+      <c r="F19" s="66"/>
+      <c r="G19" s="67" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="60" t="s">
+      <c r="C20" s="59" t="s">
         <v>168</v>
       </c>
-      <c r="F20" s="67"/>
-      <c r="G20" s="68" t="s">
+      <c r="F20" s="66"/>
+      <c r="G20" s="67" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="60" t="s">
+      <c r="C21" s="59" t="s">
         <v>170</v>
       </c>
-      <c r="F21" s="67"/>
-      <c r="G21" s="68" t="s">
+      <c r="F21" s="66"/>
+      <c r="G21" s="67" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="59" t="s">
+      <c r="C22" s="58" t="s">
         <v>172</v>
       </c>
-      <c r="F22" s="67"/>
-      <c r="G22" s="68" t="s">
+      <c r="F22" s="66"/>
+      <c r="G22" s="67" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="60" t="s">
+      <c r="C23" s="59" t="s">
         <v>174</v>
       </c>
-      <c r="F23" s="67"/>
-      <c r="G23" s="68" t="s">
+      <c r="F23" s="66"/>
+      <c r="G23" s="67" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="59" t="s">
+      <c r="C24" s="58" t="s">
         <v>176</v>
       </c>
-      <c r="F24" s="67"/>
-      <c r="G24" s="68" t="s">
+      <c r="F24" s="66"/>
+      <c r="G24" s="67" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="60" t="s">
+      <c r="C25" s="59" t="s">
         <v>178</v>
       </c>
-      <c r="F25" s="67"/>
-      <c r="G25" s="68" t="s">
+      <c r="F25" s="66"/>
+      <c r="G25" s="67" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="26">
-      <c r="F26" s="67"/>
-      <c r="G26" s="68" t="s">
+      <c r="F26" s="66"/>
+      <c r="G26" s="67" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="67"/>
-      <c r="G27" s="68"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="67"/>
     </row>
     <row r="28">
-      <c r="F28" s="67"/>
-      <c r="G28" s="68" t="s">
+      <c r="F28" s="66"/>
+      <c r="G28" s="67" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="67"/>
-      <c r="G29" s="68" t="s">
+      <c r="F29" s="66"/>
+      <c r="G29" s="67" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="69"/>
-      <c r="F30" s="67"/>
-      <c r="G30" s="68" t="s">
+      <c r="C30" s="68"/>
+      <c r="F30" s="66"/>
+      <c r="G30" s="67" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="67"/>
-      <c r="G31" s="70" t="s">
+      <c r="F31" s="66"/>
+      <c r="G31" s="69" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="63" t="s">
+      <c r="F32" s="62" t="s">
         <v>185</v>
       </c>
-      <c r="G32" s="71" t="s">
+      <c r="G32" s="70" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="60"/>
+      <c r="C33" s="59"/>
     </row>
     <row r="34">
-      <c r="C34" s="60"/>
+      <c r="C34" s="59"/>
     </row>
     <row r="36">
-      <c r="C36" s="69"/>
+      <c r="C36" s="68"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="60"/>
+      <c r="C39" s="59"/>
     </row>
     <row r="40">
-      <c r="C40" s="60"/>
+      <c r="C40" s="59"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -4089,7 +4086,7 @@
       <c r="B5" t="s">
         <v>188</v>
       </c>
-      <c r="D5" s="72" t="s">
+      <c r="D5" s="71" t="s">
         <v>189</v>
       </c>
       <c r="E5" t="s">
@@ -4121,7 +4118,7 @@
       <c r="B6" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="73" t="s">
+      <c r="D6" s="72" t="s">
         <v>197</v>
       </c>
       <c r="E6" t="s">
@@ -4133,7 +4130,7 @@
       <c r="G6" t="s">
         <v>200</v>
       </c>
-      <c r="H6" s="74" t="s">
+      <c r="H6" s="73" t="s">
         <v>201</v>
       </c>
       <c r="I6" t="s">
@@ -4153,7 +4150,7 @@
       <c r="B7" t="s">
         <v>196</v>
       </c>
-      <c r="D7" s="75" t="s">
+      <c r="D7" s="74" t="s">
         <v>206</v>
       </c>
       <c r="F7" t="s">
@@ -4162,7 +4159,7 @@
       <c r="G7" t="s">
         <v>208</v>
       </c>
-      <c r="H7" s="74" t="s">
+      <c r="H7" s="73" t="s">
         <v>209</v>
       </c>
       <c r="K7" t="s">
@@ -4170,13 +4167,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="73" t="s">
+      <c r="D8" s="72" t="s">
         <v>211</v>
       </c>
-      <c r="G8" s="76" t="s">
+      <c r="G8" s="75" t="s">
         <v>212</v>
       </c>
-      <c r="H8" s="74" t="s">
+      <c r="H8" s="73" t="s">
         <v>213</v>
       </c>
     </row>
@@ -4187,10 +4184,10 @@
       <c r="B9" t="s">
         <v>215</v>
       </c>
-      <c r="D9" s="75" t="s">
+      <c r="D9" s="74" t="s">
         <v>216</v>
       </c>
-      <c r="H9" s="74" t="s">
+      <c r="H9" s="73" t="s">
         <v>217</v>
       </c>
     </row>
@@ -4201,11 +4198,11 @@
       <c r="B10" t="s">
         <v>219</v>
       </c>
-      <c r="D10" s="73"/>
+      <c r="D10" s="72"/>
       <c r="G10" t="s">
         <v>220</v>
       </c>
-      <c r="H10" s="74" t="s">
+      <c r="H10" s="73" t="s">
         <v>221</v>
       </c>
     </row>
@@ -4216,13 +4213,13 @@
       <c r="B11" t="s">
         <v>223</v>
       </c>
-      <c r="D11" s="75" t="s">
+      <c r="D11" s="74" t="s">
         <v>224</v>
       </c>
-      <c r="G11" s="76" t="s">
+      <c r="G11" s="75" t="s">
         <v>225</v>
       </c>
-      <c r="H11" s="74" t="s">
+      <c r="H11" s="73" t="s">
         <v>226</v>
       </c>
     </row>
@@ -4233,13 +4230,13 @@
       <c r="B12" t="s">
         <v>228</v>
       </c>
-      <c r="D12" s="73" t="s">
+      <c r="D12" s="72" t="s">
         <v>229</v>
       </c>
-      <c r="G12" s="76" t="s">
+      <c r="G12" s="75" t="s">
         <v>230</v>
       </c>
-      <c r="H12" s="74" t="s">
+      <c r="H12" s="73" t="s">
         <v>231</v>
       </c>
     </row>
@@ -4250,15 +4247,15 @@
       <c r="B13" t="s">
         <v>233</v>
       </c>
-      <c r="D13" s="75" t="s">
+      <c r="D13" s="74" t="s">
         <v>234</v>
       </c>
-      <c r="G13" s="76" t="s">
+      <c r="G13" s="75" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="73" t="s">
+      <c r="D14" s="72" t="s">
         <v>236</v>
       </c>
     </row>
@@ -4269,7 +4266,7 @@
       <c r="B15" t="s">
         <v>238</v>
       </c>
-      <c r="D15" s="75"/>
+      <c r="D15" s="74"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
@@ -4278,14 +4275,14 @@
       <c r="B16" t="s">
         <v>240</v>
       </c>
-      <c r="D16" s="73"/>
+      <c r="D16" s="72"/>
       <c r="G16" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="75"/>
-      <c r="G17" s="76" t="s">
+      <c r="D17" s="74"/>
+      <c r="G17" s="75" t="s">
         <v>242</v>
       </c>
     </row>
@@ -4293,19 +4290,19 @@
       <c r="A18" t="s">
         <v>243</v>
       </c>
-      <c r="D18" s="73"/>
-      <c r="G18" s="77" t="s">
+      <c r="D18" s="72"/>
+      <c r="G18" s="76" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="75" t="s">
+      <c r="D19" s="74" t="s">
         <v>245</v>
       </c>
       <c r="E19" t="s">
         <v>246</v>
       </c>
-      <c r="G19" s="77" t="s">
+      <c r="G19" s="76" t="s">
         <v>247</v>
       </c>
       <c r="H19" t="s">
@@ -4319,100 +4316,100 @@
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="73"/>
-      <c r="G20" s="77" t="s">
+      <c r="D20" s="72"/>
+      <c r="G20" s="76" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="73"/>
-      <c r="G22" s="77" t="s">
+      <c r="D22" s="72"/>
+      <c r="G22" s="76" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="23">
-      <c r="G23" s="76"/>
+      <c r="G23" s="75"/>
     </row>
     <row r="24">
-      <c r="D24" s="73"/>
-      <c r="G24" s="76" t="s">
+      <c r="D24" s="72"/>
+      <c r="G24" s="75" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="25">
-      <c r="G25" s="77" t="s">
+      <c r="G25" s="76" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="26">
-      <c r="D26" s="73"/>
-      <c r="G26" s="77" t="s">
+      <c r="D26" s="72"/>
+      <c r="G26" s="76" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="27">
-      <c r="G27" s="77" t="s">
+      <c r="G27" s="76" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="28">
-      <c r="D28" s="73"/>
-      <c r="G28" s="77" t="s">
+      <c r="D28" s="72"/>
+      <c r="G28" s="76" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="35">
-      <c r="D35" s="78" t="s">
+      <c r="D35" s="77" t="s">
         <v>255</v>
       </c>
       <c r="E35" t="s">
         <v>256</v>
       </c>
-      <c r="F35" s="79" t="s">
+      <c r="F35" s="78" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="36">
-      <c r="D36" s="80" t="s">
+      <c r="D36" s="79" t="s">
         <v>258</v>
       </c>
       <c r="E36" t="s">
         <v>259</v>
       </c>
-      <c r="F36" s="80" t="s">
+      <c r="F36" s="79" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="37">
-      <c r="D37" s="79" t="s">
+      <c r="D37" s="78" t="s">
         <v>261</v>
       </c>
       <c r="E37" t="s">
         <v>262</v>
       </c>
-      <c r="F37" s="79" t="s">
+      <c r="F37" s="78" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="80" t="s">
+      <c r="D38" s="79" t="s">
         <v>264</v>
       </c>
       <c r="E38" t="s">
         <v>265</v>
       </c>
-      <c r="F38" s="80" t="s">
+      <c r="F38" s="79" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="39">
-      <c r="D39" s="79" t="s">
+      <c r="D39" s="78" t="s">
         <v>267</v>
       </c>
       <c r="E39" t="s">
         <v>268</v>
       </c>
-      <c r="F39" s="79" t="s">
+      <c r="F39" s="78" t="s">
         <v>269</v>
       </c>
     </row>
@@ -4420,7 +4417,7 @@
       <c r="E40" t="s">
         <v>259</v>
       </c>
-      <c r="F40" s="80" t="s">
+      <c r="F40" s="79" t="s">
         <v>270</v>
       </c>
     </row>
@@ -4428,7 +4425,7 @@
       <c r="E41" t="s">
         <v>262</v>
       </c>
-      <c r="F41" s="79" t="s">
+      <c r="F41" s="78" t="s">
         <v>271</v>
       </c>
     </row>
@@ -4475,7 +4472,7 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="81" t="s">
+      <c r="D4" s="80" t="s">
         <v>274</v>
       </c>
       <c r="E4" t="s">
@@ -4486,168 +4483,168 @@
       <c r="D5" t="s">
         <v>276</v>
       </c>
-      <c r="E5" s="81">
+      <c r="E5" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="77" t="s">
+      <c r="D6" s="76" t="s">
         <v>277</v>
       </c>
-      <c r="E6" s="81">
+      <c r="E6" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="82" t="s">
+      <c r="D7" s="81" t="s">
         <v>278</v>
       </c>
-      <c r="E7" s="81">
+      <c r="E7" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="77" t="s">
+      <c r="D8" s="76" t="s">
         <v>279</v>
       </c>
-      <c r="E8" s="81">
+      <c r="E8" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="77"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="80"/>
     </row>
     <row r="10">
-      <c r="D10" s="74" t="s">
+      <c r="D10" s="73" t="s">
         <v>280</v>
       </c>
-      <c r="E10" s="81">
+      <c r="E10" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="D11" s="77" t="s">
+      <c r="D11" s="76" t="s">
         <v>281</v>
       </c>
-      <c r="E11" s="81">
+      <c r="E11" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="D12" s="77" t="s">
+      <c r="D12" s="76" t="s">
         <v>282</v>
       </c>
-      <c r="E12" s="81">
+      <c r="E12" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="D13" s="77" t="s">
+      <c r="D13" s="76" t="s">
         <v>283</v>
       </c>
-      <c r="E13" s="81">
+      <c r="E13" s="80">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="77"/>
-      <c r="E14" s="77"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="76"/>
     </row>
     <row r="15">
-      <c r="D15" s="74" t="s">
+      <c r="D15" s="73" t="s">
         <v>284</v>
       </c>
-      <c r="E15" s="81">
+      <c r="E15" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="16">
-      <c r="D16" s="83" t="s">
+      <c r="D16" s="82" t="s">
         <v>285</v>
       </c>
-      <c r="E16" s="81">
+      <c r="E16" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="84" t="s">
+      <c r="D17" s="83" t="s">
         <v>286</v>
       </c>
-      <c r="E17" s="81">
+      <c r="E17" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="84" t="s">
+      <c r="D18" s="83" t="s">
         <v>287</v>
       </c>
-      <c r="E18" s="81">
+      <c r="E18" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="77"/>
-      <c r="E19" s="77"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
     </row>
     <row r="20">
-      <c r="D20" s="74" t="s">
+      <c r="D20" s="73" t="s">
         <v>288</v>
       </c>
-      <c r="E20" s="81">
+      <c r="E20" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="21">
-      <c r="D21" s="74" t="s">
+      <c r="D21" s="73" t="s">
         <v>289</v>
       </c>
-      <c r="E21" s="81">
+      <c r="E21" s="80">
         <v>2</v>
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="77"/>
-      <c r="E22" s="77"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
     </row>
     <row r="23">
-      <c r="D23" s="85"/>
-      <c r="E23" s="77"/>
+      <c r="D23" s="84"/>
+      <c r="E23" s="76"/>
     </row>
     <row r="24">
-      <c r="D24" s="77"/>
-      <c r="E24" s="77"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
     </row>
     <row r="25">
-      <c r="D25" s="77"/>
-      <c r="E25" s="77"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
     </row>
     <row r="26">
-      <c r="D26" s="77"/>
-      <c r="E26" s="77"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="76"/>
     </row>
     <row r="27">
-      <c r="D27" s="77"/>
-      <c r="E27" s="77"/>
+      <c r="D27" s="76"/>
+      <c r="E27" s="76"/>
     </row>
     <row r="28">
-      <c r="D28" s="77"/>
-      <c r="E28" s="77"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
     </row>
     <row r="29">
-      <c r="D29" s="77"/>
-      <c r="E29" s="77"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
     </row>
     <row r="30">
-      <c r="D30" s="77"/>
-      <c r="E30" s="77"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="76"/>
     </row>
     <row r="39">
-      <c r="B39" s="86"/>
-      <c r="C39" s="87" t="s">
+      <c r="B39" s="85"/>
+      <c r="C39" s="86" t="s">
         <v>290</v>
       </c>
-      <c r="D39" s="87" t="s">
+      <c r="D39" s="86" t="s">
         <v>291</v>
       </c>
       <c r="E39" t="s">
@@ -4658,200 +4655,200 @@
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="88">
+      <c r="C40" s="87">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="E40" s="81"/>
+      <c r="E40" s="80"/>
     </row>
     <row r="41">
-      <c r="C41" s="81" t="s">
+      <c r="C41" s="80" t="s">
         <v>293</v>
       </c>
-      <c r="D41" s="77" t="s">
+      <c r="D41" s="76" t="s">
         <v>294</v>
       </c>
-      <c r="E41" s="81"/>
+      <c r="E41" s="80"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="81" t="s">
+      <c r="C42" s="80" t="s">
         <v>295</v>
       </c>
-      <c r="D42" s="77" t="s">
+      <c r="D42" s="76" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="81" t="s">
+      <c r="C43" s="80" t="s">
         <v>297</v>
       </c>
-      <c r="D43" s="77" t="s">
+      <c r="D43" s="76" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="89" t="s">
+      <c r="C44" s="88" t="s">
         <v>299</v>
       </c>
-      <c r="D44" s="82" t="s">
+      <c r="D44" s="81" t="s">
         <v>300</v>
       </c>
-      <c r="E44" s="90"/>
-      <c r="F44" s="90"/>
+      <c r="E44" s="89"/>
+      <c r="F44" s="89"/>
     </row>
     <row r="45">
-      <c r="C45" s="87" t="s">
+      <c r="C45" s="86" t="s">
         <v>301</v>
       </c>
-      <c r="D45" s="77" t="s">
+      <c r="D45" s="76" t="s">
         <v>302</v>
       </c>
-      <c r="E45" s="81"/>
+      <c r="E45" s="80"/>
     </row>
     <row r="46">
-      <c r="C46" s="87" t="s">
+      <c r="C46" s="86" t="s">
         <v>303</v>
       </c>
-      <c r="D46" s="77" t="s">
+      <c r="D46" s="76" t="s">
         <v>304</v>
       </c>
-      <c r="E46" s="81"/>
+      <c r="E46" s="80"/>
     </row>
     <row r="47">
-      <c r="C47" s="91">
+      <c r="C47" s="90">
         <v>2</v>
       </c>
-      <c r="D47" s="92" t="s">
+      <c r="D47" s="91" t="s">
         <v>305</v>
       </c>
-      <c r="E47" s="81"/>
+      <c r="E47" s="80"/>
     </row>
     <row r="48">
-      <c r="C48" s="89" t="s">
+      <c r="C48" s="88" t="s">
         <v>306</v>
       </c>
-      <c r="D48" s="82" t="s">
+      <c r="D48" s="81" t="s">
         <v>307</v>
       </c>
-      <c r="E48" s="81"/>
+      <c r="E48" s="80"/>
     </row>
     <row r="49">
-      <c r="C49" s="88">
+      <c r="C49" s="87">
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="E49" s="81"/>
+      <c r="E49" s="80"/>
     </row>
     <row r="50">
-      <c r="C50" s="89" t="s">
+      <c r="C50" s="88" t="s">
         <v>309</v>
       </c>
-      <c r="D50" s="82" t="s">
+      <c r="D50" s="81" t="s">
         <v>310</v>
       </c>
-      <c r="F50" s="93" t="s">
+      <c r="F50" s="92" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="51">
-      <c r="C51" s="89" t="s">
+      <c r="C51" s="88" t="s">
         <v>312</v>
       </c>
-      <c r="D51" s="94" t="s">
+      <c r="D51" s="93" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="89" t="s">
+      <c r="C52" s="88" t="s">
         <v>314</v>
       </c>
-      <c r="D52" s="94" t="s">
+      <c r="D52" s="93" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="89" t="s">
+      <c r="C53" s="88" t="s">
         <v>316</v>
       </c>
-      <c r="D53" s="94" t="s">
+      <c r="D53" s="93" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="89" t="s">
+      <c r="C54" s="88" t="s">
         <v>318</v>
       </c>
-      <c r="D54" s="94" t="s">
+      <c r="D54" s="93" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="95">
+      <c r="C55" s="94">
         <v>4</v>
       </c>
-      <c r="D55" s="95" t="s">
+      <c r="D55" s="94" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="87" t="s">
+      <c r="C56" s="86" t="s">
         <v>321</v>
       </c>
-      <c r="D56" s="77" t="s">
+      <c r="D56" s="76" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="87" t="s">
+      <c r="C57" s="86" t="s">
         <v>323</v>
       </c>
-      <c r="D57" s="94" t="s">
+      <c r="D57" s="93" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="87" t="s">
+      <c r="C58" s="86" t="s">
         <v>325</v>
       </c>
-      <c r="D58" s="94" t="s">
+      <c r="D58" s="93" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="87" t="s">
+      <c r="C59" s="86" t="s">
         <v>327</v>
       </c>
-      <c r="D59" s="94" t="s">
+      <c r="D59" s="93" t="s">
         <v>328</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="95">
+      <c r="C60" s="94">
         <v>5</v>
       </c>
-      <c r="D60" s="95" t="s">
+      <c r="D60" s="94" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="87" t="s">
+      <c r="C61" s="86" t="s">
         <v>330</v>
       </c>
-      <c r="D61" s="77" t="s">
+      <c r="D61" s="76" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="87" t="s">
+      <c r="C62" s="86" t="s">
         <v>332</v>
       </c>
-      <c r="D62" s="94" t="s">
+      <c r="D62" s="93" t="s">
         <v>333</v>
       </c>
       <c r="F62" t="s">
@@ -4859,71 +4856,71 @@
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="87" t="s">
+      <c r="C63" s="86" t="s">
         <v>335</v>
       </c>
-      <c r="D63" s="94" t="s">
+      <c r="D63" s="93" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="87" t="s">
+      <c r="C64" s="86" t="s">
         <v>337</v>
       </c>
-      <c r="D64" s="94" t="s">
+      <c r="D64" s="93" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="95">
+      <c r="C65" s="94">
         <v>6</v>
       </c>
-      <c r="D65" s="95" t="s">
+      <c r="D65" s="94" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="87" t="s">
+      <c r="C66" s="86" t="s">
         <v>340</v>
       </c>
-      <c r="D66" s="77" t="s">
+      <c r="D66" s="76" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="96" t="s">
+      <c r="C67" s="95" t="s">
         <v>342</v>
       </c>
-      <c r="D67" s="97" t="s">
+      <c r="D67" s="96" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="87" t="s">
+      <c r="C68" s="86" t="s">
         <v>344</v>
       </c>
-      <c r="D68" s="94" t="s">
+      <c r="D68" s="93" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="96" t="s">
+      <c r="C69" s="95" t="s">
         <v>346</v>
       </c>
-      <c r="D69" s="94" t="s">
+      <c r="D69" s="93" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="87" t="s">
+      <c r="C70" s="86" t="s">
         <v>348</v>
       </c>
-      <c r="D70" s="94" t="s">
+      <c r="D70" s="93" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="95">
+      <c r="C71" s="94">
         <v>7</v>
       </c>
       <c r="D71" s="5" t="s">
@@ -4931,15 +4928,15 @@
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="87" t="s">
+      <c r="C72" s="86" t="s">
         <v>351</v>
       </c>
-      <c r="D72" s="77" t="s">
+      <c r="D72" s="76" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="95">
+      <c r="C73" s="94">
         <v>8</v>
       </c>
       <c r="D73" s="5" t="s">
@@ -4947,15 +4944,15 @@
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="87" t="s">
+      <c r="C74" s="86" t="s">
         <v>354</v>
       </c>
-      <c r="D74" s="77" t="s">
+      <c r="D74" s="76" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="95">
+      <c r="C75" s="94">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
@@ -4963,31 +4960,31 @@
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="87" t="s">
+      <c r="C76" s="86" t="s">
         <v>356</v>
       </c>
-      <c r="D76" s="77" t="s">
+      <c r="D76" s="76" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="87" t="s">
+      <c r="C77" s="86" t="s">
         <v>358</v>
       </c>
-      <c r="D77" s="94" t="s">
+      <c r="D77" s="93" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="87" t="s">
+      <c r="C78" s="86" t="s">
         <v>360</v>
       </c>
-      <c r="D78" s="94" t="s">
+      <c r="D78" s="93" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="79">
-      <c r="C79" s="95">
+      <c r="C79" s="94">
         <v>10</v>
       </c>
       <c r="D79" s="5" t="s">
@@ -4995,24 +4992,24 @@
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="87" t="s">
+      <c r="C80" s="86" t="s">
         <v>363</v>
       </c>
-      <c r="D80" s="77" t="s">
+      <c r="D80" s="76" t="s">
         <v>364</v>
       </c>
-      <c r="E80" s="81"/>
+      <c r="E80" s="80"/>
     </row>
     <row r="81">
-      <c r="C81" s="87" t="s">
+      <c r="C81" s="86" t="s">
         <v>365</v>
       </c>
-      <c r="D81" s="94" t="s">
+      <c r="D81" s="93" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="95">
+      <c r="C82" s="94">
         <v>11</v>
       </c>
       <c r="D82" s="5" t="s">
@@ -5020,18 +5017,18 @@
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="87" t="s">
+      <c r="C83" s="86" t="s">
         <v>368</v>
       </c>
-      <c r="D83" s="77" t="s">
+      <c r="D83" s="76" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="84">
-      <c r="C84" s="87" t="s">
+      <c r="C84" s="86" t="s">
         <v>370</v>
       </c>
-      <c r="D84" s="77" t="s">
+      <c r="D84" s="76" t="s">
         <v>371</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add goToOriin in seetin + sleep
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="371">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -386,9 +386,6 @@
   </si>
   <si>
     <t xml:space="preserve">Application, afficher les CD enregistés : fomarter la hauteur de l'image et largeur pareil pour tout. Ex : ADC et PBB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Animation photo d'un album lancé</t>
   </si>
   <si>
     <t xml:space="preserve">Image du projet sur la Raspberry</t>
@@ -1716,7 +1713,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="96">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1883,9 +1880,6 @@
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="17" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3455,7 +3449,7 @@
       <c r="C36" s="44"/>
       <c r="D36" s="45">
         <f>SUM(D37:D40)/4</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -3476,8 +3470,8 @@
       <c r="C37" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="33">
-        <v>0</v>
+      <c r="D37" s="28">
+        <v>1</v>
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -3498,8 +3492,8 @@
       <c r="C38" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="33">
-        <v>0</v>
+      <c r="D38" s="28">
+        <v>1</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
@@ -3520,8 +3514,8 @@
       <c r="C39" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D39" s="33">
-        <v>0</v>
+      <c r="D39" s="28">
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="28.5">
@@ -3615,9 +3609,6 @@
     </row>
     <row r="55" ht="16.5">
       <c r="A55" s="1"/>
-      <c r="B55" t="s">
-        <v>115</v>
-      </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
@@ -3645,7 +3636,7 @@
     <row r="57" ht="16.5">
       <c r="A57" s="1"/>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -3673,52 +3664,52 @@
     </row>
     <row r="69" ht="14.25">
       <c r="B69" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="78" ht="14.25">
       <c r="B78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C78" t="s">
         <v>67</v>
@@ -3749,15 +3740,15 @@
   <sheetData>
     <row r="2" ht="14.25">
       <c r="B2" s="47" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" t="s">
         <v>127</v>
-      </c>
-      <c r="C2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="3" ht="14.25">
       <c r="B3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3781,222 +3772,222 @@
     <row r="1" ht="15"/>
     <row r="2" ht="15">
       <c r="F2" s="48" t="s">
+        <v>129</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>130</v>
-      </c>
-      <c r="G2" s="49" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="3">
       <c r="F3" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="G3" s="51" t="s">
         <v>132</v>
-      </c>
-      <c r="G3" s="51" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="4">
       <c r="F4" s="52" t="s">
+        <v>133</v>
+      </c>
+      <c r="G4" s="53" t="s">
         <v>134</v>
-      </c>
-      <c r="G4" s="53" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="5" ht="15">
       <c r="F5" s="54" t="s">
+        <v>135</v>
+      </c>
+      <c r="G5" s="55" t="s">
         <v>136</v>
-      </c>
-      <c r="G5" s="55" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="F6" s="56"/>
       <c r="G6" s="57" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" ht="15">
       <c r="F7" s="56"/>
       <c r="G7" s="57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" ht="15">
       <c r="F8" s="56"/>
       <c r="G8" s="57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F9" s="56"/>
       <c r="G9" s="57" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C10" s="58" t="s">
         <v>143</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>144</v>
       </c>
       <c r="F10" s="56"/>
       <c r="G10" s="57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" ht="15">
       <c r="C11" s="59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F11" s="56"/>
       <c r="G11" s="57" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" ht="15">
       <c r="C12" s="58" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F12" s="50"/>
       <c r="G12" s="60" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" ht="15">
       <c r="C13" s="59" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="F13" s="52" t="s">
+      <c r="G13" s="61" t="s">
         <v>151</v>
-      </c>
-      <c r="G13" s="61" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="14" ht="15">
       <c r="C14" s="58" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" s="62" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="62" t="s">
+      <c r="G14" s="63" t="s">
         <v>154</v>
-      </c>
-      <c r="G14" s="63" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="15">
       <c r="C15" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="F15" s="64" t="s">
         <v>156</v>
       </c>
-      <c r="F15" s="64" t="s">
+      <c r="G15" s="65" t="s">
         <v>157</v>
-      </c>
-      <c r="G15" s="65" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="16">
       <c r="C16" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="F16" s="66" t="s">
         <v>159</v>
       </c>
-      <c r="F16" s="66" t="s">
+      <c r="G16" s="67" t="s">
         <v>160</v>
-      </c>
-      <c r="G16" s="67" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="17">
       <c r="C17" s="58" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F17" s="66"/>
       <c r="G17" s="67" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18">
       <c r="C18" s="59" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F18" s="66"/>
       <c r="G18" s="67" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19">
       <c r="C19" s="59" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F19" s="66"/>
       <c r="G19" s="67" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20">
       <c r="C20" s="59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F20" s="66"/>
       <c r="G20" s="67" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21">
       <c r="C21" s="59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F21" s="66"/>
       <c r="G21" s="67" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22">
       <c r="C22" s="58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F22" s="66"/>
       <c r="G22" s="67" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="59" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F23" s="66"/>
       <c r="G23" s="67" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24">
       <c r="C24" s="58" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F24" s="66"/>
       <c r="G24" s="67" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="59" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F25" s="66"/>
       <c r="G25" s="67" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26">
       <c r="F26" s="66"/>
       <c r="G26" s="67" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27">
@@ -4006,35 +3997,35 @@
     <row r="28">
       <c r="F28" s="66"/>
       <c r="G28" s="67" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29">
       <c r="F29" s="66"/>
       <c r="G29" s="67" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="68"/>
       <c r="F30" s="66"/>
       <c r="G30" s="67" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31">
       <c r="F31" s="66"/>
       <c r="G31" s="69" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
       <c r="F32" s="62" t="s">
+        <v>184</v>
+      </c>
+      <c r="G32" s="70" t="s">
         <v>185</v>
-      </c>
-      <c r="G32" s="70" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="33">
@@ -4081,13 +4072,13 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B5" t="s">
         <v>187</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" s="71" t="s">
         <v>188</v>
-      </c>
-      <c r="D5" s="71" t="s">
-        <v>189</v>
       </c>
       <c r="E5" t="s">
         <v>104</v>
@@ -4096,235 +4087,235 @@
         <v>100</v>
       </c>
       <c r="G5" t="s">
+        <v>189</v>
+      </c>
+      <c r="H5" t="s">
         <v>190</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>191</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>192</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>193</v>
-      </c>
-      <c r="K5" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B6" t="s">
         <v>195</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" s="72" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="72" t="s">
+      <c r="E6" t="s">
         <v>197</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>198</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>199</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" s="73" t="s">
         <v>200</v>
       </c>
-      <c r="H6" s="73" t="s">
+      <c r="I6" t="s">
         <v>201</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>202</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>203</v>
-      </c>
-      <c r="K6" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="74" t="s">
         <v>205</v>
       </c>
-      <c r="B7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D7" s="74" t="s">
+      <c r="F7" t="s">
         <v>206</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>207</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="73" t="s">
         <v>208</v>
       </c>
-      <c r="H7" s="73" t="s">
+      <c r="K7" t="s">
         <v>209</v>
-      </c>
-      <c r="K7" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="8">
       <c r="D8" s="72" t="s">
+        <v>210</v>
+      </c>
+      <c r="G8" s="75" t="s">
         <v>211</v>
       </c>
-      <c r="G8" s="75" t="s">
+      <c r="H8" s="73" t="s">
         <v>212</v>
-      </c>
-      <c r="H8" s="73" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" t="s">
         <v>214</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" s="74" t="s">
         <v>215</v>
       </c>
-      <c r="D9" s="74" t="s">
+      <c r="H9" s="73" t="s">
         <v>216</v>
-      </c>
-      <c r="H9" s="73" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" t="s">
         <v>218</v>
-      </c>
-      <c r="B10" t="s">
-        <v>219</v>
       </c>
       <c r="D10" s="72"/>
       <c r="G10" t="s">
+        <v>219</v>
+      </c>
+      <c r="H10" s="73" t="s">
         <v>220</v>
-      </c>
-      <c r="H10" s="73" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B11" t="s">
         <v>222</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" s="74" t="s">
         <v>223</v>
       </c>
-      <c r="D11" s="74" t="s">
+      <c r="G11" s="75" t="s">
         <v>224</v>
       </c>
-      <c r="G11" s="75" t="s">
+      <c r="H11" s="73" t="s">
         <v>225</v>
-      </c>
-      <c r="H11" s="73" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>226</v>
+      </c>
+      <c r="B12" t="s">
         <v>227</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" s="72" t="s">
         <v>228</v>
       </c>
-      <c r="D12" s="72" t="s">
+      <c r="G12" s="75" t="s">
         <v>229</v>
       </c>
-      <c r="G12" s="75" t="s">
+      <c r="H12" s="73" t="s">
         <v>230</v>
-      </c>
-      <c r="H12" s="73" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13" t="s">
         <v>232</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" s="74" t="s">
         <v>233</v>
       </c>
-      <c r="D13" s="74" t="s">
+      <c r="G13" s="75" t="s">
         <v>234</v>
-      </c>
-      <c r="G13" s="75" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="14">
       <c r="D14" s="72" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>236</v>
+      </c>
+      <c r="B15" t="s">
         <v>237</v>
-      </c>
-      <c r="B15" t="s">
-        <v>238</v>
       </c>
       <c r="D15" s="74"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>238</v>
+      </c>
+      <c r="B16" t="s">
         <v>239</v>
-      </c>
-      <c r="B16" t="s">
-        <v>240</v>
       </c>
       <c r="D16" s="72"/>
       <c r="G16" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="74"/>
       <c r="G17" s="75" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D18" s="72"/>
       <c r="G18" s="76" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="74" t="s">
+        <v>244</v>
+      </c>
+      <c r="E19" t="s">
         <v>245</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" s="76" t="s">
         <v>246</v>
       </c>
-      <c r="G19" s="76" t="s">
+      <c r="H19" t="s">
         <v>247</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>248</v>
       </c>
-      <c r="I19" t="s">
-        <v>249</v>
-      </c>
       <c r="J19" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="72"/>
       <c r="G20" s="76" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="72"/>
       <c r="G22" s="76" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23">
@@ -4333,115 +4324,115 @@
     <row r="24">
       <c r="D24" s="72"/>
       <c r="G24" s="75" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25">
       <c r="G25" s="76" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="72"/>
       <c r="G26" s="76" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="27">
       <c r="G27" s="76" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="72"/>
       <c r="G28" s="76" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="77" t="s">
+        <v>254</v>
+      </c>
+      <c r="E35" t="s">
         <v>255</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" s="78" t="s">
         <v>256</v>
-      </c>
-      <c r="F35" s="78" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="79" t="s">
+        <v>257</v>
+      </c>
+      <c r="E36" t="s">
         <v>258</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" s="79" t="s">
         <v>259</v>
-      </c>
-      <c r="F36" s="79" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="78" t="s">
+        <v>260</v>
+      </c>
+      <c r="E37" t="s">
         <v>261</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" s="78" t="s">
         <v>262</v>
-      </c>
-      <c r="F37" s="78" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="79" t="s">
+        <v>263</v>
+      </c>
+      <c r="E38" t="s">
         <v>264</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" s="79" t="s">
         <v>265</v>
-      </c>
-      <c r="F38" s="79" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="78" t="s">
+        <v>266</v>
+      </c>
+      <c r="E39" t="s">
         <v>267</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" s="78" t="s">
         <v>268</v>
-      </c>
-      <c r="F39" s="78" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F40" s="79" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F41" s="78" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -4473,15 +4464,15 @@
   <sheetData>
     <row r="4">
       <c r="D4" s="80" t="s">
+        <v>273</v>
+      </c>
+      <c r="E4" t="s">
         <v>274</v>
-      </c>
-      <c r="E4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E5" s="80">
         <v>1</v>
@@ -4489,7 +4480,7 @@
     </row>
     <row r="6">
       <c r="D6" s="76" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E6" s="80">
         <v>1</v>
@@ -4497,7 +4488,7 @@
     </row>
     <row r="7">
       <c r="D7" s="81" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E7" s="80">
         <v>1</v>
@@ -4505,7 +4496,7 @@
     </row>
     <row r="8">
       <c r="D8" s="76" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E8" s="80">
         <v>1</v>
@@ -4517,7 +4508,7 @@
     </row>
     <row r="10">
       <c r="D10" s="73" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E10" s="80">
         <v>1</v>
@@ -4525,7 +4516,7 @@
     </row>
     <row r="11">
       <c r="D11" s="76" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E11" s="80">
         <v>1</v>
@@ -4533,7 +4524,7 @@
     </row>
     <row r="12">
       <c r="D12" s="76" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E12" s="80">
         <v>1</v>
@@ -4541,7 +4532,7 @@
     </row>
     <row r="13">
       <c r="D13" s="76" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E13" s="80">
         <v>1</v>
@@ -4553,7 +4544,7 @@
     </row>
     <row r="15">
       <c r="D15" s="73" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E15" s="80">
         <v>2</v>
@@ -4561,7 +4552,7 @@
     </row>
     <row r="16">
       <c r="D16" s="82" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E16" s="80">
         <v>2</v>
@@ -4569,7 +4560,7 @@
     </row>
     <row r="17">
       <c r="D17" s="83" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E17" s="80">
         <v>2</v>
@@ -4577,7 +4568,7 @@
     </row>
     <row r="18">
       <c r="D18" s="83" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E18" s="80">
         <v>2</v>
@@ -4589,7 +4580,7 @@
     </row>
     <row r="20">
       <c r="D20" s="73" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E20" s="80">
         <v>2</v>
@@ -4597,7 +4588,7 @@
     </row>
     <row r="21">
       <c r="D21" s="73" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E21" s="80">
         <v>2</v>
@@ -4642,13 +4633,13 @@
     <row r="39">
       <c r="B39" s="85"/>
       <c r="C39" s="86" t="s">
+        <v>289</v>
+      </c>
+      <c r="D39" s="86" t="s">
         <v>290</v>
       </c>
-      <c r="D39" s="86" t="s">
-        <v>291</v>
-      </c>
       <c r="E39" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
@@ -4659,78 +4650,78 @@
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E40" s="80"/>
     </row>
     <row r="41">
       <c r="C41" s="80" t="s">
+        <v>292</v>
+      </c>
+      <c r="D41" s="76" t="s">
         <v>293</v>
-      </c>
-      <c r="D41" s="76" t="s">
-        <v>294</v>
       </c>
       <c r="E41" s="80"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="C42" s="80" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" s="76" t="s">
         <v>295</v>
-      </c>
-      <c r="D42" s="76" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="43">
       <c r="C43" s="80" t="s">
+        <v>296</v>
+      </c>
+      <c r="D43" s="76" t="s">
         <v>297</v>
       </c>
-      <c r="D43" s="76" t="s">
+    </row>
+    <row r="44">
+      <c r="C44" s="37" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="44">
-      <c r="C44" s="88" t="s">
+      <c r="D44" s="81" t="s">
         <v>299</v>
       </c>
-      <c r="D44" s="81" t="s">
-        <v>300</v>
-      </c>
-      <c r="E44" s="89"/>
-      <c r="F44" s="89"/>
+      <c r="E44" s="88"/>
+      <c r="F44" s="88"/>
     </row>
     <row r="45">
       <c r="C45" s="86" t="s">
+        <v>300</v>
+      </c>
+      <c r="D45" s="76" t="s">
         <v>301</v>
-      </c>
-      <c r="D45" s="76" t="s">
-        <v>302</v>
       </c>
       <c r="E45" s="80"/>
     </row>
     <row r="46">
       <c r="C46" s="86" t="s">
+        <v>302</v>
+      </c>
+      <c r="D46" s="76" t="s">
         <v>303</v>
       </c>
-      <c r="D46" s="76" t="s">
+      <c r="E46" s="80"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="89">
+        <v>2</v>
+      </c>
+      <c r="D47" s="90" t="s">
         <v>304</v>
       </c>
-      <c r="E46" s="80"/>
-    </row>
-    <row r="47">
-      <c r="C47" s="90">
-        <v>2</v>
-      </c>
-      <c r="D47" s="91" t="s">
+      <c r="E47" s="80"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="37" t="s">
         <v>305</v>
       </c>
-      <c r="E47" s="80"/>
-    </row>
-    <row r="48">
-      <c r="C48" s="88" t="s">
+      <c r="D48" s="81" t="s">
         <v>306</v>
-      </c>
-      <c r="D48" s="81" t="s">
-        <v>307</v>
       </c>
       <c r="E48" s="80"/>
     </row>
@@ -4739,220 +4730,220 @@
         <v>3</v>
       </c>
       <c r="D49" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="E49" s="80"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="37" t="s">
         <v>308</v>
       </c>
-      <c r="E49" s="80"/>
-    </row>
-    <row r="50">
-      <c r="C50" s="88" t="s">
+      <c r="D50" s="81" t="s">
         <v>309</v>
       </c>
-      <c r="D50" s="81" t="s">
+      <c r="F50" s="91" t="s">
         <v>310</v>
       </c>
-      <c r="F50" s="92" t="s">
+    </row>
+    <row r="51">
+      <c r="C51" s="37" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="C51" s="88" t="s">
+      <c r="D51" s="92" t="s">
         <v>312</v>
       </c>
-      <c r="D51" s="93" t="s">
+    </row>
+    <row r="52">
+      <c r="C52" s="37" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="C52" s="88" t="s">
+      <c r="D52" s="92" t="s">
         <v>314</v>
       </c>
-      <c r="D52" s="93" t="s">
+    </row>
+    <row r="53">
+      <c r="C53" s="37" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="88" t="s">
+      <c r="D53" s="92" t="s">
         <v>316</v>
       </c>
-      <c r="D53" s="93" t="s">
+    </row>
+    <row r="54">
+      <c r="C54" s="37" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="88" t="s">
+      <c r="D54" s="92" t="s">
         <v>318</v>
       </c>
-      <c r="D54" s="93" t="s">
+    </row>
+    <row r="55">
+      <c r="C55" s="93">
+        <v>4</v>
+      </c>
+      <c r="D55" s="93" t="s">
         <v>319</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" s="94">
-        <v>4</v>
-      </c>
-      <c r="D55" s="94" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="56">
       <c r="C56" s="86" t="s">
+        <v>320</v>
+      </c>
+      <c r="D56" s="76" t="s">
         <v>321</v>
-      </c>
-      <c r="D56" s="76" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="57">
       <c r="C57" s="86" t="s">
+        <v>322</v>
+      </c>
+      <c r="D57" s="92" t="s">
         <v>323</v>
-      </c>
-      <c r="D57" s="93" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="58">
       <c r="C58" s="86" t="s">
+        <v>324</v>
+      </c>
+      <c r="D58" s="92" t="s">
         <v>325</v>
-      </c>
-      <c r="D58" s="93" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="59">
       <c r="C59" s="86" t="s">
+        <v>326</v>
+      </c>
+      <c r="D59" s="92" t="s">
         <v>327</v>
-      </c>
-      <c r="D59" s="93" t="s">
-        <v>328</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="94">
+      <c r="C60" s="93">
         <v>5</v>
       </c>
-      <c r="D60" s="94" t="s">
-        <v>329</v>
+      <c r="D60" s="93" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="61">
       <c r="C61" s="86" t="s">
+        <v>329</v>
+      </c>
+      <c r="D61" s="76" t="s">
         <v>330</v>
-      </c>
-      <c r="D61" s="76" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="62">
       <c r="C62" s="86" t="s">
+        <v>331</v>
+      </c>
+      <c r="D62" s="92" t="s">
         <v>332</v>
       </c>
-      <c r="D62" s="93" t="s">
+      <c r="F62" t="s">
         <v>333</v>
-      </c>
-      <c r="F62" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="63">
       <c r="C63" s="86" t="s">
+        <v>334</v>
+      </c>
+      <c r="D63" s="92" t="s">
         <v>335</v>
-      </c>
-      <c r="D63" s="93" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="64">
       <c r="C64" s="86" t="s">
+        <v>336</v>
+      </c>
+      <c r="D64" s="92" t="s">
         <v>337</v>
       </c>
-      <c r="D64" s="93" t="s">
+    </row>
+    <row r="65">
+      <c r="C65" s="93">
+        <v>6</v>
+      </c>
+      <c r="D65" s="93" t="s">
         <v>338</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="C65" s="94">
-        <v>6</v>
-      </c>
-      <c r="D65" s="94" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="66">
       <c r="C66" s="86" t="s">
+        <v>339</v>
+      </c>
+      <c r="D66" s="76" t="s">
         <v>340</v>
       </c>
-      <c r="D66" s="76" t="s">
+    </row>
+    <row r="67">
+      <c r="C67" s="94" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="67">
-      <c r="C67" s="95" t="s">
+      <c r="D67" s="95" t="s">
         <v>342</v>
-      </c>
-      <c r="D67" s="96" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="68">
       <c r="C68" s="86" t="s">
+        <v>343</v>
+      </c>
+      <c r="D68" s="92" t="s">
         <v>344</v>
       </c>
-      <c r="D68" s="93" t="s">
+    </row>
+    <row r="69">
+      <c r="C69" s="94" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="69">
-      <c r="C69" s="95" t="s">
+      <c r="D69" s="92" t="s">
         <v>346</v>
-      </c>
-      <c r="D69" s="93" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="70">
       <c r="C70" s="86" t="s">
+        <v>347</v>
+      </c>
+      <c r="D70" s="92" t="s">
         <v>348</v>
       </c>
-      <c r="D70" s="93" t="s">
+    </row>
+    <row r="71">
+      <c r="C71" s="93">
+        <v>7</v>
+      </c>
+      <c r="D71" s="5" t="s">
         <v>349</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="C71" s="94">
-        <v>7</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="72">
       <c r="C72" s="86" t="s">
+        <v>350</v>
+      </c>
+      <c r="D72" s="76" t="s">
         <v>351</v>
       </c>
-      <c r="D72" s="76" t="s">
+    </row>
+    <row r="73">
+      <c r="C73" s="93">
+        <v>8</v>
+      </c>
+      <c r="D73" s="5" t="s">
         <v>352</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="C73" s="94">
-        <v>8</v>
-      </c>
-      <c r="D73" s="5" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="74">
       <c r="C74" s="86" t="s">
+        <v>353</v>
+      </c>
+      <c r="D74" s="76" t="s">
         <v>354</v>
       </c>
-      <c r="D74" s="76" t="s">
-        <v>355</v>
-      </c>
     </row>
     <row r="75">
-      <c r="C75" s="94">
+      <c r="C75" s="93">
         <v>9</v>
       </c>
       <c r="D75" s="5" t="s">
@@ -4961,75 +4952,75 @@
     </row>
     <row r="76">
       <c r="C76" s="86" t="s">
+        <v>355</v>
+      </c>
+      <c r="D76" s="76" t="s">
         <v>356</v>
-      </c>
-      <c r="D76" s="76" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="77">
       <c r="C77" s="86" t="s">
+        <v>357</v>
+      </c>
+      <c r="D77" s="92" t="s">
         <v>358</v>
-      </c>
-      <c r="D77" s="93" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="78">
       <c r="C78" s="86" t="s">
+        <v>359</v>
+      </c>
+      <c r="D78" s="92" t="s">
         <v>360</v>
       </c>
-      <c r="D78" s="93" t="s">
+    </row>
+    <row r="79">
+      <c r="C79" s="93">
+        <v>10</v>
+      </c>
+      <c r="D79" s="5" t="s">
         <v>361</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="C79" s="94">
-        <v>10</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="80">
       <c r="C80" s="86" t="s">
+        <v>362</v>
+      </c>
+      <c r="D80" s="76" t="s">
         <v>363</v>
-      </c>
-      <c r="D80" s="76" t="s">
-        <v>364</v>
       </c>
       <c r="E80" s="80"/>
     </row>
     <row r="81">
       <c r="C81" s="86" t="s">
+        <v>364</v>
+      </c>
+      <c r="D81" s="92" t="s">
         <v>365</v>
       </c>
-      <c r="D81" s="93" t="s">
+    </row>
+    <row r="82">
+      <c r="C82" s="93">
+        <v>11</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>366</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="C82" s="94">
-        <v>11</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="83">
       <c r="C83" s="86" t="s">
+        <v>367</v>
+      </c>
+      <c r="D83" s="76" t="s">
         <v>368</v>
-      </c>
-      <c r="D83" s="76" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="84">
       <c r="C84" s="86" t="s">
+        <v>369</v>
+      </c>
+      <c r="D84" s="76" t="s">
         <v>370</v>
-      </c>
-      <c r="D84" s="76" t="s">
-        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plus bug change cd quand player true; Petits details de visu/fonctionnement
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
   <si>
     <t xml:space="preserve">Jukebox : se poser avec feuille et réfléchir sur le lecteur, prévoir taff dans les prochains jours, dessin du rendu final, s'aider de ce qui existe</t>
   </si>
@@ -241,15 +241,12 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">-Trouver hauteur de déplacement de l'elecAimant, + des fois il bug au déplacement, et ne bouge pas/pas assez...
-   - Menu calibrage !
-comment ça marche ? Dans le sens si on lui va a X degrés, ccela correspond tjrs à la meme position
-- Calibrage origine ? Calibrage cd, Calibrage Lecteur
-Sauvegarder kes données avex X e Y
-les récupérers dans le fichiers quand besoin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A TESTER + Vérifier le nb de pas : quand on arrive au bout et recule on fait fait pas -5, a voir si ça gène</t>
+    <t xml:space="preserve">Déplacement Z
+- Calibration OK
+- Bugs : pb d'alimentation ? PWM ?
+- Tester le servo en dehors pour voir s'il a pas un pb
+Aimant
+- Alim assez puissante depuis la Raspberry ?</t>
   </si>
   <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
@@ -1713,7 +1710,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -1781,6 +1778,9 @@
     </xf>
     <xf fontId="0" fillId="12" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3103,14 +3103,12 @@
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" ht="114">
+    <row r="22" ht="99.75">
       <c r="A22" s="1"/>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="37" t="s">
-        <v>69</v>
-      </c>
+      <c r="C22" s="38"/>
       <c r="D22" s="33">
         <v>0.90000000000000002</v>
       </c>
@@ -3118,24 +3116,24 @@
       <c r="G22" s="15"/>
       <c r="H22" s="1"/>
       <c r="I22" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M22" s="34" t="s">
         <v>63</v>
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="P22" s="22" t="s">
         <v>72</v>
-      </c>
-      <c r="P22" s="22" t="s">
-        <v>73</v>
       </c>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
@@ -3143,7 +3141,7 @@
       <c r="T22" s="22"/>
       <c r="U22" s="22"/>
       <c r="X22" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
@@ -3151,17 +3149,17 @@
     <row r="23" ht="42.75">
       <c r="A23" s="1"/>
       <c r="B23" s="26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D23" s="28">
         <v>1</v>
       </c>
       <c r="H23" s="1"/>
-      <c r="I23" s="38"/>
-      <c r="J23" s="38"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M23" s="34" t="s">
         <v>63</v>
@@ -3170,14 +3168,14 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
       <c r="Q23" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
       <c r="X23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
@@ -3185,24 +3183,24 @@
     <row r="24" ht="16.5">
       <c r="A24" s="1"/>
       <c r="B24" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D24" s="33"/>
+      <c r="F24" s="40" t="s">
         <v>79</v>
-      </c>
-      <c r="D24" s="33"/>
-      <c r="F24" s="39" t="s">
-        <v>80</v>
       </c>
       <c r="G24" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="40"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="42"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="43"/>
       <c r="K24" s="1"/>
       <c r="L24" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="M24" s="19" t="s">
         <v>81</v>
-      </c>
-      <c r="M24" s="19" t="s">
-        <v>82</v>
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="22"/>
@@ -3237,11 +3235,11 @@
     </row>
     <row r="26" ht="16.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="45">
+      <c r="B26" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="45"/>
+      <c r="D26" s="46">
         <f>SUM(D27:D32)/5</f>
         <v>0</v>
       </c>
@@ -3255,10 +3253,10 @@
       <c r="M26" s="19"/>
       <c r="N26" s="1"/>
       <c r="O26" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="P26" s="22" t="s">
         <v>84</v>
-      </c>
-      <c r="P26" s="22" t="s">
-        <v>85</v>
       </c>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
@@ -3271,10 +3269,10 @@
     <row r="27" ht="16.5">
       <c r="A27" s="1"/>
       <c r="B27" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" t="s">
         <v>86</v>
-      </c>
-      <c r="C27" t="s">
-        <v>87</v>
       </c>
       <c r="D27" s="33">
         <v>0</v>
@@ -3288,7 +3286,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
       <c r="X27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
@@ -3296,7 +3294,7 @@
     <row r="28" ht="16.5">
       <c r="A28" s="1"/>
       <c r="C28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D28" s="33">
         <v>0</v>
@@ -3312,7 +3310,7 @@
       <c r="T28" s="22"/>
       <c r="U28" s="22"/>
       <c r="X28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
@@ -3320,7 +3318,7 @@
     <row r="29" ht="16.5">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D29" s="33">
         <v>0</v>
@@ -3340,10 +3338,10 @@
     <row r="30" ht="16.5">
       <c r="A30" s="1"/>
       <c r="B30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" t="s">
         <v>92</v>
-      </c>
-      <c r="C30" t="s">
-        <v>93</v>
       </c>
       <c r="D30" s="33">
         <v>0</v>
@@ -3364,10 +3362,10 @@
     <row r="31" ht="16.5">
       <c r="A31" s="1"/>
       <c r="B31" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>95</v>
       </c>
       <c r="D31" s="33">
         <v>0</v>
@@ -3386,13 +3384,13 @@
     <row r="32" ht="28.5">
       <c r="A32" s="1"/>
       <c r="B32" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D32" s="33">
         <v>0</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M32" s="19"/>
       <c r="N32" s="1"/>
@@ -3402,7 +3400,7 @@
       <c r="B33" s="4"/>
       <c r="D33" s="33"/>
       <c r="L33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
@@ -3443,11 +3441,11 @@
     </row>
     <row r="36" ht="16.5">
       <c r="A36" s="1"/>
-      <c r="B36" s="46" t="s">
-        <v>99</v>
-      </c>
-      <c r="C36" s="44"/>
-      <c r="D36" s="45">
+      <c r="B36" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" s="45"/>
+      <c r="D36" s="46">
         <f>SUM(D37:D40)/4</f>
         <v>0.75</v>
       </c>
@@ -3465,10 +3463,10 @@
     <row r="37" ht="16.5">
       <c r="A37" s="1"/>
       <c r="B37" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>101</v>
       </c>
       <c r="D37" s="28">
         <v>1</v>
@@ -3487,10 +3485,10 @@
     <row r="38" ht="16.5">
       <c r="A38" s="1"/>
       <c r="B38" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="D38" s="28">
         <v>1</v>
@@ -3509,10 +3507,10 @@
     <row r="39" ht="28.5">
       <c r="A39" s="1"/>
       <c r="B39" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="D39" s="28">
         <v>1</v>
@@ -3521,10 +3519,10 @@
     <row r="40" ht="28.5">
       <c r="A40" s="1"/>
       <c r="B40" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="26" t="s">
         <v>106</v>
-      </c>
-      <c r="C40" s="26" t="s">
-        <v>107</v>
       </c>
       <c r="D40" s="33">
         <v>0</v>
@@ -3536,7 +3534,7 @@
     <row r="42" ht="16.5">
       <c r="A42" s="1"/>
       <c r="B42" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -3544,7 +3542,7 @@
     <row r="43" ht="16.5">
       <c r="A43" s="1"/>
       <c r="B43" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -3555,7 +3553,7 @@
     <row r="45" ht="16.5">
       <c r="A45" s="1"/>
       <c r="B45" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" ht="14.25">
@@ -3567,7 +3565,7 @@
     <row r="48" ht="14.25">
       <c r="A48" s="1"/>
       <c r="B48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" ht="14.25">
@@ -3576,13 +3574,13 @@
     <row r="50" ht="14.25">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51" ht="14.25">
       <c r="A51" s="1"/>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" ht="16.5">
@@ -3594,7 +3592,7 @@
     <row r="54" ht="16.5">
       <c r="A54" s="1"/>
       <c r="B54" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -3636,7 +3634,7 @@
     <row r="57" ht="16.5">
       <c r="A57" s="1"/>
       <c r="B57" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
@@ -3664,52 +3662,52 @@
     </row>
     <row r="69" ht="14.25">
       <c r="B69" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="70" ht="14.25">
       <c r="B70" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" ht="14.25">
       <c r="B71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="72" ht="14.25">
       <c r="B72" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73" ht="14.25">
       <c r="B73" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" ht="14.25">
       <c r="B74" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="B75" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="76" ht="14.25">
       <c r="B76" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="77" ht="14.25">
       <c r="B77" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="78" ht="14.25">
       <c r="B78" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C78" t="s">
         <v>67</v>
@@ -3739,16 +3737,16 @@
   </cols>
   <sheetData>
     <row r="2" ht="14.25">
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" t="s">
         <v>126</v>
-      </c>
-      <c r="C2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="3" ht="14.25">
       <c r="B3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3771,280 +3769,280 @@
   <sheetData>
     <row r="1" ht="15"/>
     <row r="2" ht="15">
-      <c r="F2" s="48" t="s">
+      <c r="F2" s="49" t="s">
+        <v>128</v>
+      </c>
+      <c r="G2" s="50" t="s">
         <v>129</v>
       </c>
-      <c r="G2" s="49" t="s">
+    </row>
+    <row r="3">
+      <c r="F3" s="51" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="F3" s="50" t="s">
+      <c r="G3" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="G3" s="51" t="s">
+    </row>
+    <row r="4">
+      <c r="F4" s="53" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="F4" s="52" t="s">
+      <c r="G4" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="G4" s="53" t="s">
+    </row>
+    <row r="5" ht="15">
+      <c r="F5" s="55" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="5" ht="15">
-      <c r="F5" s="54" t="s">
+      <c r="G5" s="56" t="s">
         <v>135</v>
       </c>
-      <c r="G5" s="55" t="s">
+    </row>
+    <row r="6" ht="15">
+      <c r="F6" s="57"/>
+      <c r="G6" s="58" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="6" ht="15">
-      <c r="F6" s="56"/>
-      <c r="G6" s="57" t="s">
+    <row r="7" ht="15">
+      <c r="F7" s="57"/>
+      <c r="G7" s="58" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="7" ht="15">
-      <c r="F7" s="56"/>
-      <c r="G7" s="57" t="s">
+    <row r="8" ht="15">
+      <c r="F8" s="57"/>
+      <c r="G8" s="58" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="8" ht="15">
-      <c r="F8" s="56"/>
-      <c r="G8" s="57" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="B9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F9" s="57"/>
+      <c r="G9" s="58" t="s">
         <v>140</v>
-      </c>
-      <c r="F9" s="56"/>
-      <c r="G9" s="57" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="B10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="F10" s="57"/>
+      <c r="G10" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="F10" s="56"/>
-      <c r="G10" s="57" t="s">
+    </row>
+    <row r="11" ht="15">
+      <c r="C11" s="60" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="11" ht="15">
-      <c r="C11" s="59" t="s">
+      <c r="F11" s="57"/>
+      <c r="G11" s="58" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="56"/>
-      <c r="G11" s="57" t="s">
+    </row>
+    <row r="12" ht="15">
+      <c r="C12" s="59" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="12" ht="15">
-      <c r="C12" s="58" t="s">
+      <c r="F12" s="51"/>
+      <c r="G12" s="61" t="s">
         <v>147</v>
       </c>
-      <c r="F12" s="50"/>
-      <c r="G12" s="60" t="s">
+    </row>
+    <row r="13" ht="15">
+      <c r="C13" s="60" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="13" ht="15">
-      <c r="C13" s="59" t="s">
+      <c r="F13" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="F13" s="52" t="s">
+      <c r="G13" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="G13" s="61" t="s">
+    </row>
+    <row r="14" ht="15">
+      <c r="C14" s="59" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="14" ht="15">
-      <c r="C14" s="58" t="s">
+      <c r="F14" s="63" t="s">
         <v>152</v>
       </c>
-      <c r="F14" s="62" t="s">
+      <c r="G14" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="G14" s="63" t="s">
+    </row>
+    <row r="15">
+      <c r="C15" s="60" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="C15" s="59" t="s">
+      <c r="F15" s="65" t="s">
         <v>155</v>
       </c>
-      <c r="F15" s="64" t="s">
+      <c r="G15" s="66" t="s">
         <v>156</v>
       </c>
-      <c r="G15" s="65" t="s">
+    </row>
+    <row r="16">
+      <c r="C16" s="60" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="59" t="s">
+      <c r="F16" s="67" t="s">
         <v>158</v>
       </c>
-      <c r="F16" s="66" t="s">
+      <c r="G16" s="68" t="s">
         <v>159</v>
       </c>
-      <c r="G16" s="67" t="s">
+    </row>
+    <row r="17">
+      <c r="C17" s="59" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="C17" s="58" t="s">
+      <c r="F17" s="67"/>
+      <c r="G17" s="68" t="s">
         <v>161</v>
       </c>
-      <c r="F17" s="66"/>
-      <c r="G17" s="67" t="s">
+    </row>
+    <row r="18">
+      <c r="C18" s="60" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="C18" s="59" t="s">
+      <c r="F18" s="67"/>
+      <c r="G18" s="68" t="s">
         <v>163</v>
       </c>
-      <c r="F18" s="66"/>
-      <c r="G18" s="67" t="s">
+    </row>
+    <row r="19">
+      <c r="C19" s="60" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="C19" s="59" t="s">
+      <c r="F19" s="67"/>
+      <c r="G19" s="68" t="s">
         <v>165</v>
       </c>
-      <c r="F19" s="66"/>
-      <c r="G19" s="67" t="s">
+    </row>
+    <row r="20">
+      <c r="C20" s="60" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="59" t="s">
+      <c r="F20" s="67"/>
+      <c r="G20" s="68" t="s">
         <v>167</v>
       </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="67" t="s">
+    </row>
+    <row r="21">
+      <c r="C21" s="60" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="59" t="s">
+      <c r="F21" s="67"/>
+      <c r="G21" s="68" t="s">
         <v>169</v>
       </c>
-      <c r="F21" s="66"/>
-      <c r="G21" s="67" t="s">
+    </row>
+    <row r="22">
+      <c r="C22" s="59" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="58" t="s">
+      <c r="F22" s="67"/>
+      <c r="G22" s="68" t="s">
         <v>171</v>
       </c>
-      <c r="F22" s="66"/>
-      <c r="G22" s="67" t="s">
+    </row>
+    <row r="23">
+      <c r="C23" s="60" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="C23" s="59" t="s">
+      <c r="F23" s="67"/>
+      <c r="G23" s="68" t="s">
         <v>173</v>
       </c>
-      <c r="F23" s="66"/>
-      <c r="G23" s="67" t="s">
+    </row>
+    <row r="24">
+      <c r="C24" s="59" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="58" t="s">
+      <c r="F24" s="67"/>
+      <c r="G24" s="68" t="s">
         <v>175</v>
       </c>
-      <c r="F24" s="66"/>
-      <c r="G24" s="67" t="s">
+    </row>
+    <row r="25">
+      <c r="C25" s="60" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="59" t="s">
+      <c r="F25" s="67"/>
+      <c r="G25" s="68" t="s">
         <v>177</v>
       </c>
-      <c r="F25" s="66"/>
-      <c r="G25" s="67" t="s">
+    </row>
+    <row r="26">
+      <c r="F26" s="67"/>
+      <c r="G26" s="68" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="26">
-      <c r="F26" s="66"/>
-      <c r="G26" s="67" t="s">
+    <row r="27">
+      <c r="F27" s="67"/>
+      <c r="G27" s="68"/>
+    </row>
+    <row r="28">
+      <c r="F28" s="67"/>
+      <c r="G28" s="68" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="27">
-      <c r="F27" s="66"/>
-      <c r="G27" s="67"/>
-    </row>
-    <row r="28">
-      <c r="F28" s="66"/>
-      <c r="G28" s="67" t="s">
+    <row r="29">
+      <c r="F29" s="67"/>
+      <c r="G29" s="68" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="29">
-      <c r="F29" s="66"/>
-      <c r="G29" s="67" t="s">
+    <row r="30">
+      <c r="C30" s="69"/>
+      <c r="F30" s="67"/>
+      <c r="G30" s="68" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="30">
-      <c r="C30" s="68"/>
-      <c r="F30" s="66"/>
-      <c r="G30" s="67" t="s">
+    <row r="31">
+      <c r="F31" s="67"/>
+      <c r="G31" s="70" t="s">
         <v>182</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="F31" s="66"/>
-      <c r="G31" s="69" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="25"/>
-      <c r="F32" s="62" t="s">
+      <c r="F32" s="63" t="s">
+        <v>183</v>
+      </c>
+      <c r="G32" s="71" t="s">
         <v>184</v>
       </c>
-      <c r="G32" s="70" t="s">
-        <v>185</v>
-      </c>
     </row>
     <row r="33">
-      <c r="C33" s="59"/>
+      <c r="C33" s="60"/>
     </row>
     <row r="34">
-      <c r="C34" s="59"/>
+      <c r="C34" s="60"/>
     </row>
     <row r="36">
-      <c r="C36" s="68"/>
+      <c r="C36" s="69"/>
     </row>
     <row r="38">
       <c r="C38" s="25"/>
     </row>
     <row r="39">
-      <c r="C39" s="59"/>
+      <c r="C39" s="60"/>
     </row>
     <row r="40">
-      <c r="C40" s="59"/>
+      <c r="C40" s="60"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -4072,367 +4070,367 @@
   <sheetData>
     <row r="5">
       <c r="A5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" t="s">
         <v>186</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="D5" s="71" t="s">
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" t="s">
         <v>188</v>
       </c>
-      <c r="E5" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" t="s">
-        <v>100</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>189</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>190</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>191</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>192</v>
-      </c>
-      <c r="K5" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" t="s">
         <v>194</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" s="73" t="s">
         <v>195</v>
       </c>
-      <c r="D6" s="72" t="s">
+      <c r="E6" t="s">
         <v>196</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>197</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>198</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" s="74" t="s">
         <v>199</v>
       </c>
-      <c r="H6" s="73" t="s">
+      <c r="I6" t="s">
         <v>200</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>201</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>202</v>
-      </c>
-      <c r="K6" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" s="75" t="s">
         <v>204</v>
       </c>
-      <c r="B7" t="s">
-        <v>195</v>
-      </c>
-      <c r="D7" s="74" t="s">
+      <c r="F7" t="s">
         <v>205</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>206</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="74" t="s">
         <v>207</v>
       </c>
-      <c r="H7" s="73" t="s">
+      <c r="K7" t="s">
         <v>208</v>
       </c>
-      <c r="K7" t="s">
+    </row>
+    <row r="8">
+      <c r="D8" s="73" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="72" t="s">
+      <c r="G8" s="76" t="s">
         <v>210</v>
       </c>
-      <c r="G8" s="75" t="s">
+      <c r="H8" s="74" t="s">
         <v>211</v>
-      </c>
-      <c r="H8" s="73" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B9" t="s">
         <v>213</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="D9" s="74" t="s">
+      <c r="H9" s="74" t="s">
         <v>215</v>
-      </c>
-      <c r="H9" s="73" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B10" t="s">
         <v>217</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" s="73"/>
+      <c r="G10" t="s">
         <v>218</v>
       </c>
-      <c r="D10" s="72"/>
-      <c r="G10" t="s">
+      <c r="H10" s="74" t="s">
         <v>219</v>
-      </c>
-      <c r="H10" s="73" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>220</v>
+      </c>
+      <c r="B11" t="s">
         <v>221</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" s="75" t="s">
         <v>222</v>
       </c>
-      <c r="D11" s="74" t="s">
+      <c r="G11" s="76" t="s">
         <v>223</v>
       </c>
-      <c r="G11" s="75" t="s">
+      <c r="H11" s="74" t="s">
         <v>224</v>
-      </c>
-      <c r="H11" s="73" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>225</v>
+      </c>
+      <c r="B12" t="s">
         <v>226</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" s="73" t="s">
         <v>227</v>
       </c>
-      <c r="D12" s="72" t="s">
+      <c r="G12" s="76" t="s">
         <v>228</v>
       </c>
-      <c r="G12" s="75" t="s">
+      <c r="H12" s="74" t="s">
         <v>229</v>
-      </c>
-      <c r="H12" s="73" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>230</v>
+      </c>
+      <c r="B13" t="s">
         <v>231</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" s="75" t="s">
         <v>232</v>
       </c>
-      <c r="D13" s="74" t="s">
+      <c r="G13" s="76" t="s">
         <v>233</v>
       </c>
-      <c r="G13" s="75" t="s">
+    </row>
+    <row r="14">
+      <c r="D14" s="73" t="s">
         <v>234</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="72" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>235</v>
+      </c>
+      <c r="B15" t="s">
         <v>236</v>
       </c>
-      <c r="B15" t="s">
-        <v>237</v>
-      </c>
-      <c r="D15" s="74"/>
+      <c r="D15" s="75"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>237</v>
+      </c>
+      <c r="B16" t="s">
         <v>238</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" s="73"/>
+      <c r="G16" t="s">
         <v>239</v>
       </c>
-      <c r="D16" s="72"/>
-      <c r="G16" t="s">
+    </row>
+    <row r="17">
+      <c r="D17" s="75"/>
+      <c r="G17" s="76" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="74"/>
-      <c r="G17" s="75" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>241</v>
+      </c>
+      <c r="D18" s="73"/>
+      <c r="G18" s="77" t="s">
         <v>242</v>
       </c>
-      <c r="D18" s="72"/>
-      <c r="G18" s="76" t="s">
+    </row>
+    <row r="19">
+      <c r="D19" s="75" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="D19" s="74" t="s">
+      <c r="E19" t="s">
         <v>244</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" s="77" t="s">
         <v>245</v>
       </c>
-      <c r="G19" s="76" t="s">
+      <c r="H19" t="s">
         <v>246</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>247</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="73"/>
+      <c r="G20" s="77" t="s">
         <v>248</v>
       </c>
-      <c r="J19" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" s="72"/>
-      <c r="G20" s="76" t="s">
+    </row>
+    <row r="22">
+      <c r="D22" s="73"/>
+      <c r="G22" s="77" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="G23" s="76"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="73"/>
+      <c r="G24" s="76" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="22">
-      <c r="D22" s="72"/>
-      <c r="G22" s="76" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="G23" s="75"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="72"/>
-      <c r="G24" s="75" t="s">
+    <row r="25">
+      <c r="G25" s="77" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="25">
-      <c r="G25" s="76" t="s">
+    <row r="26">
+      <c r="D26" s="73"/>
+      <c r="G26" s="77" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="26">
-      <c r="D26" s="72"/>
-      <c r="G26" s="76" t="s">
+    <row r="27">
+      <c r="G27" s="77" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="27">
-      <c r="G27" s="76" t="s">
+    <row r="28">
+      <c r="D28" s="73"/>
+      <c r="G28" s="77" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="78" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="72"/>
-      <c r="G28" s="76" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" s="77" t="s">
+      <c r="E35" t="s">
         <v>254</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" s="79" t="s">
         <v>255</v>
       </c>
-      <c r="F35" s="78" t="s">
+    </row>
+    <row r="36">
+      <c r="D36" s="80" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="36">
-      <c r="D36" s="79" t="s">
+      <c r="E36" t="s">
         <v>257</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" s="80" t="s">
         <v>258</v>
       </c>
-      <c r="F36" s="79" t="s">
+    </row>
+    <row r="37">
+      <c r="D37" s="79" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="37">
-      <c r="D37" s="78" t="s">
+      <c r="E37" t="s">
         <v>260</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" s="79" t="s">
         <v>261</v>
       </c>
-      <c r="F37" s="78" t="s">
+    </row>
+    <row r="38">
+      <c r="D38" s="80" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="D38" s="79" t="s">
+      <c r="E38" t="s">
         <v>263</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" s="80" t="s">
         <v>264</v>
       </c>
-      <c r="F38" s="79" t="s">
+    </row>
+    <row r="39">
+      <c r="D39" s="79" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="D39" s="78" t="s">
+      <c r="E39" t="s">
         <v>266</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" s="79" t="s">
         <v>267</v>
-      </c>
-      <c r="F39" s="78" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="40">
       <c r="E40" t="s">
-        <v>258</v>
-      </c>
-      <c r="F40" s="79" t="s">
-        <v>269</v>
+        <v>257</v>
+      </c>
+      <c r="F40" s="80" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="41">
       <c r="E41" t="s">
-        <v>261</v>
-      </c>
-      <c r="F41" s="78" t="s">
-        <v>270</v>
+        <v>260</v>
+      </c>
+      <c r="F41" s="79" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4463,564 +4461,564 @@
   </cols>
   <sheetData>
     <row r="4">
-      <c r="D4" s="80" t="s">
+      <c r="D4" s="81" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" t="s">
         <v>273</v>
-      </c>
-      <c r="E4" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E5" s="81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="77" t="s">
         <v>275</v>
       </c>
-      <c r="E5" s="80">
+      <c r="E6" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="D6" s="76" t="s">
+    <row r="7">
+      <c r="D7" s="82" t="s">
         <v>276</v>
       </c>
-      <c r="E6" s="80">
+      <c r="E7" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="D7" s="81" t="s">
+    <row r="8">
+      <c r="D8" s="77" t="s">
         <v>277</v>
       </c>
-      <c r="E7" s="80">
+      <c r="E8" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="D8" s="76" t="s">
+    <row r="9">
+      <c r="D9" s="77"/>
+      <c r="E9" s="81"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="74" t="s">
         <v>278</v>
       </c>
-      <c r="E8" s="80">
+      <c r="E10" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="D9" s="76"/>
-      <c r="E9" s="80"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="73" t="s">
+    <row r="11">
+      <c r="D11" s="77" t="s">
         <v>279</v>
       </c>
-      <c r="E10" s="80">
+      <c r="E11" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="D11" s="76" t="s">
+    <row r="12">
+      <c r="D12" s="77" t="s">
         <v>280</v>
       </c>
-      <c r="E11" s="80">
+      <c r="E12" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="12">
-      <c r="D12" s="76" t="s">
+    <row r="13">
+      <c r="D13" s="77" t="s">
         <v>281</v>
       </c>
-      <c r="E12" s="80">
+      <c r="E13" s="81">
         <v>1</v>
       </c>
     </row>
-    <row r="13">
-      <c r="D13" s="76" t="s">
+    <row r="14">
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="74" t="s">
         <v>282</v>
       </c>
-      <c r="E13" s="80">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="73" t="s">
+      <c r="E15" s="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="83" t="s">
         <v>283</v>
       </c>
-      <c r="E15" s="80">
+      <c r="E16" s="81">
         <v>2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="D16" s="82" t="s">
+    <row r="17">
+      <c r="D17" s="84" t="s">
         <v>284</v>
       </c>
-      <c r="E16" s="80">
+      <c r="E17" s="81">
         <v>2</v>
       </c>
     </row>
-    <row r="17">
-      <c r="D17" s="83" t="s">
+    <row r="18">
+      <c r="D18" s="84" t="s">
         <v>285</v>
       </c>
-      <c r="E17" s="80">
+      <c r="E18" s="81">
         <v>2</v>
       </c>
     </row>
-    <row r="18">
-      <c r="D18" s="83" t="s">
+    <row r="19">
+      <c r="D19" s="77"/>
+      <c r="E19" s="77"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="74" t="s">
         <v>286</v>
       </c>
-      <c r="E18" s="80">
+      <c r="E20" s="81">
         <v>2</v>
       </c>
     </row>
-    <row r="19">
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-    </row>
-    <row r="20">
-      <c r="D20" s="73" t="s">
+    <row r="21">
+      <c r="D21" s="74" t="s">
         <v>287</v>
       </c>
-      <c r="E20" s="80">
+      <c r="E21" s="81">
         <v>2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="D21" s="73" t="s">
+    <row r="22">
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="85"/>
+      <c r="E23" s="77"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="77"/>
+      <c r="E24" s="77"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="77"/>
+      <c r="E25" s="77"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="77"/>
+      <c r="E26" s="77"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="77"/>
+      <c r="E27" s="77"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="77"/>
+      <c r="E28" s="77"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="77"/>
+      <c r="E29" s="77"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="86"/>
+      <c r="C39" s="87" t="s">
         <v>288</v>
       </c>
-      <c r="E21" s="80">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="84"/>
-      <c r="E23" s="76"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-    </row>
-    <row r="25">
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="76"/>
-      <c r="E26" s="76"/>
-    </row>
-    <row r="27">
-      <c r="D27" s="76"/>
-      <c r="E27" s="76"/>
-    </row>
-    <row r="28">
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-    </row>
-    <row r="29">
-      <c r="D29" s="76"/>
-      <c r="E29" s="76"/>
-    </row>
-    <row r="30">
-      <c r="D30" s="76"/>
-      <c r="E30" s="76"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="85"/>
-      <c r="C39" s="86" t="s">
+      <c r="D39" s="87" t="s">
         <v>289</v>
       </c>
-      <c r="D39" s="86" t="s">
-        <v>290</v>
-      </c>
       <c r="E39" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F39" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="87">
+      <c r="C40" s="88">
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="E40" s="81"/>
+    </row>
+    <row r="41">
+      <c r="C41" s="81" t="s">
         <v>291</v>
       </c>
-      <c r="E40" s="80"/>
-    </row>
-    <row r="41">
-      <c r="C41" s="80" t="s">
+      <c r="D41" s="77" t="s">
         <v>292</v>
       </c>
-      <c r="D41" s="76" t="s">
+      <c r="E41" s="81"/>
+    </row>
+    <row r="42" ht="14.25" customHeight="1">
+      <c r="C42" s="81" t="s">
         <v>293</v>
       </c>
-      <c r="E41" s="80"/>
-    </row>
-    <row r="42" ht="14.25" customHeight="1">
-      <c r="C42" s="80" t="s">
+      <c r="D42" s="77" t="s">
         <v>294</v>
       </c>
-      <c r="D42" s="76" t="s">
+    </row>
+    <row r="43">
+      <c r="C43" s="81" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="C43" s="80" t="s">
+      <c r="D43" s="77" t="s">
         <v>296</v>
       </c>
-      <c r="D43" s="76" t="s">
+    </row>
+    <row r="44">
+      <c r="C44" s="38" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="44">
-      <c r="C44" s="37" t="s">
+      <c r="D44" s="82" t="s">
         <v>298</v>
       </c>
-      <c r="D44" s="81" t="s">
+      <c r="E44" s="89"/>
+      <c r="F44" s="89"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="87" t="s">
         <v>299</v>
       </c>
-      <c r="E44" s="88"/>
-      <c r="F44" s="88"/>
-    </row>
-    <row r="45">
-      <c r="C45" s="86" t="s">
+      <c r="D45" s="77" t="s">
         <v>300</v>
       </c>
-      <c r="D45" s="76" t="s">
+      <c r="E45" s="81"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="87" t="s">
         <v>301</v>
       </c>
-      <c r="E45" s="80"/>
-    </row>
-    <row r="46">
-      <c r="C46" s="86" t="s">
+      <c r="D46" s="77" t="s">
         <v>302</v>
       </c>
-      <c r="D46" s="76" t="s">
+      <c r="E46" s="81"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="90">
+        <v>2</v>
+      </c>
+      <c r="D47" s="91" t="s">
         <v>303</v>
       </c>
-      <c r="E46" s="80"/>
-    </row>
-    <row r="47">
-      <c r="C47" s="89">
-        <v>2</v>
-      </c>
-      <c r="D47" s="90" t="s">
+      <c r="E47" s="81"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="38" t="s">
         <v>304</v>
       </c>
-      <c r="E47" s="80"/>
-    </row>
-    <row r="48">
-      <c r="C48" s="37" t="s">
+      <c r="D48" s="82" t="s">
         <v>305</v>
       </c>
-      <c r="D48" s="81" t="s">
+      <c r="E48" s="81"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="88">
+        <v>3</v>
+      </c>
+      <c r="D49" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="E48" s="80"/>
-    </row>
-    <row r="49">
-      <c r="C49" s="87">
-        <v>3</v>
-      </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="81"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="38" t="s">
         <v>307</v>
       </c>
-      <c r="E49" s="80"/>
-    </row>
-    <row r="50">
-      <c r="C50" s="37" t="s">
+      <c r="D50" s="82" t="s">
         <v>308</v>
       </c>
-      <c r="D50" s="81" t="s">
+      <c r="F50" s="92" t="s">
         <v>309</v>
       </c>
-      <c r="F50" s="91" t="s">
+    </row>
+    <row r="51">
+      <c r="C51" s="38" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="C51" s="37" t="s">
+      <c r="D51" s="93" t="s">
         <v>311</v>
       </c>
-      <c r="D51" s="92" t="s">
+    </row>
+    <row r="52">
+      <c r="C52" s="38" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="C52" s="37" t="s">
+      <c r="D52" s="93" t="s">
         <v>313</v>
       </c>
-      <c r="D52" s="92" t="s">
+    </row>
+    <row r="53">
+      <c r="C53" s="38" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="37" t="s">
+      <c r="D53" s="93" t="s">
         <v>315</v>
       </c>
-      <c r="D53" s="92" t="s">
+    </row>
+    <row r="54">
+      <c r="C54" s="38" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="37" t="s">
+      <c r="D54" s="93" t="s">
         <v>317</v>
       </c>
-      <c r="D54" s="92" t="s">
+    </row>
+    <row r="55">
+      <c r="C55" s="94">
+        <v>4</v>
+      </c>
+      <c r="D55" s="94" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="55">
-      <c r="C55" s="93">
-        <v>4</v>
-      </c>
-      <c r="D55" s="93" t="s">
+    <row r="56">
+      <c r="C56" s="87" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="86" t="s">
+      <c r="D56" s="77" t="s">
         <v>320</v>
       </c>
-      <c r="D56" s="76" t="s">
+    </row>
+    <row r="57">
+      <c r="C57" s="87" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="86" t="s">
+      <c r="D57" s="93" t="s">
         <v>322</v>
       </c>
-      <c r="D57" s="92" t="s">
+    </row>
+    <row r="58">
+      <c r="C58" s="87" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="C58" s="86" t="s">
+      <c r="D58" s="93" t="s">
         <v>324</v>
       </c>
-      <c r="D58" s="92" t="s">
+    </row>
+    <row r="59">
+      <c r="C59" s="87" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="86" t="s">
+      <c r="D59" s="93" t="s">
         <v>326</v>
-      </c>
-      <c r="D59" s="92" t="s">
-        <v>327</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
     </row>
     <row r="60">
-      <c r="C60" s="93">
+      <c r="C60" s="94">
         <v>5</v>
       </c>
-      <c r="D60" s="93" t="s">
+      <c r="D60" s="94" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" s="87" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="61">
-      <c r="C61" s="86" t="s">
+      <c r="D61" s="77" t="s">
         <v>329</v>
       </c>
-      <c r="D61" s="76" t="s">
+    </row>
+    <row r="62">
+      <c r="C62" s="87" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="62">
-      <c r="C62" s="86" t="s">
+      <c r="D62" s="93" t="s">
         <v>331</v>
       </c>
-      <c r="D62" s="92" t="s">
+      <c r="F62" t="s">
         <v>332</v>
       </c>
-      <c r="F62" t="s">
+    </row>
+    <row r="63">
+      <c r="C63" s="87" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="63">
-      <c r="C63" s="86" t="s">
+      <c r="D63" s="93" t="s">
         <v>334</v>
       </c>
-      <c r="D63" s="92" t="s">
+    </row>
+    <row r="64">
+      <c r="C64" s="87" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="64">
-      <c r="C64" s="86" t="s">
+      <c r="D64" s="93" t="s">
         <v>336</v>
       </c>
-      <c r="D64" s="92" t="s">
+    </row>
+    <row r="65">
+      <c r="C65" s="94">
+        <v>6</v>
+      </c>
+      <c r="D65" s="94" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="65">
-      <c r="C65" s="93">
-        <v>6</v>
-      </c>
-      <c r="D65" s="93" t="s">
+    <row r="66">
+      <c r="C66" s="87" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="66">
-      <c r="C66" s="86" t="s">
+      <c r="D66" s="77" t="s">
         <v>339</v>
       </c>
-      <c r="D66" s="76" t="s">
+    </row>
+    <row r="67">
+      <c r="C67" s="95" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="67">
-      <c r="C67" s="94" t="s">
+      <c r="D67" s="96" t="s">
         <v>341</v>
       </c>
-      <c r="D67" s="95" t="s">
+    </row>
+    <row r="68">
+      <c r="C68" s="87" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="68">
-      <c r="C68" s="86" t="s">
+      <c r="D68" s="93" t="s">
         <v>343</v>
       </c>
-      <c r="D68" s="92" t="s">
+    </row>
+    <row r="69">
+      <c r="C69" s="95" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="69">
-      <c r="C69" s="94" t="s">
+      <c r="D69" s="93" t="s">
         <v>345</v>
       </c>
-      <c r="D69" s="92" t="s">
+    </row>
+    <row r="70">
+      <c r="C70" s="87" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="70">
-      <c r="C70" s="86" t="s">
+      <c r="D70" s="93" t="s">
         <v>347</v>
       </c>
-      <c r="D70" s="92" t="s">
+    </row>
+    <row r="71">
+      <c r="C71" s="94">
+        <v>7</v>
+      </c>
+      <c r="D71" s="5" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="71">
-      <c r="C71" s="93">
-        <v>7</v>
-      </c>
-      <c r="D71" s="5" t="s">
+    <row r="72">
+      <c r="C72" s="87" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="72">
-      <c r="C72" s="86" t="s">
+      <c r="D72" s="77" t="s">
         <v>350</v>
       </c>
-      <c r="D72" s="76" t="s">
+    </row>
+    <row r="73">
+      <c r="C73" s="94">
+        <v>8</v>
+      </c>
+      <c r="D73" s="5" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="73">
-      <c r="C73" s="93">
-        <v>8</v>
-      </c>
-      <c r="D73" s="5" t="s">
+    <row r="74">
+      <c r="C74" s="87" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="74">
-      <c r="C74" s="86" t="s">
+      <c r="D74" s="77" t="s">
         <v>353</v>
       </c>
-      <c r="D74" s="76" t="s">
+    </row>
+    <row r="75">
+      <c r="C75" s="94">
+        <v>9</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" s="87" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="75">
-      <c r="C75" s="93">
-        <v>9</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="C76" s="86" t="s">
+      <c r="D76" s="77" t="s">
         <v>355</v>
       </c>
-      <c r="D76" s="76" t="s">
+    </row>
+    <row r="77">
+      <c r="C77" s="87" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="77">
-      <c r="C77" s="86" t="s">
+      <c r="D77" s="93" t="s">
         <v>357</v>
       </c>
-      <c r="D77" s="92" t="s">
+    </row>
+    <row r="78">
+      <c r="C78" s="87" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="78">
-      <c r="C78" s="86" t="s">
+      <c r="D78" s="93" t="s">
         <v>359</v>
       </c>
-      <c r="D78" s="92" t="s">
+    </row>
+    <row r="79">
+      <c r="C79" s="94">
+        <v>10</v>
+      </c>
+      <c r="D79" s="5" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="79">
-      <c r="C79" s="93">
-        <v>10</v>
-      </c>
-      <c r="D79" s="5" t="s">
+    <row r="80">
+      <c r="C80" s="87" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="80">
-      <c r="C80" s="86" t="s">
+      <c r="D80" s="77" t="s">
         <v>362</v>
       </c>
-      <c r="D80" s="76" t="s">
+      <c r="E80" s="81"/>
+    </row>
+    <row r="81">
+      <c r="C81" s="87" t="s">
         <v>363</v>
       </c>
-      <c r="E80" s="80"/>
-    </row>
-    <row r="81">
-      <c r="C81" s="86" t="s">
+      <c r="D81" s="93" t="s">
         <v>364</v>
       </c>
-      <c r="D81" s="92" t="s">
+    </row>
+    <row r="82">
+      <c r="C82" s="94">
+        <v>11</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="82">
-      <c r="C82" s="93">
-        <v>11</v>
-      </c>
-      <c r="D82" s="5" t="s">
+    <row r="83">
+      <c r="C83" s="87" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="83">
-      <c r="C83" s="86" t="s">
+      <c r="D83" s="77" t="s">
         <v>367</v>
       </c>
-      <c r="D83" s="76" t="s">
+    </row>
+    <row r="84">
+      <c r="C84" s="87" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="84">
-      <c r="C84" s="86" t="s">
+      <c r="D84" s="77" t="s">
         <v>369</v>
-      </c>
-      <c r="D84" s="76" t="s">
-        <v>370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajout lo déplaement Z
</commit_message>
<xml_diff>
--- a/Jukebox.xlsx
+++ b/Jukebox.xlsx
@@ -242,14 +242,8 @@
   </si>
   <si>
     <t xml:space="preserve"># Déplacement Z
-- Calibration OK
-- Servo Moteur testé sur Arduino : OK
-- Elec aimant testé sur Arduino : OK
-Le mecanisme fonctionne mais pas tout en même temps
-- Vérifier calibrage ElectAimant : assez bas pour attraper le cd ? Origine ?
-    - Distance au lecteur
-- Realibrer les cds en x et y
-</t>
+GOOD MAIS
+Il faut 3 plaques plutot que des rond en alu pour aimanter les cd sur la face</t>
   </si>
   <si>
     <t xml:space="preserve">IMPRIMER PIECES</t>
@@ -3109,7 +3103,7 @@
       <c r="Z21" s="1"/>
       <c r="AA21" s="1"/>
     </row>
-    <row r="22" ht="128.25">
+    <row r="22" ht="57">
       <c r="A22" s="1"/>
       <c r="B22" s="37" t="s">
         <v>68</v>

</xml_diff>